<commit_message>
Aggiornamento automatico del 07/09/2026 alle 20:55
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3406,8 +3406,12 @@
           <t>Lecce</t>
         </is>
       </c>
-      <c r="G21" s="71" t="n"/>
-      <c r="H21" s="71" t="n"/>
+      <c r="G21" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="I21" s="76">
         <f>IF(OR($G21="",$H21=""),"",IF($G21&gt;$H21,"1",IF($G21=$H21,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 07/09/2026 alle 23:49
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3454,8 +3454,12 @@
           <t>Lazio</t>
         </is>
       </c>
-      <c r="G22" s="71" t="n"/>
-      <c r="H22" s="71" t="n"/>
+      <c r="G22" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I22" s="76">
         <f>IF(OR($G22="",$H22=""),"",IF($G22&gt;$H22,"1",IF($G22=$H22,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/09/2026 alle 21:35
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -6454,21 +6454,61 @@
         <f>IF(Partite!$F23="","",Partite!$F23)</f>
         <v/>
       </c>
-      <c r="E23" s="71" t="n"/>
-      <c r="F23" s="71" t="n"/>
-      <c r="G23" s="71" t="n"/>
-      <c r="H23" s="71" t="n"/>
-      <c r="I23" s="71" t="n"/>
-      <c r="J23" s="71" t="n"/>
-      <c r="K23" s="71" t="n"/>
-      <c r="L23" s="71" t="n"/>
-      <c r="M23" s="71" t="n"/>
-      <c r="N23" s="71" t="n"/>
-      <c r="O23" s="71" t="n"/>
-      <c r="P23" s="71" t="n"/>
-      <c r="Q23" s="71" t="n"/>
-      <c r="R23" s="71" t="n"/>
-      <c r="S23" s="71" t="n"/>
+      <c r="E23" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F23" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I23" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L23" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N23" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O23" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q23" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R23" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="69">
@@ -6487,21 +6527,61 @@
         <f>IF(Partite!$F24="","",Partite!$F24)</f>
         <v/>
       </c>
-      <c r="E24" s="71" t="n"/>
-      <c r="F24" s="71" t="n"/>
-      <c r="G24" s="71" t="n"/>
-      <c r="H24" s="71" t="n"/>
-      <c r="I24" s="71" t="n"/>
-      <c r="J24" s="71" t="n"/>
-      <c r="K24" s="71" t="n"/>
-      <c r="L24" s="71" t="n"/>
-      <c r="M24" s="71" t="n"/>
-      <c r="N24" s="71" t="n"/>
-      <c r="O24" s="71" t="n"/>
-      <c r="P24" s="71" t="n"/>
-      <c r="Q24" s="71" t="n"/>
-      <c r="R24" s="71" t="n"/>
-      <c r="S24" s="71" t="n"/>
+      <c r="E24" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F24" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L24" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N24" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="69">
@@ -6520,21 +6600,61 @@
         <f>IF(Partite!$F25="","",Partite!$F25)</f>
         <v/>
       </c>
-      <c r="E25" s="71" t="n"/>
-      <c r="F25" s="71" t="n"/>
-      <c r="G25" s="71" t="n"/>
-      <c r="H25" s="71" t="n"/>
-      <c r="I25" s="71" t="n"/>
-      <c r="J25" s="71" t="n"/>
-      <c r="K25" s="71" t="n"/>
-      <c r="L25" s="71" t="n"/>
-      <c r="M25" s="71" t="n"/>
-      <c r="N25" s="71" t="n"/>
-      <c r="O25" s="71" t="n"/>
-      <c r="P25" s="71" t="n"/>
-      <c r="Q25" s="71" t="n"/>
-      <c r="R25" s="71" t="n"/>
-      <c r="S25" s="71" t="n"/>
+      <c r="E25" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F25" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I25" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L25" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O25" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R25" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="69">
@@ -6553,21 +6673,61 @@
         <f>IF(Partite!$F26="","",Partite!$F26)</f>
         <v/>
       </c>
-      <c r="E26" s="71" t="n"/>
-      <c r="F26" s="71" t="n"/>
-      <c r="G26" s="71" t="n"/>
-      <c r="H26" s="71" t="n"/>
-      <c r="I26" s="71" t="n"/>
-      <c r="J26" s="71" t="n"/>
-      <c r="K26" s="71" t="n"/>
-      <c r="L26" s="71" t="n"/>
-      <c r="M26" s="71" t="n"/>
-      <c r="N26" s="71" t="n"/>
-      <c r="O26" s="71" t="n"/>
-      <c r="P26" s="71" t="n"/>
-      <c r="Q26" s="71" t="n"/>
-      <c r="R26" s="71" t="n"/>
-      <c r="S26" s="71" t="n"/>
+      <c r="E26" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F26" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L26" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O26" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q26" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R26" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" s="71" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="69">
@@ -6586,21 +6746,61 @@
         <f>IF(Partite!$F27="","",Partite!$F27)</f>
         <v/>
       </c>
-      <c r="E27" s="71" t="n"/>
-      <c r="F27" s="71" t="n"/>
-      <c r="G27" s="71" t="n"/>
-      <c r="H27" s="71" t="n"/>
-      <c r="I27" s="71" t="n"/>
-      <c r="J27" s="71" t="n"/>
-      <c r="K27" s="71" t="n"/>
-      <c r="L27" s="71" t="n"/>
-      <c r="M27" s="71" t="n"/>
-      <c r="N27" s="71" t="n"/>
-      <c r="O27" s="71" t="n"/>
-      <c r="P27" s="71" t="n"/>
-      <c r="Q27" s="71" t="n"/>
-      <c r="R27" s="71" t="n"/>
-      <c r="S27" s="71" t="n"/>
+      <c r="E27" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F27" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I27" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L27" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O27" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P27" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S27" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="69">
@@ -6619,21 +6819,61 @@
         <f>IF(Partite!$F28="","",Partite!$F28)</f>
         <v/>
       </c>
-      <c r="E28" s="71" t="n"/>
-      <c r="F28" s="71" t="n"/>
-      <c r="G28" s="71" t="n"/>
-      <c r="H28" s="71" t="n"/>
-      <c r="I28" s="71" t="n"/>
-      <c r="J28" s="71" t="n"/>
-      <c r="K28" s="71" t="n"/>
-      <c r="L28" s="71" t="n"/>
-      <c r="M28" s="71" t="n"/>
-      <c r="N28" s="71" t="n"/>
-      <c r="O28" s="71" t="n"/>
-      <c r="P28" s="71" t="n"/>
-      <c r="Q28" s="71" t="n"/>
-      <c r="R28" s="71" t="n"/>
-      <c r="S28" s="71" t="n"/>
+      <c r="E28" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F28" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L28" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N28" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O28" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P28" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q28" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R28" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="69">
@@ -6652,21 +6892,61 @@
         <f>IF(Partite!$F29="","",Partite!$F29)</f>
         <v/>
       </c>
-      <c r="E29" s="71" t="n"/>
-      <c r="F29" s="71" t="n"/>
-      <c r="G29" s="71" t="n"/>
-      <c r="H29" s="71" t="n"/>
-      <c r="I29" s="71" t="n"/>
-      <c r="J29" s="71" t="n"/>
-      <c r="K29" s="71" t="n"/>
-      <c r="L29" s="71" t="n"/>
-      <c r="M29" s="71" t="n"/>
-      <c r="N29" s="71" t="n"/>
-      <c r="O29" s="71" t="n"/>
-      <c r="P29" s="71" t="n"/>
-      <c r="Q29" s="71" t="n"/>
-      <c r="R29" s="71" t="n"/>
-      <c r="S29" s="71" t="n"/>
+      <c r="E29" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F29" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I29" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L29" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M29" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N29" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O29" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P29" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S29" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="69">
@@ -6685,21 +6965,61 @@
         <f>IF(Partite!$F30="","",Partite!$F30)</f>
         <v/>
       </c>
-      <c r="E30" s="71" t="n"/>
-      <c r="F30" s="71" t="n"/>
-      <c r="G30" s="71" t="n"/>
-      <c r="H30" s="71" t="n"/>
-      <c r="I30" s="71" t="n"/>
-      <c r="J30" s="71" t="n"/>
-      <c r="K30" s="71" t="n"/>
-      <c r="L30" s="71" t="n"/>
-      <c r="M30" s="71" t="n"/>
-      <c r="N30" s="71" t="n"/>
-      <c r="O30" s="71" t="n"/>
-      <c r="P30" s="71" t="n"/>
-      <c r="Q30" s="71" t="n"/>
-      <c r="R30" s="71" t="n"/>
-      <c r="S30" s="71" t="n"/>
+      <c r="E30" s="71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="71" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R30" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S30" s="71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="69">
@@ -6718,21 +7038,61 @@
         <f>IF(Partite!$F31="","",Partite!$F31)</f>
         <v/>
       </c>
-      <c r="E31" s="71" t="n"/>
-      <c r="F31" s="71" t="n"/>
-      <c r="G31" s="71" t="n"/>
-      <c r="H31" s="71" t="n"/>
-      <c r="I31" s="71" t="n"/>
-      <c r="J31" s="71" t="n"/>
-      <c r="K31" s="71" t="n"/>
-      <c r="L31" s="71" t="n"/>
-      <c r="M31" s="71" t="n"/>
-      <c r="N31" s="71" t="n"/>
-      <c r="O31" s="71" t="n"/>
-      <c r="P31" s="71" t="n"/>
-      <c r="Q31" s="71" t="n"/>
-      <c r="R31" s="71" t="n"/>
-      <c r="S31" s="71" t="n"/>
+      <c r="E31" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I31" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L31" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O31" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="69">
@@ -6751,21 +7111,61 @@
         <f>IF(Partite!$F32="","",Partite!$F32)</f>
         <v/>
       </c>
-      <c r="E32" s="71" t="n"/>
-      <c r="F32" s="71" t="n"/>
-      <c r="G32" s="71" t="n"/>
-      <c r="H32" s="71" t="n"/>
-      <c r="I32" s="71" t="n"/>
-      <c r="J32" s="71" t="n"/>
-      <c r="K32" s="71" t="n"/>
-      <c r="L32" s="71" t="n"/>
-      <c r="M32" s="71" t="n"/>
-      <c r="N32" s="71" t="n"/>
-      <c r="O32" s="71" t="n"/>
-      <c r="P32" s="71" t="n"/>
-      <c r="Q32" s="71" t="n"/>
-      <c r="R32" s="71" t="n"/>
-      <c r="S32" s="71" t="n"/>
+      <c r="E32" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I32" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L32" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="M32" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O32" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="P32" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="71" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="S32" s="71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="74">

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/09/2026 alle 22:15
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -1595,11 +1595,11 @@
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$7)+COUNTIF(Punti!$D$3:$D$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$7)+COUNTIF(Punti!$D$3:$D$52,Config!$D$6)+COUNTIF(Punti!$D$3:$D$52,Config!$D$10)+COUNTIF(Punti!$D$3:$D$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$D$3:$D$52,Config!$D$6)+COUNTIF(Punti!$D$3:$D$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="F12" s="25">
@@ -1629,11 +1629,11 @@
         <v/>
       </c>
       <c r="D13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$7)+COUNTIF(Punti!$E$3:$E$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$7)+COUNTIF(Punti!$E$3:$E$52,Config!$D$6)+COUNTIF(Punti!$E$3:$E$52,Config!$D$10)+COUNTIF(Punti!$E$3:$E$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="E13" s="30">
-        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$E$3:$E$52,Config!$D$6)+COUNTIF(Punti!$E$3:$E$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="F13" s="30">
@@ -1663,11 +1663,11 @@
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$7)+COUNTIF(Punti!$F$3:$F$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$7)+COUNTIF(Punti!$F$3:$F$52,Config!$D$6)+COUNTIF(Punti!$F$3:$F$52,Config!$D$10)+COUNTIF(Punti!$F$3:$F$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$F$3:$F$52,Config!$D$6)+COUNTIF(Punti!$F$3:$F$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="F14" s="25">
@@ -1697,11 +1697,11 @@
         <v/>
       </c>
       <c r="D15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$7)+COUNTIF(Punti!$G$3:$G$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$7)+COUNTIF(Punti!$G$3:$G$52,Config!$D$6)+COUNTIF(Punti!$G$3:$G$52,Config!$D$10)+COUNTIF(Punti!$G$3:$G$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="E15" s="30">
-        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$G$3:$G$52,Config!$D$6)+COUNTIF(Punti!$G$3:$G$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="F15" s="30">
@@ -1731,11 +1731,11 @@
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$7)+COUNTIF(Punti!$H$3:$H$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$7)+COUNTIF(Punti!$H$3:$H$52,Config!$D$6)+COUNTIF(Punti!$H$3:$H$52,Config!$D$10)+COUNTIF(Punti!$H$3:$H$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$6)</f>
+        <f>COUNTIF(Punti!$H$3:$H$52,Config!$D$6)+COUNTIF(Punti!$H$3:$H$52,Config!$D$9)</f>
         <v/>
       </c>
       <c r="F16" s="25">
@@ -7853,7 +7853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:T52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7869,6 +7869,11 @@
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -7886,7 +7891,7 @@
       <c r="H1" s="2" t="n"/>
       <c r="J1" s="35" t="inlineStr">
         <is>
-          <t>servizio: segno effettivo (dichiarato, o dedotto dal punteggio)</t>
+          <t>servizio: a sinistra il segno effettivo (dichiarato, o dedotto dal punteggio), a destra il punteggio scritto. Servono a vedere chi era da solo.</t>
         </is>
       </c>
     </row>
@@ -7943,6 +7948,26 @@
         <v/>
       </c>
       <c r="N2" s="60">
+        <f>Config!$A$10</f>
+        <v/>
+      </c>
+      <c r="P2" s="60">
+        <f>Config!$A$6</f>
+        <v/>
+      </c>
+      <c r="Q2" s="60">
+        <f>Config!$A$7</f>
+        <v/>
+      </c>
+      <c r="R2" s="60">
+        <f>Config!$A$8</f>
+        <v/>
+      </c>
+      <c r="S2" s="60">
+        <f>Config!$A$9</f>
+        <v/>
+      </c>
+      <c r="T2" s="60">
         <f>Config!$A$10</f>
         <v/>
       </c>
@@ -7961,23 +7986,23 @@
         <v/>
       </c>
       <c r="D3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$F3&lt;&gt;"",Pronostici!$G3&lt;&gt;"",Pronostici!$F3=Partite!$G3,Pronostici!$G3=Partite!$H3),Config!$D$6,IF(AND($J3&lt;&gt;"",$J3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$F3&lt;&gt;"",Pronostici!$G3&lt;&gt;"",Pronostici!$F3=Partite!$G3,Pronostici!$G3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$P3)=1),Config!$D$9,Config!$D$6),IF(AND($J3&lt;&gt;"",$J3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$J3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$I3&lt;&gt;"",Pronostici!$J3&lt;&gt;"",Pronostici!$I3=Partite!$G3,Pronostici!$J3=Partite!$H3),Config!$D$6,IF(AND($K3&lt;&gt;"",$K3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$I3&lt;&gt;"",Pronostici!$J3&lt;&gt;"",Pronostici!$I3=Partite!$G3,Pronostici!$J3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$Q3)=1),Config!$D$9,Config!$D$6),IF(AND($K3&lt;&gt;"",$K3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$K3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$L3&lt;&gt;"",Pronostici!$M3&lt;&gt;"",Pronostici!$L3=Partite!$G3,Pronostici!$M3=Partite!$H3),Config!$D$6,IF(AND($L3&lt;&gt;"",$L3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$L3&lt;&gt;"",Pronostici!$M3&lt;&gt;"",Pronostici!$L3=Partite!$G3,Pronostici!$M3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$R3)=1),Config!$D$9,Config!$D$6),IF(AND($L3&lt;&gt;"",$L3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$L3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$O3&lt;&gt;"",Pronostici!$P3&lt;&gt;"",Pronostici!$O3=Partite!$G3,Pronostici!$P3=Partite!$H3),Config!$D$6,IF(AND($M3&lt;&gt;"",$M3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$O3&lt;&gt;"",Pronostici!$P3&lt;&gt;"",Pronostici!$O3=Partite!$G3,Pronostici!$P3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$S3)=1),Config!$D$9,Config!$D$6),IF(AND($M3&lt;&gt;"",$M3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$M3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H3" s="22">
-        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$R3&lt;&gt;"",Pronostici!$S3&lt;&gt;"",Pronostici!$R3=Partite!$G3,Pronostici!$S3=Partite!$H3),Config!$D$6,IF(AND($N3&lt;&gt;"",$N3=Partite!$I3),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K3&lt;&gt;"Giocata","",IF(AND(Pronostici!$R3&lt;&gt;"",Pronostici!$S3&lt;&gt;"",Pronostici!$R3=Partite!$G3,Pronostici!$S3=Partite!$H3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($P3:$T3,$T3)=1),Config!$D$9,Config!$D$6),IF(AND($N3&lt;&gt;"",$N3=Partite!$I3),IF(AND($B3&gt;=Config!$D$17,COUNTIF($J3:$N3,$N3)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J3" s="63">
@@ -7998,6 +8023,26 @@
       </c>
       <c r="N3" s="63">
         <f>IF(Pronostici!$Q3&lt;&gt;"",UPPER(Pronostici!$Q3),IF(OR(Pronostici!$R3="",Pronostici!$S3=""),"",IF(Pronostici!$R3&gt;Pronostici!$S3,"1",IF(Pronostici!$R3=Pronostici!$S3,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P3" s="63">
+        <f>IF(OR(Pronostici!$F3="",Pronostici!$G3=""),"",Pronostici!$F3&amp;" a "&amp;Pronostici!$G3)</f>
+        <v/>
+      </c>
+      <c r="Q3" s="63">
+        <f>IF(OR(Pronostici!$I3="",Pronostici!$J3=""),"",Pronostici!$I3&amp;" a "&amp;Pronostici!$J3)</f>
+        <v/>
+      </c>
+      <c r="R3" s="63">
+        <f>IF(OR(Pronostici!$L3="",Pronostici!$M3=""),"",Pronostici!$L3&amp;" a "&amp;Pronostici!$M3)</f>
+        <v/>
+      </c>
+      <c r="S3" s="63">
+        <f>IF(OR(Pronostici!$O3="",Pronostici!$P3=""),"",Pronostici!$O3&amp;" a "&amp;Pronostici!$P3)</f>
+        <v/>
+      </c>
+      <c r="T3" s="63">
+        <f>IF(OR(Pronostici!$R3="",Pronostici!$S3=""),"",Pronostici!$R3&amp;" a "&amp;Pronostici!$S3)</f>
         <v/>
       </c>
     </row>
@@ -8015,23 +8060,23 @@
         <v/>
       </c>
       <c r="D4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$F4&lt;&gt;"",Pronostici!$G4&lt;&gt;"",Pronostici!$F4=Partite!$G4,Pronostici!$G4=Partite!$H4),Config!$D$6,IF(AND($J4&lt;&gt;"",$J4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$F4&lt;&gt;"",Pronostici!$G4&lt;&gt;"",Pronostici!$F4=Partite!$G4,Pronostici!$G4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$P4)=1),Config!$D$9,Config!$D$6),IF(AND($J4&lt;&gt;"",$J4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$J4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$I4&lt;&gt;"",Pronostici!$J4&lt;&gt;"",Pronostici!$I4=Partite!$G4,Pronostici!$J4=Partite!$H4),Config!$D$6,IF(AND($K4&lt;&gt;"",$K4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$I4&lt;&gt;"",Pronostici!$J4&lt;&gt;"",Pronostici!$I4=Partite!$G4,Pronostici!$J4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$Q4)=1),Config!$D$9,Config!$D$6),IF(AND($K4&lt;&gt;"",$K4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$K4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$L4&lt;&gt;"",Pronostici!$M4&lt;&gt;"",Pronostici!$L4=Partite!$G4,Pronostici!$M4=Partite!$H4),Config!$D$6,IF(AND($L4&lt;&gt;"",$L4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$L4&lt;&gt;"",Pronostici!$M4&lt;&gt;"",Pronostici!$L4=Partite!$G4,Pronostici!$M4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$R4)=1),Config!$D$9,Config!$D$6),IF(AND($L4&lt;&gt;"",$L4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$L4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$O4&lt;&gt;"",Pronostici!$P4&lt;&gt;"",Pronostici!$O4=Partite!$G4,Pronostici!$P4=Partite!$H4),Config!$D$6,IF(AND($M4&lt;&gt;"",$M4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$O4&lt;&gt;"",Pronostici!$P4&lt;&gt;"",Pronostici!$O4=Partite!$G4,Pronostici!$P4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$S4)=1),Config!$D$9,Config!$D$6),IF(AND($M4&lt;&gt;"",$M4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$M4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H4" s="22">
-        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$R4&lt;&gt;"",Pronostici!$S4&lt;&gt;"",Pronostici!$R4=Partite!$G4,Pronostici!$S4=Partite!$H4),Config!$D$6,IF(AND($N4&lt;&gt;"",$N4=Partite!$I4),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K4&lt;&gt;"Giocata","",IF(AND(Pronostici!$R4&lt;&gt;"",Pronostici!$S4&lt;&gt;"",Pronostici!$R4=Partite!$G4,Pronostici!$S4=Partite!$H4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($P4:$T4,$T4)=1),Config!$D$9,Config!$D$6),IF(AND($N4&lt;&gt;"",$N4=Partite!$I4),IF(AND($B4&gt;=Config!$D$17,COUNTIF($J4:$N4,$N4)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J4" s="63">
@@ -8052,6 +8097,26 @@
       </c>
       <c r="N4" s="63">
         <f>IF(Pronostici!$Q4&lt;&gt;"",UPPER(Pronostici!$Q4),IF(OR(Pronostici!$R4="",Pronostici!$S4=""),"",IF(Pronostici!$R4&gt;Pronostici!$S4,"1",IF(Pronostici!$R4=Pronostici!$S4,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P4" s="63">
+        <f>IF(OR(Pronostici!$F4="",Pronostici!$G4=""),"",Pronostici!$F4&amp;" a "&amp;Pronostici!$G4)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="63">
+        <f>IF(OR(Pronostici!$I4="",Pronostici!$J4=""),"",Pronostici!$I4&amp;" a "&amp;Pronostici!$J4)</f>
+        <v/>
+      </c>
+      <c r="R4" s="63">
+        <f>IF(OR(Pronostici!$L4="",Pronostici!$M4=""),"",Pronostici!$L4&amp;" a "&amp;Pronostici!$M4)</f>
+        <v/>
+      </c>
+      <c r="S4" s="63">
+        <f>IF(OR(Pronostici!$O4="",Pronostici!$P4=""),"",Pronostici!$O4&amp;" a "&amp;Pronostici!$P4)</f>
+        <v/>
+      </c>
+      <c r="T4" s="63">
+        <f>IF(OR(Pronostici!$R4="",Pronostici!$S4=""),"",Pronostici!$R4&amp;" a "&amp;Pronostici!$S4)</f>
         <v/>
       </c>
     </row>
@@ -8069,23 +8134,23 @@
         <v/>
       </c>
       <c r="D5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$F5&lt;&gt;"",Pronostici!$G5&lt;&gt;"",Pronostici!$F5=Partite!$G5,Pronostici!$G5=Partite!$H5),Config!$D$6,IF(AND($J5&lt;&gt;"",$J5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$F5&lt;&gt;"",Pronostici!$G5&lt;&gt;"",Pronostici!$F5=Partite!$G5,Pronostici!$G5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$P5)=1),Config!$D$9,Config!$D$6),IF(AND($J5&lt;&gt;"",$J5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$J5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$I5&lt;&gt;"",Pronostici!$J5&lt;&gt;"",Pronostici!$I5=Partite!$G5,Pronostici!$J5=Partite!$H5),Config!$D$6,IF(AND($K5&lt;&gt;"",$K5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$I5&lt;&gt;"",Pronostici!$J5&lt;&gt;"",Pronostici!$I5=Partite!$G5,Pronostici!$J5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$Q5)=1),Config!$D$9,Config!$D$6),IF(AND($K5&lt;&gt;"",$K5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$K5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$L5&lt;&gt;"",Pronostici!$M5&lt;&gt;"",Pronostici!$L5=Partite!$G5,Pronostici!$M5=Partite!$H5),Config!$D$6,IF(AND($L5&lt;&gt;"",$L5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$L5&lt;&gt;"",Pronostici!$M5&lt;&gt;"",Pronostici!$L5=Partite!$G5,Pronostici!$M5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$R5)=1),Config!$D$9,Config!$D$6),IF(AND($L5&lt;&gt;"",$L5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$L5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$O5&lt;&gt;"",Pronostici!$P5&lt;&gt;"",Pronostici!$O5=Partite!$G5,Pronostici!$P5=Partite!$H5),Config!$D$6,IF(AND($M5&lt;&gt;"",$M5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$O5&lt;&gt;"",Pronostici!$P5&lt;&gt;"",Pronostici!$O5=Partite!$G5,Pronostici!$P5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$S5)=1),Config!$D$9,Config!$D$6),IF(AND($M5&lt;&gt;"",$M5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$M5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H5" s="22">
-        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$R5&lt;&gt;"",Pronostici!$S5&lt;&gt;"",Pronostici!$R5=Partite!$G5,Pronostici!$S5=Partite!$H5),Config!$D$6,IF(AND($N5&lt;&gt;"",$N5=Partite!$I5),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K5&lt;&gt;"Giocata","",IF(AND(Pronostici!$R5&lt;&gt;"",Pronostici!$S5&lt;&gt;"",Pronostici!$R5=Partite!$G5,Pronostici!$S5=Partite!$H5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($P5:$T5,$T5)=1),Config!$D$9,Config!$D$6),IF(AND($N5&lt;&gt;"",$N5=Partite!$I5),IF(AND($B5&gt;=Config!$D$17,COUNTIF($J5:$N5,$N5)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J5" s="63">
@@ -8106,6 +8171,26 @@
       </c>
       <c r="N5" s="63">
         <f>IF(Pronostici!$Q5&lt;&gt;"",UPPER(Pronostici!$Q5),IF(OR(Pronostici!$R5="",Pronostici!$S5=""),"",IF(Pronostici!$R5&gt;Pronostici!$S5,"1",IF(Pronostici!$R5=Pronostici!$S5,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P5" s="63">
+        <f>IF(OR(Pronostici!$F5="",Pronostici!$G5=""),"",Pronostici!$F5&amp;" a "&amp;Pronostici!$G5)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="63">
+        <f>IF(OR(Pronostici!$I5="",Pronostici!$J5=""),"",Pronostici!$I5&amp;" a "&amp;Pronostici!$J5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="63">
+        <f>IF(OR(Pronostici!$L5="",Pronostici!$M5=""),"",Pronostici!$L5&amp;" a "&amp;Pronostici!$M5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="63">
+        <f>IF(OR(Pronostici!$O5="",Pronostici!$P5=""),"",Pronostici!$O5&amp;" a "&amp;Pronostici!$P5)</f>
+        <v/>
+      </c>
+      <c r="T5" s="63">
+        <f>IF(OR(Pronostici!$R5="",Pronostici!$S5=""),"",Pronostici!$R5&amp;" a "&amp;Pronostici!$S5)</f>
         <v/>
       </c>
     </row>
@@ -8123,23 +8208,23 @@
         <v/>
       </c>
       <c r="D6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$F6&lt;&gt;"",Pronostici!$G6&lt;&gt;"",Pronostici!$F6=Partite!$G6,Pronostici!$G6=Partite!$H6),Config!$D$6,IF(AND($J6&lt;&gt;"",$J6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$F6&lt;&gt;"",Pronostici!$G6&lt;&gt;"",Pronostici!$F6=Partite!$G6,Pronostici!$G6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$P6)=1),Config!$D$9,Config!$D$6),IF(AND($J6&lt;&gt;"",$J6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$J6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$I6&lt;&gt;"",Pronostici!$J6&lt;&gt;"",Pronostici!$I6=Partite!$G6,Pronostici!$J6=Partite!$H6),Config!$D$6,IF(AND($K6&lt;&gt;"",$K6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$I6&lt;&gt;"",Pronostici!$J6&lt;&gt;"",Pronostici!$I6=Partite!$G6,Pronostici!$J6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$Q6)=1),Config!$D$9,Config!$D$6),IF(AND($K6&lt;&gt;"",$K6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$K6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$L6&lt;&gt;"",Pronostici!$M6&lt;&gt;"",Pronostici!$L6=Partite!$G6,Pronostici!$M6=Partite!$H6),Config!$D$6,IF(AND($L6&lt;&gt;"",$L6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$L6&lt;&gt;"",Pronostici!$M6&lt;&gt;"",Pronostici!$L6=Partite!$G6,Pronostici!$M6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$R6)=1),Config!$D$9,Config!$D$6),IF(AND($L6&lt;&gt;"",$L6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$L6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$O6&lt;&gt;"",Pronostici!$P6&lt;&gt;"",Pronostici!$O6=Partite!$G6,Pronostici!$P6=Partite!$H6),Config!$D$6,IF(AND($M6&lt;&gt;"",$M6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$O6&lt;&gt;"",Pronostici!$P6&lt;&gt;"",Pronostici!$O6=Partite!$G6,Pronostici!$P6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$S6)=1),Config!$D$9,Config!$D$6),IF(AND($M6&lt;&gt;"",$M6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$M6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$R6&lt;&gt;"",Pronostici!$S6&lt;&gt;"",Pronostici!$R6=Partite!$G6,Pronostici!$S6=Partite!$H6),Config!$D$6,IF(AND($N6&lt;&gt;"",$N6=Partite!$I6),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K6&lt;&gt;"Giocata","",IF(AND(Pronostici!$R6&lt;&gt;"",Pronostici!$S6&lt;&gt;"",Pronostici!$R6=Partite!$G6,Pronostici!$S6=Partite!$H6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($P6:$T6,$T6)=1),Config!$D$9,Config!$D$6),IF(AND($N6&lt;&gt;"",$N6=Partite!$I6),IF(AND($B6&gt;=Config!$D$17,COUNTIF($J6:$N6,$N6)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J6" s="63">
@@ -8160,6 +8245,26 @@
       </c>
       <c r="N6" s="63">
         <f>IF(Pronostici!$Q6&lt;&gt;"",UPPER(Pronostici!$Q6),IF(OR(Pronostici!$R6="",Pronostici!$S6=""),"",IF(Pronostici!$R6&gt;Pronostici!$S6,"1",IF(Pronostici!$R6=Pronostici!$S6,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P6" s="63">
+        <f>IF(OR(Pronostici!$F6="",Pronostici!$G6=""),"",Pronostici!$F6&amp;" a "&amp;Pronostici!$G6)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="63">
+        <f>IF(OR(Pronostici!$I6="",Pronostici!$J6=""),"",Pronostici!$I6&amp;" a "&amp;Pronostici!$J6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="63">
+        <f>IF(OR(Pronostici!$L6="",Pronostici!$M6=""),"",Pronostici!$L6&amp;" a "&amp;Pronostici!$M6)</f>
+        <v/>
+      </c>
+      <c r="S6" s="63">
+        <f>IF(OR(Pronostici!$O6="",Pronostici!$P6=""),"",Pronostici!$O6&amp;" a "&amp;Pronostici!$P6)</f>
+        <v/>
+      </c>
+      <c r="T6" s="63">
+        <f>IF(OR(Pronostici!$R6="",Pronostici!$S6=""),"",Pronostici!$R6&amp;" a "&amp;Pronostici!$S6)</f>
         <v/>
       </c>
     </row>
@@ -8177,23 +8282,23 @@
         <v/>
       </c>
       <c r="D7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$F7&lt;&gt;"",Pronostici!$G7&lt;&gt;"",Pronostici!$F7=Partite!$G7,Pronostici!$G7=Partite!$H7),Config!$D$6,IF(AND($J7&lt;&gt;"",$J7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$F7&lt;&gt;"",Pronostici!$G7&lt;&gt;"",Pronostici!$F7=Partite!$G7,Pronostici!$G7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$P7)=1),Config!$D$9,Config!$D$6),IF(AND($J7&lt;&gt;"",$J7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$J7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$I7&lt;&gt;"",Pronostici!$J7&lt;&gt;"",Pronostici!$I7=Partite!$G7,Pronostici!$J7=Partite!$H7),Config!$D$6,IF(AND($K7&lt;&gt;"",$K7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$I7&lt;&gt;"",Pronostici!$J7&lt;&gt;"",Pronostici!$I7=Partite!$G7,Pronostici!$J7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$Q7)=1),Config!$D$9,Config!$D$6),IF(AND($K7&lt;&gt;"",$K7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$K7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$L7&lt;&gt;"",Pronostici!$M7&lt;&gt;"",Pronostici!$L7=Partite!$G7,Pronostici!$M7=Partite!$H7),Config!$D$6,IF(AND($L7&lt;&gt;"",$L7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$L7&lt;&gt;"",Pronostici!$M7&lt;&gt;"",Pronostici!$L7=Partite!$G7,Pronostici!$M7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$R7)=1),Config!$D$9,Config!$D$6),IF(AND($L7&lt;&gt;"",$L7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$L7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$O7&lt;&gt;"",Pronostici!$P7&lt;&gt;"",Pronostici!$O7=Partite!$G7,Pronostici!$P7=Partite!$H7),Config!$D$6,IF(AND($M7&lt;&gt;"",$M7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$O7&lt;&gt;"",Pronostici!$P7&lt;&gt;"",Pronostici!$O7=Partite!$G7,Pronostici!$P7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$S7)=1),Config!$D$9,Config!$D$6),IF(AND($M7&lt;&gt;"",$M7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$M7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H7" s="22">
-        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$R7&lt;&gt;"",Pronostici!$S7&lt;&gt;"",Pronostici!$R7=Partite!$G7,Pronostici!$S7=Partite!$H7),Config!$D$6,IF(AND($N7&lt;&gt;"",$N7=Partite!$I7),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K7&lt;&gt;"Giocata","",IF(AND(Pronostici!$R7&lt;&gt;"",Pronostici!$S7&lt;&gt;"",Pronostici!$R7=Partite!$G7,Pronostici!$S7=Partite!$H7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($P7:$T7,$T7)=1),Config!$D$9,Config!$D$6),IF(AND($N7&lt;&gt;"",$N7=Partite!$I7),IF(AND($B7&gt;=Config!$D$17,COUNTIF($J7:$N7,$N7)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J7" s="63">
@@ -8214,6 +8319,26 @@
       </c>
       <c r="N7" s="63">
         <f>IF(Pronostici!$Q7&lt;&gt;"",UPPER(Pronostici!$Q7),IF(OR(Pronostici!$R7="",Pronostici!$S7=""),"",IF(Pronostici!$R7&gt;Pronostici!$S7,"1",IF(Pronostici!$R7=Pronostici!$S7,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P7" s="63">
+        <f>IF(OR(Pronostici!$F7="",Pronostici!$G7=""),"",Pronostici!$F7&amp;" a "&amp;Pronostici!$G7)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="63">
+        <f>IF(OR(Pronostici!$I7="",Pronostici!$J7=""),"",Pronostici!$I7&amp;" a "&amp;Pronostici!$J7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="63">
+        <f>IF(OR(Pronostici!$L7="",Pronostici!$M7=""),"",Pronostici!$L7&amp;" a "&amp;Pronostici!$M7)</f>
+        <v/>
+      </c>
+      <c r="S7" s="63">
+        <f>IF(OR(Pronostici!$O7="",Pronostici!$P7=""),"",Pronostici!$O7&amp;" a "&amp;Pronostici!$P7)</f>
+        <v/>
+      </c>
+      <c r="T7" s="63">
+        <f>IF(OR(Pronostici!$R7="",Pronostici!$S7=""),"",Pronostici!$R7&amp;" a "&amp;Pronostici!$S7)</f>
         <v/>
       </c>
     </row>
@@ -8231,23 +8356,23 @@
         <v/>
       </c>
       <c r="D8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$F8&lt;&gt;"",Pronostici!$G8&lt;&gt;"",Pronostici!$F8=Partite!$G8,Pronostici!$G8=Partite!$H8),Config!$D$6,IF(AND($J8&lt;&gt;"",$J8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$F8&lt;&gt;"",Pronostici!$G8&lt;&gt;"",Pronostici!$F8=Partite!$G8,Pronostici!$G8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$P8)=1),Config!$D$9,Config!$D$6),IF(AND($J8&lt;&gt;"",$J8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$J8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$I8&lt;&gt;"",Pronostici!$J8&lt;&gt;"",Pronostici!$I8=Partite!$G8,Pronostici!$J8=Partite!$H8),Config!$D$6,IF(AND($K8&lt;&gt;"",$K8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$I8&lt;&gt;"",Pronostici!$J8&lt;&gt;"",Pronostici!$I8=Partite!$G8,Pronostici!$J8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$Q8)=1),Config!$D$9,Config!$D$6),IF(AND($K8&lt;&gt;"",$K8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$K8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$L8&lt;&gt;"",Pronostici!$M8&lt;&gt;"",Pronostici!$L8=Partite!$G8,Pronostici!$M8=Partite!$H8),Config!$D$6,IF(AND($L8&lt;&gt;"",$L8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$L8&lt;&gt;"",Pronostici!$M8&lt;&gt;"",Pronostici!$L8=Partite!$G8,Pronostici!$M8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$R8)=1),Config!$D$9,Config!$D$6),IF(AND($L8&lt;&gt;"",$L8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$L8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$O8&lt;&gt;"",Pronostici!$P8&lt;&gt;"",Pronostici!$O8=Partite!$G8,Pronostici!$P8=Partite!$H8),Config!$D$6,IF(AND($M8&lt;&gt;"",$M8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$O8&lt;&gt;"",Pronostici!$P8&lt;&gt;"",Pronostici!$O8=Partite!$G8,Pronostici!$P8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$S8)=1),Config!$D$9,Config!$D$6),IF(AND($M8&lt;&gt;"",$M8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$M8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$R8&lt;&gt;"",Pronostici!$S8&lt;&gt;"",Pronostici!$R8=Partite!$G8,Pronostici!$S8=Partite!$H8),Config!$D$6,IF(AND($N8&lt;&gt;"",$N8=Partite!$I8),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K8&lt;&gt;"Giocata","",IF(AND(Pronostici!$R8&lt;&gt;"",Pronostici!$S8&lt;&gt;"",Pronostici!$R8=Partite!$G8,Pronostici!$S8=Partite!$H8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($P8:$T8,$T8)=1),Config!$D$9,Config!$D$6),IF(AND($N8&lt;&gt;"",$N8=Partite!$I8),IF(AND($B8&gt;=Config!$D$17,COUNTIF($J8:$N8,$N8)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J8" s="63">
@@ -8268,6 +8393,26 @@
       </c>
       <c r="N8" s="63">
         <f>IF(Pronostici!$Q8&lt;&gt;"",UPPER(Pronostici!$Q8),IF(OR(Pronostici!$R8="",Pronostici!$S8=""),"",IF(Pronostici!$R8&gt;Pronostici!$S8,"1",IF(Pronostici!$R8=Pronostici!$S8,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P8" s="63">
+        <f>IF(OR(Pronostici!$F8="",Pronostici!$G8=""),"",Pronostici!$F8&amp;" a "&amp;Pronostici!$G8)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="63">
+        <f>IF(OR(Pronostici!$I8="",Pronostici!$J8=""),"",Pronostici!$I8&amp;" a "&amp;Pronostici!$J8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="63">
+        <f>IF(OR(Pronostici!$L8="",Pronostici!$M8=""),"",Pronostici!$L8&amp;" a "&amp;Pronostici!$M8)</f>
+        <v/>
+      </c>
+      <c r="S8" s="63">
+        <f>IF(OR(Pronostici!$O8="",Pronostici!$P8=""),"",Pronostici!$O8&amp;" a "&amp;Pronostici!$P8)</f>
+        <v/>
+      </c>
+      <c r="T8" s="63">
+        <f>IF(OR(Pronostici!$R8="",Pronostici!$S8=""),"",Pronostici!$R8&amp;" a "&amp;Pronostici!$S8)</f>
         <v/>
       </c>
     </row>
@@ -8285,23 +8430,23 @@
         <v/>
       </c>
       <c r="D9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$F9&lt;&gt;"",Pronostici!$G9&lt;&gt;"",Pronostici!$F9=Partite!$G9,Pronostici!$G9=Partite!$H9),Config!$D$6,IF(AND($J9&lt;&gt;"",$J9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$F9&lt;&gt;"",Pronostici!$G9&lt;&gt;"",Pronostici!$F9=Partite!$G9,Pronostici!$G9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$P9)=1),Config!$D$9,Config!$D$6),IF(AND($J9&lt;&gt;"",$J9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$J9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$I9&lt;&gt;"",Pronostici!$J9&lt;&gt;"",Pronostici!$I9=Partite!$G9,Pronostici!$J9=Partite!$H9),Config!$D$6,IF(AND($K9&lt;&gt;"",$K9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$I9&lt;&gt;"",Pronostici!$J9&lt;&gt;"",Pronostici!$I9=Partite!$G9,Pronostici!$J9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$Q9)=1),Config!$D$9,Config!$D$6),IF(AND($K9&lt;&gt;"",$K9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$K9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$L9&lt;&gt;"",Pronostici!$M9&lt;&gt;"",Pronostici!$L9=Partite!$G9,Pronostici!$M9=Partite!$H9),Config!$D$6,IF(AND($L9&lt;&gt;"",$L9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$L9&lt;&gt;"",Pronostici!$M9&lt;&gt;"",Pronostici!$L9=Partite!$G9,Pronostici!$M9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$R9)=1),Config!$D$9,Config!$D$6),IF(AND($L9&lt;&gt;"",$L9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$L9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$O9&lt;&gt;"",Pronostici!$P9&lt;&gt;"",Pronostici!$O9=Partite!$G9,Pronostici!$P9=Partite!$H9),Config!$D$6,IF(AND($M9&lt;&gt;"",$M9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$O9&lt;&gt;"",Pronostici!$P9&lt;&gt;"",Pronostici!$O9=Partite!$G9,Pronostici!$P9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$S9)=1),Config!$D$9,Config!$D$6),IF(AND($M9&lt;&gt;"",$M9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$M9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H9" s="22">
-        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$R9&lt;&gt;"",Pronostici!$S9&lt;&gt;"",Pronostici!$R9=Partite!$G9,Pronostici!$S9=Partite!$H9),Config!$D$6,IF(AND($N9&lt;&gt;"",$N9=Partite!$I9),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K9&lt;&gt;"Giocata","",IF(AND(Pronostici!$R9&lt;&gt;"",Pronostici!$S9&lt;&gt;"",Pronostici!$R9=Partite!$G9,Pronostici!$S9=Partite!$H9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($P9:$T9,$T9)=1),Config!$D$9,Config!$D$6),IF(AND($N9&lt;&gt;"",$N9=Partite!$I9),IF(AND($B9&gt;=Config!$D$17,COUNTIF($J9:$N9,$N9)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J9" s="63">
@@ -8322,6 +8467,26 @@
       </c>
       <c r="N9" s="63">
         <f>IF(Pronostici!$Q9&lt;&gt;"",UPPER(Pronostici!$Q9),IF(OR(Pronostici!$R9="",Pronostici!$S9=""),"",IF(Pronostici!$R9&gt;Pronostici!$S9,"1",IF(Pronostici!$R9=Pronostici!$S9,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P9" s="63">
+        <f>IF(OR(Pronostici!$F9="",Pronostici!$G9=""),"",Pronostici!$F9&amp;" a "&amp;Pronostici!$G9)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="63">
+        <f>IF(OR(Pronostici!$I9="",Pronostici!$J9=""),"",Pronostici!$I9&amp;" a "&amp;Pronostici!$J9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="63">
+        <f>IF(OR(Pronostici!$L9="",Pronostici!$M9=""),"",Pronostici!$L9&amp;" a "&amp;Pronostici!$M9)</f>
+        <v/>
+      </c>
+      <c r="S9" s="63">
+        <f>IF(OR(Pronostici!$O9="",Pronostici!$P9=""),"",Pronostici!$O9&amp;" a "&amp;Pronostici!$P9)</f>
+        <v/>
+      </c>
+      <c r="T9" s="63">
+        <f>IF(OR(Pronostici!$R9="",Pronostici!$S9=""),"",Pronostici!$R9&amp;" a "&amp;Pronostici!$S9)</f>
         <v/>
       </c>
     </row>
@@ -8339,23 +8504,23 @@
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$F10&lt;&gt;"",Pronostici!$G10&lt;&gt;"",Pronostici!$F10=Partite!$G10,Pronostici!$G10=Partite!$H10),Config!$D$6,IF(AND($J10&lt;&gt;"",$J10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$F10&lt;&gt;"",Pronostici!$G10&lt;&gt;"",Pronostici!$F10=Partite!$G10,Pronostici!$G10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$P10)=1),Config!$D$9,Config!$D$6),IF(AND($J10&lt;&gt;"",$J10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$J10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$I10&lt;&gt;"",Pronostici!$J10&lt;&gt;"",Pronostici!$I10=Partite!$G10,Pronostici!$J10=Partite!$H10),Config!$D$6,IF(AND($K10&lt;&gt;"",$K10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$I10&lt;&gt;"",Pronostici!$J10&lt;&gt;"",Pronostici!$I10=Partite!$G10,Pronostici!$J10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$Q10)=1),Config!$D$9,Config!$D$6),IF(AND($K10&lt;&gt;"",$K10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$K10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$L10&lt;&gt;"",Pronostici!$M10&lt;&gt;"",Pronostici!$L10=Partite!$G10,Pronostici!$M10=Partite!$H10),Config!$D$6,IF(AND($L10&lt;&gt;"",$L10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$L10&lt;&gt;"",Pronostici!$M10&lt;&gt;"",Pronostici!$L10=Partite!$G10,Pronostici!$M10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$R10)=1),Config!$D$9,Config!$D$6),IF(AND($L10&lt;&gt;"",$L10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$L10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$O10&lt;&gt;"",Pronostici!$P10&lt;&gt;"",Pronostici!$O10=Partite!$G10,Pronostici!$P10=Partite!$H10),Config!$D$6,IF(AND($M10&lt;&gt;"",$M10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$O10&lt;&gt;"",Pronostici!$P10&lt;&gt;"",Pronostici!$O10=Partite!$G10,Pronostici!$P10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$S10)=1),Config!$D$9,Config!$D$6),IF(AND($M10&lt;&gt;"",$M10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$M10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$R10&lt;&gt;"",Pronostici!$S10&lt;&gt;"",Pronostici!$R10=Partite!$G10,Pronostici!$S10=Partite!$H10),Config!$D$6,IF(AND($N10&lt;&gt;"",$N10=Partite!$I10),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K10&lt;&gt;"Giocata","",IF(AND(Pronostici!$R10&lt;&gt;"",Pronostici!$S10&lt;&gt;"",Pronostici!$R10=Partite!$G10,Pronostici!$S10=Partite!$H10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($P10:$T10,$T10)=1),Config!$D$9,Config!$D$6),IF(AND($N10&lt;&gt;"",$N10=Partite!$I10),IF(AND($B10&gt;=Config!$D$17,COUNTIF($J10:$N10,$N10)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J10" s="63">
@@ -8376,6 +8541,26 @@
       </c>
       <c r="N10" s="63">
         <f>IF(Pronostici!$Q10&lt;&gt;"",UPPER(Pronostici!$Q10),IF(OR(Pronostici!$R10="",Pronostici!$S10=""),"",IF(Pronostici!$R10&gt;Pronostici!$S10,"1",IF(Pronostici!$R10=Pronostici!$S10,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P10" s="63">
+        <f>IF(OR(Pronostici!$F10="",Pronostici!$G10=""),"",Pronostici!$F10&amp;" a "&amp;Pronostici!$G10)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="63">
+        <f>IF(OR(Pronostici!$I10="",Pronostici!$J10=""),"",Pronostici!$I10&amp;" a "&amp;Pronostici!$J10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="63">
+        <f>IF(OR(Pronostici!$L10="",Pronostici!$M10=""),"",Pronostici!$L10&amp;" a "&amp;Pronostici!$M10)</f>
+        <v/>
+      </c>
+      <c r="S10" s="63">
+        <f>IF(OR(Pronostici!$O10="",Pronostici!$P10=""),"",Pronostici!$O10&amp;" a "&amp;Pronostici!$P10)</f>
+        <v/>
+      </c>
+      <c r="T10" s="63">
+        <f>IF(OR(Pronostici!$R10="",Pronostici!$S10=""),"",Pronostici!$R10&amp;" a "&amp;Pronostici!$S10)</f>
         <v/>
       </c>
     </row>
@@ -8393,23 +8578,23 @@
         <v/>
       </c>
       <c r="D11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$F11&lt;&gt;"",Pronostici!$G11&lt;&gt;"",Pronostici!$F11=Partite!$G11,Pronostici!$G11=Partite!$H11),Config!$D$6,IF(AND($J11&lt;&gt;"",$J11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$F11&lt;&gt;"",Pronostici!$G11&lt;&gt;"",Pronostici!$F11=Partite!$G11,Pronostici!$G11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$P11)=1),Config!$D$9,Config!$D$6),IF(AND($J11&lt;&gt;"",$J11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$J11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$I11&lt;&gt;"",Pronostici!$J11&lt;&gt;"",Pronostici!$I11=Partite!$G11,Pronostici!$J11=Partite!$H11),Config!$D$6,IF(AND($K11&lt;&gt;"",$K11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$I11&lt;&gt;"",Pronostici!$J11&lt;&gt;"",Pronostici!$I11=Partite!$G11,Pronostici!$J11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$Q11)=1),Config!$D$9,Config!$D$6),IF(AND($K11&lt;&gt;"",$K11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$K11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$L11&lt;&gt;"",Pronostici!$M11&lt;&gt;"",Pronostici!$L11=Partite!$G11,Pronostici!$M11=Partite!$H11),Config!$D$6,IF(AND($L11&lt;&gt;"",$L11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$L11&lt;&gt;"",Pronostici!$M11&lt;&gt;"",Pronostici!$L11=Partite!$G11,Pronostici!$M11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$R11)=1),Config!$D$9,Config!$D$6),IF(AND($L11&lt;&gt;"",$L11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$L11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$O11&lt;&gt;"",Pronostici!$P11&lt;&gt;"",Pronostici!$O11=Partite!$G11,Pronostici!$P11=Partite!$H11),Config!$D$6,IF(AND($M11&lt;&gt;"",$M11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$O11&lt;&gt;"",Pronostici!$P11&lt;&gt;"",Pronostici!$O11=Partite!$G11,Pronostici!$P11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$S11)=1),Config!$D$9,Config!$D$6),IF(AND($M11&lt;&gt;"",$M11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$M11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H11" s="22">
-        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$R11&lt;&gt;"",Pronostici!$S11&lt;&gt;"",Pronostici!$R11=Partite!$G11,Pronostici!$S11=Partite!$H11),Config!$D$6,IF(AND($N11&lt;&gt;"",$N11=Partite!$I11),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K11&lt;&gt;"Giocata","",IF(AND(Pronostici!$R11&lt;&gt;"",Pronostici!$S11&lt;&gt;"",Pronostici!$R11=Partite!$G11,Pronostici!$S11=Partite!$H11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($P11:$T11,$T11)=1),Config!$D$9,Config!$D$6),IF(AND($N11&lt;&gt;"",$N11=Partite!$I11),IF(AND($B11&gt;=Config!$D$17,COUNTIF($J11:$N11,$N11)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J11" s="63">
@@ -8430,6 +8615,26 @@
       </c>
       <c r="N11" s="63">
         <f>IF(Pronostici!$Q11&lt;&gt;"",UPPER(Pronostici!$Q11),IF(OR(Pronostici!$R11="",Pronostici!$S11=""),"",IF(Pronostici!$R11&gt;Pronostici!$S11,"1",IF(Pronostici!$R11=Pronostici!$S11,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P11" s="63">
+        <f>IF(OR(Pronostici!$F11="",Pronostici!$G11=""),"",Pronostici!$F11&amp;" a "&amp;Pronostici!$G11)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="63">
+        <f>IF(OR(Pronostici!$I11="",Pronostici!$J11=""),"",Pronostici!$I11&amp;" a "&amp;Pronostici!$J11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="63">
+        <f>IF(OR(Pronostici!$L11="",Pronostici!$M11=""),"",Pronostici!$L11&amp;" a "&amp;Pronostici!$M11)</f>
+        <v/>
+      </c>
+      <c r="S11" s="63">
+        <f>IF(OR(Pronostici!$O11="",Pronostici!$P11=""),"",Pronostici!$O11&amp;" a "&amp;Pronostici!$P11)</f>
+        <v/>
+      </c>
+      <c r="T11" s="63">
+        <f>IF(OR(Pronostici!$R11="",Pronostici!$S11=""),"",Pronostici!$R11&amp;" a "&amp;Pronostici!$S11)</f>
         <v/>
       </c>
     </row>
@@ -8447,23 +8652,23 @@
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$F12&lt;&gt;"",Pronostici!$G12&lt;&gt;"",Pronostici!$F12=Partite!$G12,Pronostici!$G12=Partite!$H12),Config!$D$6,IF(AND($J12&lt;&gt;"",$J12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$F12&lt;&gt;"",Pronostici!$G12&lt;&gt;"",Pronostici!$F12=Partite!$G12,Pronostici!$G12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$P12)=1),Config!$D$9,Config!$D$6),IF(AND($J12&lt;&gt;"",$J12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$J12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$I12&lt;&gt;"",Pronostici!$J12&lt;&gt;"",Pronostici!$I12=Partite!$G12,Pronostici!$J12=Partite!$H12),Config!$D$6,IF(AND($K12&lt;&gt;"",$K12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$I12&lt;&gt;"",Pronostici!$J12&lt;&gt;"",Pronostici!$I12=Partite!$G12,Pronostici!$J12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$Q12)=1),Config!$D$9,Config!$D$6),IF(AND($K12&lt;&gt;"",$K12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$K12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$L12&lt;&gt;"",Pronostici!$M12&lt;&gt;"",Pronostici!$L12=Partite!$G12,Pronostici!$M12=Partite!$H12),Config!$D$6,IF(AND($L12&lt;&gt;"",$L12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$L12&lt;&gt;"",Pronostici!$M12&lt;&gt;"",Pronostici!$L12=Partite!$G12,Pronostici!$M12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$R12)=1),Config!$D$9,Config!$D$6),IF(AND($L12&lt;&gt;"",$L12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$L12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$O12&lt;&gt;"",Pronostici!$P12&lt;&gt;"",Pronostici!$O12=Partite!$G12,Pronostici!$P12=Partite!$H12),Config!$D$6,IF(AND($M12&lt;&gt;"",$M12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$O12&lt;&gt;"",Pronostici!$P12&lt;&gt;"",Pronostici!$O12=Partite!$G12,Pronostici!$P12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$S12)=1),Config!$D$9,Config!$D$6),IF(AND($M12&lt;&gt;"",$M12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$M12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$R12&lt;&gt;"",Pronostici!$S12&lt;&gt;"",Pronostici!$R12=Partite!$G12,Pronostici!$S12=Partite!$H12),Config!$D$6,IF(AND($N12&lt;&gt;"",$N12=Partite!$I12),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K12&lt;&gt;"Giocata","",IF(AND(Pronostici!$R12&lt;&gt;"",Pronostici!$S12&lt;&gt;"",Pronostici!$R12=Partite!$G12,Pronostici!$S12=Partite!$H12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($P12:$T12,$T12)=1),Config!$D$9,Config!$D$6),IF(AND($N12&lt;&gt;"",$N12=Partite!$I12),IF(AND($B12&gt;=Config!$D$17,COUNTIF($J12:$N12,$N12)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J12" s="63">
@@ -8484,6 +8689,26 @@
       </c>
       <c r="N12" s="63">
         <f>IF(Pronostici!$Q12&lt;&gt;"",UPPER(Pronostici!$Q12),IF(OR(Pronostici!$R12="",Pronostici!$S12=""),"",IF(Pronostici!$R12&gt;Pronostici!$S12,"1",IF(Pronostici!$R12=Pronostici!$S12,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P12" s="63">
+        <f>IF(OR(Pronostici!$F12="",Pronostici!$G12=""),"",Pronostici!$F12&amp;" a "&amp;Pronostici!$G12)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="63">
+        <f>IF(OR(Pronostici!$I12="",Pronostici!$J12=""),"",Pronostici!$I12&amp;" a "&amp;Pronostici!$J12)</f>
+        <v/>
+      </c>
+      <c r="R12" s="63">
+        <f>IF(OR(Pronostici!$L12="",Pronostici!$M12=""),"",Pronostici!$L12&amp;" a "&amp;Pronostici!$M12)</f>
+        <v/>
+      </c>
+      <c r="S12" s="63">
+        <f>IF(OR(Pronostici!$O12="",Pronostici!$P12=""),"",Pronostici!$O12&amp;" a "&amp;Pronostici!$P12)</f>
+        <v/>
+      </c>
+      <c r="T12" s="63">
+        <f>IF(OR(Pronostici!$R12="",Pronostici!$S12=""),"",Pronostici!$R12&amp;" a "&amp;Pronostici!$S12)</f>
         <v/>
       </c>
     </row>
@@ -8501,23 +8726,23 @@
         <v/>
       </c>
       <c r="D13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$F13&lt;&gt;"",Pronostici!$G13&lt;&gt;"",Pronostici!$F13=Partite!$G13,Pronostici!$G13=Partite!$H13),Config!$D$6,IF(AND($J13&lt;&gt;"",$J13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$F13&lt;&gt;"",Pronostici!$G13&lt;&gt;"",Pronostici!$F13=Partite!$G13,Pronostici!$G13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$P13)=1),Config!$D$9,Config!$D$6),IF(AND($J13&lt;&gt;"",$J13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$J13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$I13&lt;&gt;"",Pronostici!$J13&lt;&gt;"",Pronostici!$I13=Partite!$G13,Pronostici!$J13=Partite!$H13),Config!$D$6,IF(AND($K13&lt;&gt;"",$K13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$I13&lt;&gt;"",Pronostici!$J13&lt;&gt;"",Pronostici!$I13=Partite!$G13,Pronostici!$J13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$Q13)=1),Config!$D$9,Config!$D$6),IF(AND($K13&lt;&gt;"",$K13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$K13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$L13&lt;&gt;"",Pronostici!$M13&lt;&gt;"",Pronostici!$L13=Partite!$G13,Pronostici!$M13=Partite!$H13),Config!$D$6,IF(AND($L13&lt;&gt;"",$L13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$L13&lt;&gt;"",Pronostici!$M13&lt;&gt;"",Pronostici!$L13=Partite!$G13,Pronostici!$M13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$R13)=1),Config!$D$9,Config!$D$6),IF(AND($L13&lt;&gt;"",$L13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$L13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$O13&lt;&gt;"",Pronostici!$P13&lt;&gt;"",Pronostici!$O13=Partite!$G13,Pronostici!$P13=Partite!$H13),Config!$D$6,IF(AND($M13&lt;&gt;"",$M13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$O13&lt;&gt;"",Pronostici!$P13&lt;&gt;"",Pronostici!$O13=Partite!$G13,Pronostici!$P13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$S13)=1),Config!$D$9,Config!$D$6),IF(AND($M13&lt;&gt;"",$M13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$M13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H13" s="27">
-        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$R13&lt;&gt;"",Pronostici!$S13&lt;&gt;"",Pronostici!$R13=Partite!$G13,Pronostici!$S13=Partite!$H13),Config!$D$6,IF(AND($N13&lt;&gt;"",$N13=Partite!$I13),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K13&lt;&gt;"Giocata","",IF(AND(Pronostici!$R13&lt;&gt;"",Pronostici!$S13&lt;&gt;"",Pronostici!$R13=Partite!$G13,Pronostici!$S13=Partite!$H13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($P13:$T13,$T13)=1),Config!$D$9,Config!$D$6),IF(AND($N13&lt;&gt;"",$N13=Partite!$I13),IF(AND($B13&gt;=Config!$D$17,COUNTIF($J13:$N13,$N13)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J13" s="63">
@@ -8538,6 +8763,26 @@
       </c>
       <c r="N13" s="63">
         <f>IF(Pronostici!$Q13&lt;&gt;"",UPPER(Pronostici!$Q13),IF(OR(Pronostici!$R13="",Pronostici!$S13=""),"",IF(Pronostici!$R13&gt;Pronostici!$S13,"1",IF(Pronostici!$R13=Pronostici!$S13,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P13" s="63">
+        <f>IF(OR(Pronostici!$F13="",Pronostici!$G13=""),"",Pronostici!$F13&amp;" a "&amp;Pronostici!$G13)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="63">
+        <f>IF(OR(Pronostici!$I13="",Pronostici!$J13=""),"",Pronostici!$I13&amp;" a "&amp;Pronostici!$J13)</f>
+        <v/>
+      </c>
+      <c r="R13" s="63">
+        <f>IF(OR(Pronostici!$L13="",Pronostici!$M13=""),"",Pronostici!$L13&amp;" a "&amp;Pronostici!$M13)</f>
+        <v/>
+      </c>
+      <c r="S13" s="63">
+        <f>IF(OR(Pronostici!$O13="",Pronostici!$P13=""),"",Pronostici!$O13&amp;" a "&amp;Pronostici!$P13)</f>
+        <v/>
+      </c>
+      <c r="T13" s="63">
+        <f>IF(OR(Pronostici!$R13="",Pronostici!$S13=""),"",Pronostici!$R13&amp;" a "&amp;Pronostici!$S13)</f>
         <v/>
       </c>
     </row>
@@ -8555,23 +8800,23 @@
         <v/>
       </c>
       <c r="D14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$F14&lt;&gt;"",Pronostici!$G14&lt;&gt;"",Pronostici!$F14=Partite!$G14,Pronostici!$G14=Partite!$H14),Config!$D$6,IF(AND($J14&lt;&gt;"",$J14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$F14&lt;&gt;"",Pronostici!$G14&lt;&gt;"",Pronostici!$F14=Partite!$G14,Pronostici!$G14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$P14)=1),Config!$D$9,Config!$D$6),IF(AND($J14&lt;&gt;"",$J14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$J14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$I14&lt;&gt;"",Pronostici!$J14&lt;&gt;"",Pronostici!$I14=Partite!$G14,Pronostici!$J14=Partite!$H14),Config!$D$6,IF(AND($K14&lt;&gt;"",$K14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$I14&lt;&gt;"",Pronostici!$J14&lt;&gt;"",Pronostici!$I14=Partite!$G14,Pronostici!$J14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$Q14)=1),Config!$D$9,Config!$D$6),IF(AND($K14&lt;&gt;"",$K14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$K14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$L14&lt;&gt;"",Pronostici!$M14&lt;&gt;"",Pronostici!$L14=Partite!$G14,Pronostici!$M14=Partite!$H14),Config!$D$6,IF(AND($L14&lt;&gt;"",$L14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$L14&lt;&gt;"",Pronostici!$M14&lt;&gt;"",Pronostici!$L14=Partite!$G14,Pronostici!$M14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$R14)=1),Config!$D$9,Config!$D$6),IF(AND($L14&lt;&gt;"",$L14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$L14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$O14&lt;&gt;"",Pronostici!$P14&lt;&gt;"",Pronostici!$O14=Partite!$G14,Pronostici!$P14=Partite!$H14),Config!$D$6,IF(AND($M14&lt;&gt;"",$M14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$O14&lt;&gt;"",Pronostici!$P14&lt;&gt;"",Pronostici!$O14=Partite!$G14,Pronostici!$P14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$S14)=1),Config!$D$9,Config!$D$6),IF(AND($M14&lt;&gt;"",$M14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$M14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H14" s="27">
-        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$R14&lt;&gt;"",Pronostici!$S14&lt;&gt;"",Pronostici!$R14=Partite!$G14,Pronostici!$S14=Partite!$H14),Config!$D$6,IF(AND($N14&lt;&gt;"",$N14=Partite!$I14),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K14&lt;&gt;"Giocata","",IF(AND(Pronostici!$R14&lt;&gt;"",Pronostici!$S14&lt;&gt;"",Pronostici!$R14=Partite!$G14,Pronostici!$S14=Partite!$H14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($P14:$T14,$T14)=1),Config!$D$9,Config!$D$6),IF(AND($N14&lt;&gt;"",$N14=Partite!$I14),IF(AND($B14&gt;=Config!$D$17,COUNTIF($J14:$N14,$N14)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J14" s="63">
@@ -8592,6 +8837,26 @@
       </c>
       <c r="N14" s="63">
         <f>IF(Pronostici!$Q14&lt;&gt;"",UPPER(Pronostici!$Q14),IF(OR(Pronostici!$R14="",Pronostici!$S14=""),"",IF(Pronostici!$R14&gt;Pronostici!$S14,"1",IF(Pronostici!$R14=Pronostici!$S14,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P14" s="63">
+        <f>IF(OR(Pronostici!$F14="",Pronostici!$G14=""),"",Pronostici!$F14&amp;" a "&amp;Pronostici!$G14)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="63">
+        <f>IF(OR(Pronostici!$I14="",Pronostici!$J14=""),"",Pronostici!$I14&amp;" a "&amp;Pronostici!$J14)</f>
+        <v/>
+      </c>
+      <c r="R14" s="63">
+        <f>IF(OR(Pronostici!$L14="",Pronostici!$M14=""),"",Pronostici!$L14&amp;" a "&amp;Pronostici!$M14)</f>
+        <v/>
+      </c>
+      <c r="S14" s="63">
+        <f>IF(OR(Pronostici!$O14="",Pronostici!$P14=""),"",Pronostici!$O14&amp;" a "&amp;Pronostici!$P14)</f>
+        <v/>
+      </c>
+      <c r="T14" s="63">
+        <f>IF(OR(Pronostici!$R14="",Pronostici!$S14=""),"",Pronostici!$R14&amp;" a "&amp;Pronostici!$S14)</f>
         <v/>
       </c>
     </row>
@@ -8609,23 +8874,23 @@
         <v/>
       </c>
       <c r="D15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$F15&lt;&gt;"",Pronostici!$G15&lt;&gt;"",Pronostici!$F15=Partite!$G15,Pronostici!$G15=Partite!$H15),Config!$D$6,IF(AND($J15&lt;&gt;"",$J15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$F15&lt;&gt;"",Pronostici!$G15&lt;&gt;"",Pronostici!$F15=Partite!$G15,Pronostici!$G15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$P15)=1),Config!$D$9,Config!$D$6),IF(AND($J15&lt;&gt;"",$J15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$J15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$I15&lt;&gt;"",Pronostici!$J15&lt;&gt;"",Pronostici!$I15=Partite!$G15,Pronostici!$J15=Partite!$H15),Config!$D$6,IF(AND($K15&lt;&gt;"",$K15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$I15&lt;&gt;"",Pronostici!$J15&lt;&gt;"",Pronostici!$I15=Partite!$G15,Pronostici!$J15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$Q15)=1),Config!$D$9,Config!$D$6),IF(AND($K15&lt;&gt;"",$K15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$K15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$L15&lt;&gt;"",Pronostici!$M15&lt;&gt;"",Pronostici!$L15=Partite!$G15,Pronostici!$M15=Partite!$H15),Config!$D$6,IF(AND($L15&lt;&gt;"",$L15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$L15&lt;&gt;"",Pronostici!$M15&lt;&gt;"",Pronostici!$L15=Partite!$G15,Pronostici!$M15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$R15)=1),Config!$D$9,Config!$D$6),IF(AND($L15&lt;&gt;"",$L15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$L15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$O15&lt;&gt;"",Pronostici!$P15&lt;&gt;"",Pronostici!$O15=Partite!$G15,Pronostici!$P15=Partite!$H15),Config!$D$6,IF(AND($M15&lt;&gt;"",$M15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$O15&lt;&gt;"",Pronostici!$P15&lt;&gt;"",Pronostici!$O15=Partite!$G15,Pronostici!$P15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$S15)=1),Config!$D$9,Config!$D$6),IF(AND($M15&lt;&gt;"",$M15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$M15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H15" s="27">
-        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$R15&lt;&gt;"",Pronostici!$S15&lt;&gt;"",Pronostici!$R15=Partite!$G15,Pronostici!$S15=Partite!$H15),Config!$D$6,IF(AND($N15&lt;&gt;"",$N15=Partite!$I15),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K15&lt;&gt;"Giocata","",IF(AND(Pronostici!$R15&lt;&gt;"",Pronostici!$S15&lt;&gt;"",Pronostici!$R15=Partite!$G15,Pronostici!$S15=Partite!$H15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($P15:$T15,$T15)=1),Config!$D$9,Config!$D$6),IF(AND($N15&lt;&gt;"",$N15=Partite!$I15),IF(AND($B15&gt;=Config!$D$17,COUNTIF($J15:$N15,$N15)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J15" s="63">
@@ -8646,6 +8911,26 @@
       </c>
       <c r="N15" s="63">
         <f>IF(Pronostici!$Q15&lt;&gt;"",UPPER(Pronostici!$Q15),IF(OR(Pronostici!$R15="",Pronostici!$S15=""),"",IF(Pronostici!$R15&gt;Pronostici!$S15,"1",IF(Pronostici!$R15=Pronostici!$S15,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P15" s="63">
+        <f>IF(OR(Pronostici!$F15="",Pronostici!$G15=""),"",Pronostici!$F15&amp;" a "&amp;Pronostici!$G15)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="63">
+        <f>IF(OR(Pronostici!$I15="",Pronostici!$J15=""),"",Pronostici!$I15&amp;" a "&amp;Pronostici!$J15)</f>
+        <v/>
+      </c>
+      <c r="R15" s="63">
+        <f>IF(OR(Pronostici!$L15="",Pronostici!$M15=""),"",Pronostici!$L15&amp;" a "&amp;Pronostici!$M15)</f>
+        <v/>
+      </c>
+      <c r="S15" s="63">
+        <f>IF(OR(Pronostici!$O15="",Pronostici!$P15=""),"",Pronostici!$O15&amp;" a "&amp;Pronostici!$P15)</f>
+        <v/>
+      </c>
+      <c r="T15" s="63">
+        <f>IF(OR(Pronostici!$R15="",Pronostici!$S15=""),"",Pronostici!$R15&amp;" a "&amp;Pronostici!$S15)</f>
         <v/>
       </c>
     </row>
@@ -8663,23 +8948,23 @@
         <v/>
       </c>
       <c r="D16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$F16&lt;&gt;"",Pronostici!$G16&lt;&gt;"",Pronostici!$F16=Partite!$G16,Pronostici!$G16=Partite!$H16),Config!$D$6,IF(AND($J16&lt;&gt;"",$J16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$F16&lt;&gt;"",Pronostici!$G16&lt;&gt;"",Pronostici!$F16=Partite!$G16,Pronostici!$G16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$P16)=1),Config!$D$9,Config!$D$6),IF(AND($J16&lt;&gt;"",$J16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$J16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$I16&lt;&gt;"",Pronostici!$J16&lt;&gt;"",Pronostici!$I16=Partite!$G16,Pronostici!$J16=Partite!$H16),Config!$D$6,IF(AND($K16&lt;&gt;"",$K16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$I16&lt;&gt;"",Pronostici!$J16&lt;&gt;"",Pronostici!$I16=Partite!$G16,Pronostici!$J16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$Q16)=1),Config!$D$9,Config!$D$6),IF(AND($K16&lt;&gt;"",$K16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$K16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$L16&lt;&gt;"",Pronostici!$M16&lt;&gt;"",Pronostici!$L16=Partite!$G16,Pronostici!$M16=Partite!$H16),Config!$D$6,IF(AND($L16&lt;&gt;"",$L16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$L16&lt;&gt;"",Pronostici!$M16&lt;&gt;"",Pronostici!$L16=Partite!$G16,Pronostici!$M16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$R16)=1),Config!$D$9,Config!$D$6),IF(AND($L16&lt;&gt;"",$L16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$L16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$O16&lt;&gt;"",Pronostici!$P16&lt;&gt;"",Pronostici!$O16=Partite!$G16,Pronostici!$P16=Partite!$H16),Config!$D$6,IF(AND($M16&lt;&gt;"",$M16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$O16&lt;&gt;"",Pronostici!$P16&lt;&gt;"",Pronostici!$O16=Partite!$G16,Pronostici!$P16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$S16)=1),Config!$D$9,Config!$D$6),IF(AND($M16&lt;&gt;"",$M16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$M16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H16" s="27">
-        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$R16&lt;&gt;"",Pronostici!$S16&lt;&gt;"",Pronostici!$R16=Partite!$G16,Pronostici!$S16=Partite!$H16),Config!$D$6,IF(AND($N16&lt;&gt;"",$N16=Partite!$I16),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K16&lt;&gt;"Giocata","",IF(AND(Pronostici!$R16&lt;&gt;"",Pronostici!$S16&lt;&gt;"",Pronostici!$R16=Partite!$G16,Pronostici!$S16=Partite!$H16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($P16:$T16,$T16)=1),Config!$D$9,Config!$D$6),IF(AND($N16&lt;&gt;"",$N16=Partite!$I16),IF(AND($B16&gt;=Config!$D$17,COUNTIF($J16:$N16,$N16)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J16" s="63">
@@ -8700,6 +8985,26 @@
       </c>
       <c r="N16" s="63">
         <f>IF(Pronostici!$Q16&lt;&gt;"",UPPER(Pronostici!$Q16),IF(OR(Pronostici!$R16="",Pronostici!$S16=""),"",IF(Pronostici!$R16&gt;Pronostici!$S16,"1",IF(Pronostici!$R16=Pronostici!$S16,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P16" s="63">
+        <f>IF(OR(Pronostici!$F16="",Pronostici!$G16=""),"",Pronostici!$F16&amp;" a "&amp;Pronostici!$G16)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="63">
+        <f>IF(OR(Pronostici!$I16="",Pronostici!$J16=""),"",Pronostici!$I16&amp;" a "&amp;Pronostici!$J16)</f>
+        <v/>
+      </c>
+      <c r="R16" s="63">
+        <f>IF(OR(Pronostici!$L16="",Pronostici!$M16=""),"",Pronostici!$L16&amp;" a "&amp;Pronostici!$M16)</f>
+        <v/>
+      </c>
+      <c r="S16" s="63">
+        <f>IF(OR(Pronostici!$O16="",Pronostici!$P16=""),"",Pronostici!$O16&amp;" a "&amp;Pronostici!$P16)</f>
+        <v/>
+      </c>
+      <c r="T16" s="63">
+        <f>IF(OR(Pronostici!$R16="",Pronostici!$S16=""),"",Pronostici!$R16&amp;" a "&amp;Pronostici!$S16)</f>
         <v/>
       </c>
     </row>
@@ -8717,23 +9022,23 @@
         <v/>
       </c>
       <c r="D17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$F17&lt;&gt;"",Pronostici!$G17&lt;&gt;"",Pronostici!$F17=Partite!$G17,Pronostici!$G17=Partite!$H17),Config!$D$6,IF(AND($J17&lt;&gt;"",$J17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$F17&lt;&gt;"",Pronostici!$G17&lt;&gt;"",Pronostici!$F17=Partite!$G17,Pronostici!$G17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$P17)=1),Config!$D$9,Config!$D$6),IF(AND($J17&lt;&gt;"",$J17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$J17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$I17&lt;&gt;"",Pronostici!$J17&lt;&gt;"",Pronostici!$I17=Partite!$G17,Pronostici!$J17=Partite!$H17),Config!$D$6,IF(AND($K17&lt;&gt;"",$K17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$I17&lt;&gt;"",Pronostici!$J17&lt;&gt;"",Pronostici!$I17=Partite!$G17,Pronostici!$J17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$Q17)=1),Config!$D$9,Config!$D$6),IF(AND($K17&lt;&gt;"",$K17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$K17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$L17&lt;&gt;"",Pronostici!$M17&lt;&gt;"",Pronostici!$L17=Partite!$G17,Pronostici!$M17=Partite!$H17),Config!$D$6,IF(AND($L17&lt;&gt;"",$L17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$L17&lt;&gt;"",Pronostici!$M17&lt;&gt;"",Pronostici!$L17=Partite!$G17,Pronostici!$M17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$R17)=1),Config!$D$9,Config!$D$6),IF(AND($L17&lt;&gt;"",$L17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$L17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$O17&lt;&gt;"",Pronostici!$P17&lt;&gt;"",Pronostici!$O17=Partite!$G17,Pronostici!$P17=Partite!$H17),Config!$D$6,IF(AND($M17&lt;&gt;"",$M17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$O17&lt;&gt;"",Pronostici!$P17&lt;&gt;"",Pronostici!$O17=Partite!$G17,Pronostici!$P17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$S17)=1),Config!$D$9,Config!$D$6),IF(AND($M17&lt;&gt;"",$M17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$M17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H17" s="27">
-        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$R17&lt;&gt;"",Pronostici!$S17&lt;&gt;"",Pronostici!$R17=Partite!$G17,Pronostici!$S17=Partite!$H17),Config!$D$6,IF(AND($N17&lt;&gt;"",$N17=Partite!$I17),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K17&lt;&gt;"Giocata","",IF(AND(Pronostici!$R17&lt;&gt;"",Pronostici!$S17&lt;&gt;"",Pronostici!$R17=Partite!$G17,Pronostici!$S17=Partite!$H17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($P17:$T17,$T17)=1),Config!$D$9,Config!$D$6),IF(AND($N17&lt;&gt;"",$N17=Partite!$I17),IF(AND($B17&gt;=Config!$D$17,COUNTIF($J17:$N17,$N17)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J17" s="63">
@@ -8754,6 +9059,26 @@
       </c>
       <c r="N17" s="63">
         <f>IF(Pronostici!$Q17&lt;&gt;"",UPPER(Pronostici!$Q17),IF(OR(Pronostici!$R17="",Pronostici!$S17=""),"",IF(Pronostici!$R17&gt;Pronostici!$S17,"1",IF(Pronostici!$R17=Pronostici!$S17,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P17" s="63">
+        <f>IF(OR(Pronostici!$F17="",Pronostici!$G17=""),"",Pronostici!$F17&amp;" a "&amp;Pronostici!$G17)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="63">
+        <f>IF(OR(Pronostici!$I17="",Pronostici!$J17=""),"",Pronostici!$I17&amp;" a "&amp;Pronostici!$J17)</f>
+        <v/>
+      </c>
+      <c r="R17" s="63">
+        <f>IF(OR(Pronostici!$L17="",Pronostici!$M17=""),"",Pronostici!$L17&amp;" a "&amp;Pronostici!$M17)</f>
+        <v/>
+      </c>
+      <c r="S17" s="63">
+        <f>IF(OR(Pronostici!$O17="",Pronostici!$P17=""),"",Pronostici!$O17&amp;" a "&amp;Pronostici!$P17)</f>
+        <v/>
+      </c>
+      <c r="T17" s="63">
+        <f>IF(OR(Pronostici!$R17="",Pronostici!$S17=""),"",Pronostici!$R17&amp;" a "&amp;Pronostici!$S17)</f>
         <v/>
       </c>
     </row>
@@ -8771,23 +9096,23 @@
         <v/>
       </c>
       <c r="D18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$F18&lt;&gt;"",Pronostici!$G18&lt;&gt;"",Pronostici!$F18=Partite!$G18,Pronostici!$G18=Partite!$H18),Config!$D$6,IF(AND($J18&lt;&gt;"",$J18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$F18&lt;&gt;"",Pronostici!$G18&lt;&gt;"",Pronostici!$F18=Partite!$G18,Pronostici!$G18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$P18)=1),Config!$D$9,Config!$D$6),IF(AND($J18&lt;&gt;"",$J18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$J18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$I18&lt;&gt;"",Pronostici!$J18&lt;&gt;"",Pronostici!$I18=Partite!$G18,Pronostici!$J18=Partite!$H18),Config!$D$6,IF(AND($K18&lt;&gt;"",$K18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$I18&lt;&gt;"",Pronostici!$J18&lt;&gt;"",Pronostici!$I18=Partite!$G18,Pronostici!$J18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$Q18)=1),Config!$D$9,Config!$D$6),IF(AND($K18&lt;&gt;"",$K18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$K18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$L18&lt;&gt;"",Pronostici!$M18&lt;&gt;"",Pronostici!$L18=Partite!$G18,Pronostici!$M18=Partite!$H18),Config!$D$6,IF(AND($L18&lt;&gt;"",$L18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$L18&lt;&gt;"",Pronostici!$M18&lt;&gt;"",Pronostici!$L18=Partite!$G18,Pronostici!$M18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$R18)=1),Config!$D$9,Config!$D$6),IF(AND($L18&lt;&gt;"",$L18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$L18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$O18&lt;&gt;"",Pronostici!$P18&lt;&gt;"",Pronostici!$O18=Partite!$G18,Pronostici!$P18=Partite!$H18),Config!$D$6,IF(AND($M18&lt;&gt;"",$M18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$O18&lt;&gt;"",Pronostici!$P18&lt;&gt;"",Pronostici!$O18=Partite!$G18,Pronostici!$P18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$S18)=1),Config!$D$9,Config!$D$6),IF(AND($M18&lt;&gt;"",$M18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$M18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H18" s="27">
-        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$R18&lt;&gt;"",Pronostici!$S18&lt;&gt;"",Pronostici!$R18=Partite!$G18,Pronostici!$S18=Partite!$H18),Config!$D$6,IF(AND($N18&lt;&gt;"",$N18=Partite!$I18),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K18&lt;&gt;"Giocata","",IF(AND(Pronostici!$R18&lt;&gt;"",Pronostici!$S18&lt;&gt;"",Pronostici!$R18=Partite!$G18,Pronostici!$S18=Partite!$H18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($P18:$T18,$T18)=1),Config!$D$9,Config!$D$6),IF(AND($N18&lt;&gt;"",$N18=Partite!$I18),IF(AND($B18&gt;=Config!$D$17,COUNTIF($J18:$N18,$N18)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J18" s="63">
@@ -8808,6 +9133,26 @@
       </c>
       <c r="N18" s="63">
         <f>IF(Pronostici!$Q18&lt;&gt;"",UPPER(Pronostici!$Q18),IF(OR(Pronostici!$R18="",Pronostici!$S18=""),"",IF(Pronostici!$R18&gt;Pronostici!$S18,"1",IF(Pronostici!$R18=Pronostici!$S18,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P18" s="63">
+        <f>IF(OR(Pronostici!$F18="",Pronostici!$G18=""),"",Pronostici!$F18&amp;" a "&amp;Pronostici!$G18)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="63">
+        <f>IF(OR(Pronostici!$I18="",Pronostici!$J18=""),"",Pronostici!$I18&amp;" a "&amp;Pronostici!$J18)</f>
+        <v/>
+      </c>
+      <c r="R18" s="63">
+        <f>IF(OR(Pronostici!$L18="",Pronostici!$M18=""),"",Pronostici!$L18&amp;" a "&amp;Pronostici!$M18)</f>
+        <v/>
+      </c>
+      <c r="S18" s="63">
+        <f>IF(OR(Pronostici!$O18="",Pronostici!$P18=""),"",Pronostici!$O18&amp;" a "&amp;Pronostici!$P18)</f>
+        <v/>
+      </c>
+      <c r="T18" s="63">
+        <f>IF(OR(Pronostici!$R18="",Pronostici!$S18=""),"",Pronostici!$R18&amp;" a "&amp;Pronostici!$S18)</f>
         <v/>
       </c>
     </row>
@@ -8825,23 +9170,23 @@
         <v/>
       </c>
       <c r="D19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$F19&lt;&gt;"",Pronostici!$G19&lt;&gt;"",Pronostici!$F19=Partite!$G19,Pronostici!$G19=Partite!$H19),Config!$D$6,IF(AND($J19&lt;&gt;"",$J19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$F19&lt;&gt;"",Pronostici!$G19&lt;&gt;"",Pronostici!$F19=Partite!$G19,Pronostici!$G19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$P19)=1),Config!$D$9,Config!$D$6),IF(AND($J19&lt;&gt;"",$J19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$J19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$I19&lt;&gt;"",Pronostici!$J19&lt;&gt;"",Pronostici!$I19=Partite!$G19,Pronostici!$J19=Partite!$H19),Config!$D$6,IF(AND($K19&lt;&gt;"",$K19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$I19&lt;&gt;"",Pronostici!$J19&lt;&gt;"",Pronostici!$I19=Partite!$G19,Pronostici!$J19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$Q19)=1),Config!$D$9,Config!$D$6),IF(AND($K19&lt;&gt;"",$K19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$K19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$L19&lt;&gt;"",Pronostici!$M19&lt;&gt;"",Pronostici!$L19=Partite!$G19,Pronostici!$M19=Partite!$H19),Config!$D$6,IF(AND($L19&lt;&gt;"",$L19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$L19&lt;&gt;"",Pronostici!$M19&lt;&gt;"",Pronostici!$L19=Partite!$G19,Pronostici!$M19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$R19)=1),Config!$D$9,Config!$D$6),IF(AND($L19&lt;&gt;"",$L19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$L19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$O19&lt;&gt;"",Pronostici!$P19&lt;&gt;"",Pronostici!$O19=Partite!$G19,Pronostici!$P19=Partite!$H19),Config!$D$6,IF(AND($M19&lt;&gt;"",$M19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$O19&lt;&gt;"",Pronostici!$P19&lt;&gt;"",Pronostici!$O19=Partite!$G19,Pronostici!$P19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$S19)=1),Config!$D$9,Config!$D$6),IF(AND($M19&lt;&gt;"",$M19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$M19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H19" s="27">
-        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$R19&lt;&gt;"",Pronostici!$S19&lt;&gt;"",Pronostici!$R19=Partite!$G19,Pronostici!$S19=Partite!$H19),Config!$D$6,IF(AND($N19&lt;&gt;"",$N19=Partite!$I19),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K19&lt;&gt;"Giocata","",IF(AND(Pronostici!$R19&lt;&gt;"",Pronostici!$S19&lt;&gt;"",Pronostici!$R19=Partite!$G19,Pronostici!$S19=Partite!$H19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($P19:$T19,$T19)=1),Config!$D$9,Config!$D$6),IF(AND($N19&lt;&gt;"",$N19=Partite!$I19),IF(AND($B19&gt;=Config!$D$17,COUNTIF($J19:$N19,$N19)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J19" s="63">
@@ -8862,6 +9207,26 @@
       </c>
       <c r="N19" s="63">
         <f>IF(Pronostici!$Q19&lt;&gt;"",UPPER(Pronostici!$Q19),IF(OR(Pronostici!$R19="",Pronostici!$S19=""),"",IF(Pronostici!$R19&gt;Pronostici!$S19,"1",IF(Pronostici!$R19=Pronostici!$S19,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P19" s="63">
+        <f>IF(OR(Pronostici!$F19="",Pronostici!$G19=""),"",Pronostici!$F19&amp;" a "&amp;Pronostici!$G19)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="63">
+        <f>IF(OR(Pronostici!$I19="",Pronostici!$J19=""),"",Pronostici!$I19&amp;" a "&amp;Pronostici!$J19)</f>
+        <v/>
+      </c>
+      <c r="R19" s="63">
+        <f>IF(OR(Pronostici!$L19="",Pronostici!$M19=""),"",Pronostici!$L19&amp;" a "&amp;Pronostici!$M19)</f>
+        <v/>
+      </c>
+      <c r="S19" s="63">
+        <f>IF(OR(Pronostici!$O19="",Pronostici!$P19=""),"",Pronostici!$O19&amp;" a "&amp;Pronostici!$P19)</f>
+        <v/>
+      </c>
+      <c r="T19" s="63">
+        <f>IF(OR(Pronostici!$R19="",Pronostici!$S19=""),"",Pronostici!$R19&amp;" a "&amp;Pronostici!$S19)</f>
         <v/>
       </c>
     </row>
@@ -8879,23 +9244,23 @@
         <v/>
       </c>
       <c r="D20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$F20&lt;&gt;"",Pronostici!$G20&lt;&gt;"",Pronostici!$F20=Partite!$G20,Pronostici!$G20=Partite!$H20),Config!$D$6,IF(AND($J20&lt;&gt;"",$J20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$F20&lt;&gt;"",Pronostici!$G20&lt;&gt;"",Pronostici!$F20=Partite!$G20,Pronostici!$G20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$P20)=1),Config!$D$9,Config!$D$6),IF(AND($J20&lt;&gt;"",$J20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$J20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$I20&lt;&gt;"",Pronostici!$J20&lt;&gt;"",Pronostici!$I20=Partite!$G20,Pronostici!$J20=Partite!$H20),Config!$D$6,IF(AND($K20&lt;&gt;"",$K20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$I20&lt;&gt;"",Pronostici!$J20&lt;&gt;"",Pronostici!$I20=Partite!$G20,Pronostici!$J20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$Q20)=1),Config!$D$9,Config!$D$6),IF(AND($K20&lt;&gt;"",$K20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$K20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$L20&lt;&gt;"",Pronostici!$M20&lt;&gt;"",Pronostici!$L20=Partite!$G20,Pronostici!$M20=Partite!$H20),Config!$D$6,IF(AND($L20&lt;&gt;"",$L20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$L20&lt;&gt;"",Pronostici!$M20&lt;&gt;"",Pronostici!$L20=Partite!$G20,Pronostici!$M20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$R20)=1),Config!$D$9,Config!$D$6),IF(AND($L20&lt;&gt;"",$L20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$L20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$O20&lt;&gt;"",Pronostici!$P20&lt;&gt;"",Pronostici!$O20=Partite!$G20,Pronostici!$P20=Partite!$H20),Config!$D$6,IF(AND($M20&lt;&gt;"",$M20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$O20&lt;&gt;"",Pronostici!$P20&lt;&gt;"",Pronostici!$O20=Partite!$G20,Pronostici!$P20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$S20)=1),Config!$D$9,Config!$D$6),IF(AND($M20&lt;&gt;"",$M20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$M20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H20" s="27">
-        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$R20&lt;&gt;"",Pronostici!$S20&lt;&gt;"",Pronostici!$R20=Partite!$G20,Pronostici!$S20=Partite!$H20),Config!$D$6,IF(AND($N20&lt;&gt;"",$N20=Partite!$I20),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K20&lt;&gt;"Giocata","",IF(AND(Pronostici!$R20&lt;&gt;"",Pronostici!$S20&lt;&gt;"",Pronostici!$R20=Partite!$G20,Pronostici!$S20=Partite!$H20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($P20:$T20,$T20)=1),Config!$D$9,Config!$D$6),IF(AND($N20&lt;&gt;"",$N20=Partite!$I20),IF(AND($B20&gt;=Config!$D$17,COUNTIF($J20:$N20,$N20)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J20" s="63">
@@ -8916,6 +9281,26 @@
       </c>
       <c r="N20" s="63">
         <f>IF(Pronostici!$Q20&lt;&gt;"",UPPER(Pronostici!$Q20),IF(OR(Pronostici!$R20="",Pronostici!$S20=""),"",IF(Pronostici!$R20&gt;Pronostici!$S20,"1",IF(Pronostici!$R20=Pronostici!$S20,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P20" s="63">
+        <f>IF(OR(Pronostici!$F20="",Pronostici!$G20=""),"",Pronostici!$F20&amp;" a "&amp;Pronostici!$G20)</f>
+        <v/>
+      </c>
+      <c r="Q20" s="63">
+        <f>IF(OR(Pronostici!$I20="",Pronostici!$J20=""),"",Pronostici!$I20&amp;" a "&amp;Pronostici!$J20)</f>
+        <v/>
+      </c>
+      <c r="R20" s="63">
+        <f>IF(OR(Pronostici!$L20="",Pronostici!$M20=""),"",Pronostici!$L20&amp;" a "&amp;Pronostici!$M20)</f>
+        <v/>
+      </c>
+      <c r="S20" s="63">
+        <f>IF(OR(Pronostici!$O20="",Pronostici!$P20=""),"",Pronostici!$O20&amp;" a "&amp;Pronostici!$P20)</f>
+        <v/>
+      </c>
+      <c r="T20" s="63">
+        <f>IF(OR(Pronostici!$R20="",Pronostici!$S20=""),"",Pronostici!$R20&amp;" a "&amp;Pronostici!$S20)</f>
         <v/>
       </c>
     </row>
@@ -8933,23 +9318,23 @@
         <v/>
       </c>
       <c r="D21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$F21&lt;&gt;"",Pronostici!$G21&lt;&gt;"",Pronostici!$F21=Partite!$G21,Pronostici!$G21=Partite!$H21),Config!$D$6,IF(AND($J21&lt;&gt;"",$J21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$F21&lt;&gt;"",Pronostici!$G21&lt;&gt;"",Pronostici!$F21=Partite!$G21,Pronostici!$G21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$P21)=1),Config!$D$9,Config!$D$6),IF(AND($J21&lt;&gt;"",$J21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$J21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$I21&lt;&gt;"",Pronostici!$J21&lt;&gt;"",Pronostici!$I21=Partite!$G21,Pronostici!$J21=Partite!$H21),Config!$D$6,IF(AND($K21&lt;&gt;"",$K21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$I21&lt;&gt;"",Pronostici!$J21&lt;&gt;"",Pronostici!$I21=Partite!$G21,Pronostici!$J21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$Q21)=1),Config!$D$9,Config!$D$6),IF(AND($K21&lt;&gt;"",$K21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$K21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$L21&lt;&gt;"",Pronostici!$M21&lt;&gt;"",Pronostici!$L21=Partite!$G21,Pronostici!$M21=Partite!$H21),Config!$D$6,IF(AND($L21&lt;&gt;"",$L21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$L21&lt;&gt;"",Pronostici!$M21&lt;&gt;"",Pronostici!$L21=Partite!$G21,Pronostici!$M21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$R21)=1),Config!$D$9,Config!$D$6),IF(AND($L21&lt;&gt;"",$L21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$L21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$O21&lt;&gt;"",Pronostici!$P21&lt;&gt;"",Pronostici!$O21=Partite!$G21,Pronostici!$P21=Partite!$H21),Config!$D$6,IF(AND($M21&lt;&gt;"",$M21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$O21&lt;&gt;"",Pronostici!$P21&lt;&gt;"",Pronostici!$O21=Partite!$G21,Pronostici!$P21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$S21)=1),Config!$D$9,Config!$D$6),IF(AND($M21&lt;&gt;"",$M21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$M21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H21" s="27">
-        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$R21&lt;&gt;"",Pronostici!$S21&lt;&gt;"",Pronostici!$R21=Partite!$G21,Pronostici!$S21=Partite!$H21),Config!$D$6,IF(AND($N21&lt;&gt;"",$N21=Partite!$I21),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K21&lt;&gt;"Giocata","",IF(AND(Pronostici!$R21&lt;&gt;"",Pronostici!$S21&lt;&gt;"",Pronostici!$R21=Partite!$G21,Pronostici!$S21=Partite!$H21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($P21:$T21,$T21)=1),Config!$D$9,Config!$D$6),IF(AND($N21&lt;&gt;"",$N21=Partite!$I21),IF(AND($B21&gt;=Config!$D$17,COUNTIF($J21:$N21,$N21)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J21" s="63">
@@ -8970,6 +9355,26 @@
       </c>
       <c r="N21" s="63">
         <f>IF(Pronostici!$Q21&lt;&gt;"",UPPER(Pronostici!$Q21),IF(OR(Pronostici!$R21="",Pronostici!$S21=""),"",IF(Pronostici!$R21&gt;Pronostici!$S21,"1",IF(Pronostici!$R21=Pronostici!$S21,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P21" s="63">
+        <f>IF(OR(Pronostici!$F21="",Pronostici!$G21=""),"",Pronostici!$F21&amp;" a "&amp;Pronostici!$G21)</f>
+        <v/>
+      </c>
+      <c r="Q21" s="63">
+        <f>IF(OR(Pronostici!$I21="",Pronostici!$J21=""),"",Pronostici!$I21&amp;" a "&amp;Pronostici!$J21)</f>
+        <v/>
+      </c>
+      <c r="R21" s="63">
+        <f>IF(OR(Pronostici!$L21="",Pronostici!$M21=""),"",Pronostici!$L21&amp;" a "&amp;Pronostici!$M21)</f>
+        <v/>
+      </c>
+      <c r="S21" s="63">
+        <f>IF(OR(Pronostici!$O21="",Pronostici!$P21=""),"",Pronostici!$O21&amp;" a "&amp;Pronostici!$P21)</f>
+        <v/>
+      </c>
+      <c r="T21" s="63">
+        <f>IF(OR(Pronostici!$R21="",Pronostici!$S21=""),"",Pronostici!$R21&amp;" a "&amp;Pronostici!$S21)</f>
         <v/>
       </c>
     </row>
@@ -8987,23 +9392,23 @@
         <v/>
       </c>
       <c r="D22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$F22&lt;&gt;"",Pronostici!$G22&lt;&gt;"",Pronostici!$F22=Partite!$G22,Pronostici!$G22=Partite!$H22),Config!$D$6,IF(AND($J22&lt;&gt;"",$J22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$F22&lt;&gt;"",Pronostici!$G22&lt;&gt;"",Pronostici!$F22=Partite!$G22,Pronostici!$G22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$P22)=1),Config!$D$9,Config!$D$6),IF(AND($J22&lt;&gt;"",$J22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$J22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$I22&lt;&gt;"",Pronostici!$J22&lt;&gt;"",Pronostici!$I22=Partite!$G22,Pronostici!$J22=Partite!$H22),Config!$D$6,IF(AND($K22&lt;&gt;"",$K22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$I22&lt;&gt;"",Pronostici!$J22&lt;&gt;"",Pronostici!$I22=Partite!$G22,Pronostici!$J22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$Q22)=1),Config!$D$9,Config!$D$6),IF(AND($K22&lt;&gt;"",$K22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$K22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$L22&lt;&gt;"",Pronostici!$M22&lt;&gt;"",Pronostici!$L22=Partite!$G22,Pronostici!$M22=Partite!$H22),Config!$D$6,IF(AND($L22&lt;&gt;"",$L22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$L22&lt;&gt;"",Pronostici!$M22&lt;&gt;"",Pronostici!$L22=Partite!$G22,Pronostici!$M22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$R22)=1),Config!$D$9,Config!$D$6),IF(AND($L22&lt;&gt;"",$L22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$L22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$O22&lt;&gt;"",Pronostici!$P22&lt;&gt;"",Pronostici!$O22=Partite!$G22,Pronostici!$P22=Partite!$H22),Config!$D$6,IF(AND($M22&lt;&gt;"",$M22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$O22&lt;&gt;"",Pronostici!$P22&lt;&gt;"",Pronostici!$O22=Partite!$G22,Pronostici!$P22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$S22)=1),Config!$D$9,Config!$D$6),IF(AND($M22&lt;&gt;"",$M22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$M22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H22" s="27">
-        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$R22&lt;&gt;"",Pronostici!$S22&lt;&gt;"",Pronostici!$R22=Partite!$G22,Pronostici!$S22=Partite!$H22),Config!$D$6,IF(AND($N22&lt;&gt;"",$N22=Partite!$I22),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K22&lt;&gt;"Giocata","",IF(AND(Pronostici!$R22&lt;&gt;"",Pronostici!$S22&lt;&gt;"",Pronostici!$R22=Partite!$G22,Pronostici!$S22=Partite!$H22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($P22:$T22,$T22)=1),Config!$D$9,Config!$D$6),IF(AND($N22&lt;&gt;"",$N22=Partite!$I22),IF(AND($B22&gt;=Config!$D$17,COUNTIF($J22:$N22,$N22)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J22" s="63">
@@ -9024,6 +9429,26 @@
       </c>
       <c r="N22" s="63">
         <f>IF(Pronostici!$Q22&lt;&gt;"",UPPER(Pronostici!$Q22),IF(OR(Pronostici!$R22="",Pronostici!$S22=""),"",IF(Pronostici!$R22&gt;Pronostici!$S22,"1",IF(Pronostici!$R22=Pronostici!$S22,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P22" s="63">
+        <f>IF(OR(Pronostici!$F22="",Pronostici!$G22=""),"",Pronostici!$F22&amp;" a "&amp;Pronostici!$G22)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="63">
+        <f>IF(OR(Pronostici!$I22="",Pronostici!$J22=""),"",Pronostici!$I22&amp;" a "&amp;Pronostici!$J22)</f>
+        <v/>
+      </c>
+      <c r="R22" s="63">
+        <f>IF(OR(Pronostici!$L22="",Pronostici!$M22=""),"",Pronostici!$L22&amp;" a "&amp;Pronostici!$M22)</f>
+        <v/>
+      </c>
+      <c r="S22" s="63">
+        <f>IF(OR(Pronostici!$O22="",Pronostici!$P22=""),"",Pronostici!$O22&amp;" a "&amp;Pronostici!$P22)</f>
+        <v/>
+      </c>
+      <c r="T22" s="63">
+        <f>IF(OR(Pronostici!$R22="",Pronostici!$S22=""),"",Pronostici!$R22&amp;" a "&amp;Pronostici!$S22)</f>
         <v/>
       </c>
     </row>
@@ -9041,23 +9466,23 @@
         <v/>
       </c>
       <c r="D23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$F23&lt;&gt;"",Pronostici!$G23&lt;&gt;"",Pronostici!$F23=Partite!$G23,Pronostici!$G23=Partite!$H23),Config!$D$6,IF(AND($J23&lt;&gt;"",$J23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$F23&lt;&gt;"",Pronostici!$G23&lt;&gt;"",Pronostici!$F23=Partite!$G23,Pronostici!$G23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$P23)=1),Config!$D$9,Config!$D$6),IF(AND($J23&lt;&gt;"",$J23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$J23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$I23&lt;&gt;"",Pronostici!$J23&lt;&gt;"",Pronostici!$I23=Partite!$G23,Pronostici!$J23=Partite!$H23),Config!$D$6,IF(AND($K23&lt;&gt;"",$K23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$I23&lt;&gt;"",Pronostici!$J23&lt;&gt;"",Pronostici!$I23=Partite!$G23,Pronostici!$J23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$Q23)=1),Config!$D$9,Config!$D$6),IF(AND($K23&lt;&gt;"",$K23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$K23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$L23&lt;&gt;"",Pronostici!$M23&lt;&gt;"",Pronostici!$L23=Partite!$G23,Pronostici!$M23=Partite!$H23),Config!$D$6,IF(AND($L23&lt;&gt;"",$L23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$L23&lt;&gt;"",Pronostici!$M23&lt;&gt;"",Pronostici!$L23=Partite!$G23,Pronostici!$M23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$R23)=1),Config!$D$9,Config!$D$6),IF(AND($L23&lt;&gt;"",$L23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$L23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$O23&lt;&gt;"",Pronostici!$P23&lt;&gt;"",Pronostici!$O23=Partite!$G23,Pronostici!$P23=Partite!$H23),Config!$D$6,IF(AND($M23&lt;&gt;"",$M23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$O23&lt;&gt;"",Pronostici!$P23&lt;&gt;"",Pronostici!$O23=Partite!$G23,Pronostici!$P23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$S23)=1),Config!$D$9,Config!$D$6),IF(AND($M23&lt;&gt;"",$M23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$M23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H23" s="22">
-        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$R23&lt;&gt;"",Pronostici!$S23&lt;&gt;"",Pronostici!$R23=Partite!$G23,Pronostici!$S23=Partite!$H23),Config!$D$6,IF(AND($N23&lt;&gt;"",$N23=Partite!$I23),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K23&lt;&gt;"Giocata","",IF(AND(Pronostici!$R23&lt;&gt;"",Pronostici!$S23&lt;&gt;"",Pronostici!$R23=Partite!$G23,Pronostici!$S23=Partite!$H23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($P23:$T23,$T23)=1),Config!$D$9,Config!$D$6),IF(AND($N23&lt;&gt;"",$N23=Partite!$I23),IF(AND($B23&gt;=Config!$D$17,COUNTIF($J23:$N23,$N23)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J23" s="63">
@@ -9078,6 +9503,26 @@
       </c>
       <c r="N23" s="63">
         <f>IF(Pronostici!$Q23&lt;&gt;"",UPPER(Pronostici!$Q23),IF(OR(Pronostici!$R23="",Pronostici!$S23=""),"",IF(Pronostici!$R23&gt;Pronostici!$S23,"1",IF(Pronostici!$R23=Pronostici!$S23,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P23" s="63">
+        <f>IF(OR(Pronostici!$F23="",Pronostici!$G23=""),"",Pronostici!$F23&amp;" a "&amp;Pronostici!$G23)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="63">
+        <f>IF(OR(Pronostici!$I23="",Pronostici!$J23=""),"",Pronostici!$I23&amp;" a "&amp;Pronostici!$J23)</f>
+        <v/>
+      </c>
+      <c r="R23" s="63">
+        <f>IF(OR(Pronostici!$L23="",Pronostici!$M23=""),"",Pronostici!$L23&amp;" a "&amp;Pronostici!$M23)</f>
+        <v/>
+      </c>
+      <c r="S23" s="63">
+        <f>IF(OR(Pronostici!$O23="",Pronostici!$P23=""),"",Pronostici!$O23&amp;" a "&amp;Pronostici!$P23)</f>
+        <v/>
+      </c>
+      <c r="T23" s="63">
+        <f>IF(OR(Pronostici!$R23="",Pronostici!$S23=""),"",Pronostici!$R23&amp;" a "&amp;Pronostici!$S23)</f>
         <v/>
       </c>
     </row>
@@ -9095,23 +9540,23 @@
         <v/>
       </c>
       <c r="D24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$F24&lt;&gt;"",Pronostici!$G24&lt;&gt;"",Pronostici!$F24=Partite!$G24,Pronostici!$G24=Partite!$H24),Config!$D$6,IF(AND($J24&lt;&gt;"",$J24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$F24&lt;&gt;"",Pronostici!$G24&lt;&gt;"",Pronostici!$F24=Partite!$G24,Pronostici!$G24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$P24)=1),Config!$D$9,Config!$D$6),IF(AND($J24&lt;&gt;"",$J24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$J24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$I24&lt;&gt;"",Pronostici!$J24&lt;&gt;"",Pronostici!$I24=Partite!$G24,Pronostici!$J24=Partite!$H24),Config!$D$6,IF(AND($K24&lt;&gt;"",$K24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$I24&lt;&gt;"",Pronostici!$J24&lt;&gt;"",Pronostici!$I24=Partite!$G24,Pronostici!$J24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$Q24)=1),Config!$D$9,Config!$D$6),IF(AND($K24&lt;&gt;"",$K24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$K24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$L24&lt;&gt;"",Pronostici!$M24&lt;&gt;"",Pronostici!$L24=Partite!$G24,Pronostici!$M24=Partite!$H24),Config!$D$6,IF(AND($L24&lt;&gt;"",$L24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$L24&lt;&gt;"",Pronostici!$M24&lt;&gt;"",Pronostici!$L24=Partite!$G24,Pronostici!$M24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$R24)=1),Config!$D$9,Config!$D$6),IF(AND($L24&lt;&gt;"",$L24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$L24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$O24&lt;&gt;"",Pronostici!$P24&lt;&gt;"",Pronostici!$O24=Partite!$G24,Pronostici!$P24=Partite!$H24),Config!$D$6,IF(AND($M24&lt;&gt;"",$M24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$O24&lt;&gt;"",Pronostici!$P24&lt;&gt;"",Pronostici!$O24=Partite!$G24,Pronostici!$P24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$S24)=1),Config!$D$9,Config!$D$6),IF(AND($M24&lt;&gt;"",$M24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$M24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$R24&lt;&gt;"",Pronostici!$S24&lt;&gt;"",Pronostici!$R24=Partite!$G24,Pronostici!$S24=Partite!$H24),Config!$D$6,IF(AND($N24&lt;&gt;"",$N24=Partite!$I24),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K24&lt;&gt;"Giocata","",IF(AND(Pronostici!$R24&lt;&gt;"",Pronostici!$S24&lt;&gt;"",Pronostici!$R24=Partite!$G24,Pronostici!$S24=Partite!$H24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($P24:$T24,$T24)=1),Config!$D$9,Config!$D$6),IF(AND($N24&lt;&gt;"",$N24=Partite!$I24),IF(AND($B24&gt;=Config!$D$17,COUNTIF($J24:$N24,$N24)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J24" s="63">
@@ -9132,6 +9577,26 @@
       </c>
       <c r="N24" s="63">
         <f>IF(Pronostici!$Q24&lt;&gt;"",UPPER(Pronostici!$Q24),IF(OR(Pronostici!$R24="",Pronostici!$S24=""),"",IF(Pronostici!$R24&gt;Pronostici!$S24,"1",IF(Pronostici!$R24=Pronostici!$S24,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P24" s="63">
+        <f>IF(OR(Pronostici!$F24="",Pronostici!$G24=""),"",Pronostici!$F24&amp;" a "&amp;Pronostici!$G24)</f>
+        <v/>
+      </c>
+      <c r="Q24" s="63">
+        <f>IF(OR(Pronostici!$I24="",Pronostici!$J24=""),"",Pronostici!$I24&amp;" a "&amp;Pronostici!$J24)</f>
+        <v/>
+      </c>
+      <c r="R24" s="63">
+        <f>IF(OR(Pronostici!$L24="",Pronostici!$M24=""),"",Pronostici!$L24&amp;" a "&amp;Pronostici!$M24)</f>
+        <v/>
+      </c>
+      <c r="S24" s="63">
+        <f>IF(OR(Pronostici!$O24="",Pronostici!$P24=""),"",Pronostici!$O24&amp;" a "&amp;Pronostici!$P24)</f>
+        <v/>
+      </c>
+      <c r="T24" s="63">
+        <f>IF(OR(Pronostici!$R24="",Pronostici!$S24=""),"",Pronostici!$R24&amp;" a "&amp;Pronostici!$S24)</f>
         <v/>
       </c>
     </row>
@@ -9149,23 +9614,23 @@
         <v/>
       </c>
       <c r="D25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$F25&lt;&gt;"",Pronostici!$G25&lt;&gt;"",Pronostici!$F25=Partite!$G25,Pronostici!$G25=Partite!$H25),Config!$D$6,IF(AND($J25&lt;&gt;"",$J25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$F25&lt;&gt;"",Pronostici!$G25&lt;&gt;"",Pronostici!$F25=Partite!$G25,Pronostici!$G25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$P25)=1),Config!$D$9,Config!$D$6),IF(AND($J25&lt;&gt;"",$J25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$J25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$I25&lt;&gt;"",Pronostici!$J25&lt;&gt;"",Pronostici!$I25=Partite!$G25,Pronostici!$J25=Partite!$H25),Config!$D$6,IF(AND($K25&lt;&gt;"",$K25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$I25&lt;&gt;"",Pronostici!$J25&lt;&gt;"",Pronostici!$I25=Partite!$G25,Pronostici!$J25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$Q25)=1),Config!$D$9,Config!$D$6),IF(AND($K25&lt;&gt;"",$K25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$K25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$L25&lt;&gt;"",Pronostici!$M25&lt;&gt;"",Pronostici!$L25=Partite!$G25,Pronostici!$M25=Partite!$H25),Config!$D$6,IF(AND($L25&lt;&gt;"",$L25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$L25&lt;&gt;"",Pronostici!$M25&lt;&gt;"",Pronostici!$L25=Partite!$G25,Pronostici!$M25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$R25)=1),Config!$D$9,Config!$D$6),IF(AND($L25&lt;&gt;"",$L25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$L25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$O25&lt;&gt;"",Pronostici!$P25&lt;&gt;"",Pronostici!$O25=Partite!$G25,Pronostici!$P25=Partite!$H25),Config!$D$6,IF(AND($M25&lt;&gt;"",$M25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$O25&lt;&gt;"",Pronostici!$P25&lt;&gt;"",Pronostici!$O25=Partite!$G25,Pronostici!$P25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$S25)=1),Config!$D$9,Config!$D$6),IF(AND($M25&lt;&gt;"",$M25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$M25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H25" s="22">
-        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$R25&lt;&gt;"",Pronostici!$S25&lt;&gt;"",Pronostici!$R25=Partite!$G25,Pronostici!$S25=Partite!$H25),Config!$D$6,IF(AND($N25&lt;&gt;"",$N25=Partite!$I25),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K25&lt;&gt;"Giocata","",IF(AND(Pronostici!$R25&lt;&gt;"",Pronostici!$S25&lt;&gt;"",Pronostici!$R25=Partite!$G25,Pronostici!$S25=Partite!$H25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($P25:$T25,$T25)=1),Config!$D$9,Config!$D$6),IF(AND($N25&lt;&gt;"",$N25=Partite!$I25),IF(AND($B25&gt;=Config!$D$17,COUNTIF($J25:$N25,$N25)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J25" s="63">
@@ -9186,6 +9651,26 @@
       </c>
       <c r="N25" s="63">
         <f>IF(Pronostici!$Q25&lt;&gt;"",UPPER(Pronostici!$Q25),IF(OR(Pronostici!$R25="",Pronostici!$S25=""),"",IF(Pronostici!$R25&gt;Pronostici!$S25,"1",IF(Pronostici!$R25=Pronostici!$S25,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P25" s="63">
+        <f>IF(OR(Pronostici!$F25="",Pronostici!$G25=""),"",Pronostici!$F25&amp;" a "&amp;Pronostici!$G25)</f>
+        <v/>
+      </c>
+      <c r="Q25" s="63">
+        <f>IF(OR(Pronostici!$I25="",Pronostici!$J25=""),"",Pronostici!$I25&amp;" a "&amp;Pronostici!$J25)</f>
+        <v/>
+      </c>
+      <c r="R25" s="63">
+        <f>IF(OR(Pronostici!$L25="",Pronostici!$M25=""),"",Pronostici!$L25&amp;" a "&amp;Pronostici!$M25)</f>
+        <v/>
+      </c>
+      <c r="S25" s="63">
+        <f>IF(OR(Pronostici!$O25="",Pronostici!$P25=""),"",Pronostici!$O25&amp;" a "&amp;Pronostici!$P25)</f>
+        <v/>
+      </c>
+      <c r="T25" s="63">
+        <f>IF(OR(Pronostici!$R25="",Pronostici!$S25=""),"",Pronostici!$R25&amp;" a "&amp;Pronostici!$S25)</f>
         <v/>
       </c>
     </row>
@@ -9203,23 +9688,23 @@
         <v/>
       </c>
       <c r="D26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$F26&lt;&gt;"",Pronostici!$G26&lt;&gt;"",Pronostici!$F26=Partite!$G26,Pronostici!$G26=Partite!$H26),Config!$D$6,IF(AND($J26&lt;&gt;"",$J26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$F26&lt;&gt;"",Pronostici!$G26&lt;&gt;"",Pronostici!$F26=Partite!$G26,Pronostici!$G26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$P26)=1),Config!$D$9,Config!$D$6),IF(AND($J26&lt;&gt;"",$J26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$J26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$I26&lt;&gt;"",Pronostici!$J26&lt;&gt;"",Pronostici!$I26=Partite!$G26,Pronostici!$J26=Partite!$H26),Config!$D$6,IF(AND($K26&lt;&gt;"",$K26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$I26&lt;&gt;"",Pronostici!$J26&lt;&gt;"",Pronostici!$I26=Partite!$G26,Pronostici!$J26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$Q26)=1),Config!$D$9,Config!$D$6),IF(AND($K26&lt;&gt;"",$K26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$K26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$L26&lt;&gt;"",Pronostici!$M26&lt;&gt;"",Pronostici!$L26=Partite!$G26,Pronostici!$M26=Partite!$H26),Config!$D$6,IF(AND($L26&lt;&gt;"",$L26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$L26&lt;&gt;"",Pronostici!$M26&lt;&gt;"",Pronostici!$L26=Partite!$G26,Pronostici!$M26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$R26)=1),Config!$D$9,Config!$D$6),IF(AND($L26&lt;&gt;"",$L26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$L26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$O26&lt;&gt;"",Pronostici!$P26&lt;&gt;"",Pronostici!$O26=Partite!$G26,Pronostici!$P26=Partite!$H26),Config!$D$6,IF(AND($M26&lt;&gt;"",$M26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$O26&lt;&gt;"",Pronostici!$P26&lt;&gt;"",Pronostici!$O26=Partite!$G26,Pronostici!$P26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$S26)=1),Config!$D$9,Config!$D$6),IF(AND($M26&lt;&gt;"",$M26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$M26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H26" s="22">
-        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$R26&lt;&gt;"",Pronostici!$S26&lt;&gt;"",Pronostici!$R26=Partite!$G26,Pronostici!$S26=Partite!$H26),Config!$D$6,IF(AND($N26&lt;&gt;"",$N26=Partite!$I26),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K26&lt;&gt;"Giocata","",IF(AND(Pronostici!$R26&lt;&gt;"",Pronostici!$S26&lt;&gt;"",Pronostici!$R26=Partite!$G26,Pronostici!$S26=Partite!$H26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($P26:$T26,$T26)=1),Config!$D$9,Config!$D$6),IF(AND($N26&lt;&gt;"",$N26=Partite!$I26),IF(AND($B26&gt;=Config!$D$17,COUNTIF($J26:$N26,$N26)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J26" s="63">
@@ -9240,6 +9725,26 @@
       </c>
       <c r="N26" s="63">
         <f>IF(Pronostici!$Q26&lt;&gt;"",UPPER(Pronostici!$Q26),IF(OR(Pronostici!$R26="",Pronostici!$S26=""),"",IF(Pronostici!$R26&gt;Pronostici!$S26,"1",IF(Pronostici!$R26=Pronostici!$S26,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P26" s="63">
+        <f>IF(OR(Pronostici!$F26="",Pronostici!$G26=""),"",Pronostici!$F26&amp;" a "&amp;Pronostici!$G26)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="63">
+        <f>IF(OR(Pronostici!$I26="",Pronostici!$J26=""),"",Pronostici!$I26&amp;" a "&amp;Pronostici!$J26)</f>
+        <v/>
+      </c>
+      <c r="R26" s="63">
+        <f>IF(OR(Pronostici!$L26="",Pronostici!$M26=""),"",Pronostici!$L26&amp;" a "&amp;Pronostici!$M26)</f>
+        <v/>
+      </c>
+      <c r="S26" s="63">
+        <f>IF(OR(Pronostici!$O26="",Pronostici!$P26=""),"",Pronostici!$O26&amp;" a "&amp;Pronostici!$P26)</f>
+        <v/>
+      </c>
+      <c r="T26" s="63">
+        <f>IF(OR(Pronostici!$R26="",Pronostici!$S26=""),"",Pronostici!$R26&amp;" a "&amp;Pronostici!$S26)</f>
         <v/>
       </c>
     </row>
@@ -9257,23 +9762,23 @@
         <v/>
       </c>
       <c r="D27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$F27&lt;&gt;"",Pronostici!$G27&lt;&gt;"",Pronostici!$F27=Partite!$G27,Pronostici!$G27=Partite!$H27),Config!$D$6,IF(AND($J27&lt;&gt;"",$J27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$F27&lt;&gt;"",Pronostici!$G27&lt;&gt;"",Pronostici!$F27=Partite!$G27,Pronostici!$G27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$P27)=1),Config!$D$9,Config!$D$6),IF(AND($J27&lt;&gt;"",$J27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$J27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$I27&lt;&gt;"",Pronostici!$J27&lt;&gt;"",Pronostici!$I27=Partite!$G27,Pronostici!$J27=Partite!$H27),Config!$D$6,IF(AND($K27&lt;&gt;"",$K27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$I27&lt;&gt;"",Pronostici!$J27&lt;&gt;"",Pronostici!$I27=Partite!$G27,Pronostici!$J27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$Q27)=1),Config!$D$9,Config!$D$6),IF(AND($K27&lt;&gt;"",$K27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$K27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$L27&lt;&gt;"",Pronostici!$M27&lt;&gt;"",Pronostici!$L27=Partite!$G27,Pronostici!$M27=Partite!$H27),Config!$D$6,IF(AND($L27&lt;&gt;"",$L27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$L27&lt;&gt;"",Pronostici!$M27&lt;&gt;"",Pronostici!$L27=Partite!$G27,Pronostici!$M27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$R27)=1),Config!$D$9,Config!$D$6),IF(AND($L27&lt;&gt;"",$L27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$L27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$O27&lt;&gt;"",Pronostici!$P27&lt;&gt;"",Pronostici!$O27=Partite!$G27,Pronostici!$P27=Partite!$H27),Config!$D$6,IF(AND($M27&lt;&gt;"",$M27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$O27&lt;&gt;"",Pronostici!$P27&lt;&gt;"",Pronostici!$O27=Partite!$G27,Pronostici!$P27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$S27)=1),Config!$D$9,Config!$D$6),IF(AND($M27&lt;&gt;"",$M27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$M27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H27" s="22">
-        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$R27&lt;&gt;"",Pronostici!$S27&lt;&gt;"",Pronostici!$R27=Partite!$G27,Pronostici!$S27=Partite!$H27),Config!$D$6,IF(AND($N27&lt;&gt;"",$N27=Partite!$I27),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K27&lt;&gt;"Giocata","",IF(AND(Pronostici!$R27&lt;&gt;"",Pronostici!$S27&lt;&gt;"",Pronostici!$R27=Partite!$G27,Pronostici!$S27=Partite!$H27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($P27:$T27,$T27)=1),Config!$D$9,Config!$D$6),IF(AND($N27&lt;&gt;"",$N27=Partite!$I27),IF(AND($B27&gt;=Config!$D$17,COUNTIF($J27:$N27,$N27)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J27" s="63">
@@ -9294,6 +9799,26 @@
       </c>
       <c r="N27" s="63">
         <f>IF(Pronostici!$Q27&lt;&gt;"",UPPER(Pronostici!$Q27),IF(OR(Pronostici!$R27="",Pronostici!$S27=""),"",IF(Pronostici!$R27&gt;Pronostici!$S27,"1",IF(Pronostici!$R27=Pronostici!$S27,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P27" s="63">
+        <f>IF(OR(Pronostici!$F27="",Pronostici!$G27=""),"",Pronostici!$F27&amp;" a "&amp;Pronostici!$G27)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="63">
+        <f>IF(OR(Pronostici!$I27="",Pronostici!$J27=""),"",Pronostici!$I27&amp;" a "&amp;Pronostici!$J27)</f>
+        <v/>
+      </c>
+      <c r="R27" s="63">
+        <f>IF(OR(Pronostici!$L27="",Pronostici!$M27=""),"",Pronostici!$L27&amp;" a "&amp;Pronostici!$M27)</f>
+        <v/>
+      </c>
+      <c r="S27" s="63">
+        <f>IF(OR(Pronostici!$O27="",Pronostici!$P27=""),"",Pronostici!$O27&amp;" a "&amp;Pronostici!$P27)</f>
+        <v/>
+      </c>
+      <c r="T27" s="63">
+        <f>IF(OR(Pronostici!$R27="",Pronostici!$S27=""),"",Pronostici!$R27&amp;" a "&amp;Pronostici!$S27)</f>
         <v/>
       </c>
     </row>
@@ -9311,23 +9836,23 @@
         <v/>
       </c>
       <c r="D28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$F28&lt;&gt;"",Pronostici!$G28&lt;&gt;"",Pronostici!$F28=Partite!$G28,Pronostici!$G28=Partite!$H28),Config!$D$6,IF(AND($J28&lt;&gt;"",$J28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$F28&lt;&gt;"",Pronostici!$G28&lt;&gt;"",Pronostici!$F28=Partite!$G28,Pronostici!$G28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$P28)=1),Config!$D$9,Config!$D$6),IF(AND($J28&lt;&gt;"",$J28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$J28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$I28&lt;&gt;"",Pronostici!$J28&lt;&gt;"",Pronostici!$I28=Partite!$G28,Pronostici!$J28=Partite!$H28),Config!$D$6,IF(AND($K28&lt;&gt;"",$K28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$I28&lt;&gt;"",Pronostici!$J28&lt;&gt;"",Pronostici!$I28=Partite!$G28,Pronostici!$J28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$Q28)=1),Config!$D$9,Config!$D$6),IF(AND($K28&lt;&gt;"",$K28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$K28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$L28&lt;&gt;"",Pronostici!$M28&lt;&gt;"",Pronostici!$L28=Partite!$G28,Pronostici!$M28=Partite!$H28),Config!$D$6,IF(AND($L28&lt;&gt;"",$L28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$L28&lt;&gt;"",Pronostici!$M28&lt;&gt;"",Pronostici!$L28=Partite!$G28,Pronostici!$M28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$R28)=1),Config!$D$9,Config!$D$6),IF(AND($L28&lt;&gt;"",$L28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$L28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$O28&lt;&gt;"",Pronostici!$P28&lt;&gt;"",Pronostici!$O28=Partite!$G28,Pronostici!$P28=Partite!$H28),Config!$D$6,IF(AND($M28&lt;&gt;"",$M28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$O28&lt;&gt;"",Pronostici!$P28&lt;&gt;"",Pronostici!$O28=Partite!$G28,Pronostici!$P28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$S28)=1),Config!$D$9,Config!$D$6),IF(AND($M28&lt;&gt;"",$M28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$M28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H28" s="22">
-        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$R28&lt;&gt;"",Pronostici!$S28&lt;&gt;"",Pronostici!$R28=Partite!$G28,Pronostici!$S28=Partite!$H28),Config!$D$6,IF(AND($N28&lt;&gt;"",$N28=Partite!$I28),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K28&lt;&gt;"Giocata","",IF(AND(Pronostici!$R28&lt;&gt;"",Pronostici!$S28&lt;&gt;"",Pronostici!$R28=Partite!$G28,Pronostici!$S28=Partite!$H28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($P28:$T28,$T28)=1),Config!$D$9,Config!$D$6),IF(AND($N28&lt;&gt;"",$N28=Partite!$I28),IF(AND($B28&gt;=Config!$D$17,COUNTIF($J28:$N28,$N28)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J28" s="63">
@@ -9348,6 +9873,26 @@
       </c>
       <c r="N28" s="63">
         <f>IF(Pronostici!$Q28&lt;&gt;"",UPPER(Pronostici!$Q28),IF(OR(Pronostici!$R28="",Pronostici!$S28=""),"",IF(Pronostici!$R28&gt;Pronostici!$S28,"1",IF(Pronostici!$R28=Pronostici!$S28,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P28" s="63">
+        <f>IF(OR(Pronostici!$F28="",Pronostici!$G28=""),"",Pronostici!$F28&amp;" a "&amp;Pronostici!$G28)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="63">
+        <f>IF(OR(Pronostici!$I28="",Pronostici!$J28=""),"",Pronostici!$I28&amp;" a "&amp;Pronostici!$J28)</f>
+        <v/>
+      </c>
+      <c r="R28" s="63">
+        <f>IF(OR(Pronostici!$L28="",Pronostici!$M28=""),"",Pronostici!$L28&amp;" a "&amp;Pronostici!$M28)</f>
+        <v/>
+      </c>
+      <c r="S28" s="63">
+        <f>IF(OR(Pronostici!$O28="",Pronostici!$P28=""),"",Pronostici!$O28&amp;" a "&amp;Pronostici!$P28)</f>
+        <v/>
+      </c>
+      <c r="T28" s="63">
+        <f>IF(OR(Pronostici!$R28="",Pronostici!$S28=""),"",Pronostici!$R28&amp;" a "&amp;Pronostici!$S28)</f>
         <v/>
       </c>
     </row>
@@ -9365,23 +9910,23 @@
         <v/>
       </c>
       <c r="D29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$F29&lt;&gt;"",Pronostici!$G29&lt;&gt;"",Pronostici!$F29=Partite!$G29,Pronostici!$G29=Partite!$H29),Config!$D$6,IF(AND($J29&lt;&gt;"",$J29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$F29&lt;&gt;"",Pronostici!$G29&lt;&gt;"",Pronostici!$F29=Partite!$G29,Pronostici!$G29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$P29)=1),Config!$D$9,Config!$D$6),IF(AND($J29&lt;&gt;"",$J29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$J29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$I29&lt;&gt;"",Pronostici!$J29&lt;&gt;"",Pronostici!$I29=Partite!$G29,Pronostici!$J29=Partite!$H29),Config!$D$6,IF(AND($K29&lt;&gt;"",$K29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$I29&lt;&gt;"",Pronostici!$J29&lt;&gt;"",Pronostici!$I29=Partite!$G29,Pronostici!$J29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$Q29)=1),Config!$D$9,Config!$D$6),IF(AND($K29&lt;&gt;"",$K29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$K29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$L29&lt;&gt;"",Pronostici!$M29&lt;&gt;"",Pronostici!$L29=Partite!$G29,Pronostici!$M29=Partite!$H29),Config!$D$6,IF(AND($L29&lt;&gt;"",$L29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$L29&lt;&gt;"",Pronostici!$M29&lt;&gt;"",Pronostici!$L29=Partite!$G29,Pronostici!$M29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$R29)=1),Config!$D$9,Config!$D$6),IF(AND($L29&lt;&gt;"",$L29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$L29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$O29&lt;&gt;"",Pronostici!$P29&lt;&gt;"",Pronostici!$O29=Partite!$G29,Pronostici!$P29=Partite!$H29),Config!$D$6,IF(AND($M29&lt;&gt;"",$M29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$O29&lt;&gt;"",Pronostici!$P29&lt;&gt;"",Pronostici!$O29=Partite!$G29,Pronostici!$P29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$S29)=1),Config!$D$9,Config!$D$6),IF(AND($M29&lt;&gt;"",$M29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$M29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H29" s="22">
-        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$R29&lt;&gt;"",Pronostici!$S29&lt;&gt;"",Pronostici!$R29=Partite!$G29,Pronostici!$S29=Partite!$H29),Config!$D$6,IF(AND($N29&lt;&gt;"",$N29=Partite!$I29),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K29&lt;&gt;"Giocata","",IF(AND(Pronostici!$R29&lt;&gt;"",Pronostici!$S29&lt;&gt;"",Pronostici!$R29=Partite!$G29,Pronostici!$S29=Partite!$H29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($P29:$T29,$T29)=1),Config!$D$9,Config!$D$6),IF(AND($N29&lt;&gt;"",$N29=Partite!$I29),IF(AND($B29&gt;=Config!$D$17,COUNTIF($J29:$N29,$N29)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J29" s="63">
@@ -9402,6 +9947,26 @@
       </c>
       <c r="N29" s="63">
         <f>IF(Pronostici!$Q29&lt;&gt;"",UPPER(Pronostici!$Q29),IF(OR(Pronostici!$R29="",Pronostici!$S29=""),"",IF(Pronostici!$R29&gt;Pronostici!$S29,"1",IF(Pronostici!$R29=Pronostici!$S29,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P29" s="63">
+        <f>IF(OR(Pronostici!$F29="",Pronostici!$G29=""),"",Pronostici!$F29&amp;" a "&amp;Pronostici!$G29)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="63">
+        <f>IF(OR(Pronostici!$I29="",Pronostici!$J29=""),"",Pronostici!$I29&amp;" a "&amp;Pronostici!$J29)</f>
+        <v/>
+      </c>
+      <c r="R29" s="63">
+        <f>IF(OR(Pronostici!$L29="",Pronostici!$M29=""),"",Pronostici!$L29&amp;" a "&amp;Pronostici!$M29)</f>
+        <v/>
+      </c>
+      <c r="S29" s="63">
+        <f>IF(OR(Pronostici!$O29="",Pronostici!$P29=""),"",Pronostici!$O29&amp;" a "&amp;Pronostici!$P29)</f>
+        <v/>
+      </c>
+      <c r="T29" s="63">
+        <f>IF(OR(Pronostici!$R29="",Pronostici!$S29=""),"",Pronostici!$R29&amp;" a "&amp;Pronostici!$S29)</f>
         <v/>
       </c>
     </row>
@@ -9419,23 +9984,23 @@
         <v/>
       </c>
       <c r="D30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$F30&lt;&gt;"",Pronostici!$G30&lt;&gt;"",Pronostici!$F30=Partite!$G30,Pronostici!$G30=Partite!$H30),Config!$D$6,IF(AND($J30&lt;&gt;"",$J30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$F30&lt;&gt;"",Pronostici!$G30&lt;&gt;"",Pronostici!$F30=Partite!$G30,Pronostici!$G30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$P30)=1),Config!$D$9,Config!$D$6),IF(AND($J30&lt;&gt;"",$J30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$J30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$I30&lt;&gt;"",Pronostici!$J30&lt;&gt;"",Pronostici!$I30=Partite!$G30,Pronostici!$J30=Partite!$H30),Config!$D$6,IF(AND($K30&lt;&gt;"",$K30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$I30&lt;&gt;"",Pronostici!$J30&lt;&gt;"",Pronostici!$I30=Partite!$G30,Pronostici!$J30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$Q30)=1),Config!$D$9,Config!$D$6),IF(AND($K30&lt;&gt;"",$K30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$K30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$L30&lt;&gt;"",Pronostici!$M30&lt;&gt;"",Pronostici!$L30=Partite!$G30,Pronostici!$M30=Partite!$H30),Config!$D$6,IF(AND($L30&lt;&gt;"",$L30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$L30&lt;&gt;"",Pronostici!$M30&lt;&gt;"",Pronostici!$L30=Partite!$G30,Pronostici!$M30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$R30)=1),Config!$D$9,Config!$D$6),IF(AND($L30&lt;&gt;"",$L30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$L30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$O30&lt;&gt;"",Pronostici!$P30&lt;&gt;"",Pronostici!$O30=Partite!$G30,Pronostici!$P30=Partite!$H30),Config!$D$6,IF(AND($M30&lt;&gt;"",$M30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$O30&lt;&gt;"",Pronostici!$P30&lt;&gt;"",Pronostici!$O30=Partite!$G30,Pronostici!$P30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$S30)=1),Config!$D$9,Config!$D$6),IF(AND($M30&lt;&gt;"",$M30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$M30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H30" s="22">
-        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$R30&lt;&gt;"",Pronostici!$S30&lt;&gt;"",Pronostici!$R30=Partite!$G30,Pronostici!$S30=Partite!$H30),Config!$D$6,IF(AND($N30&lt;&gt;"",$N30=Partite!$I30),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K30&lt;&gt;"Giocata","",IF(AND(Pronostici!$R30&lt;&gt;"",Pronostici!$S30&lt;&gt;"",Pronostici!$R30=Partite!$G30,Pronostici!$S30=Partite!$H30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($P30:$T30,$T30)=1),Config!$D$9,Config!$D$6),IF(AND($N30&lt;&gt;"",$N30=Partite!$I30),IF(AND($B30&gt;=Config!$D$17,COUNTIF($J30:$N30,$N30)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J30" s="63">
@@ -9456,6 +10021,26 @@
       </c>
       <c r="N30" s="63">
         <f>IF(Pronostici!$Q30&lt;&gt;"",UPPER(Pronostici!$Q30),IF(OR(Pronostici!$R30="",Pronostici!$S30=""),"",IF(Pronostici!$R30&gt;Pronostici!$S30,"1",IF(Pronostici!$R30=Pronostici!$S30,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P30" s="63">
+        <f>IF(OR(Pronostici!$F30="",Pronostici!$G30=""),"",Pronostici!$F30&amp;" a "&amp;Pronostici!$G30)</f>
+        <v/>
+      </c>
+      <c r="Q30" s="63">
+        <f>IF(OR(Pronostici!$I30="",Pronostici!$J30=""),"",Pronostici!$I30&amp;" a "&amp;Pronostici!$J30)</f>
+        <v/>
+      </c>
+      <c r="R30" s="63">
+        <f>IF(OR(Pronostici!$L30="",Pronostici!$M30=""),"",Pronostici!$L30&amp;" a "&amp;Pronostici!$M30)</f>
+        <v/>
+      </c>
+      <c r="S30" s="63">
+        <f>IF(OR(Pronostici!$O30="",Pronostici!$P30=""),"",Pronostici!$O30&amp;" a "&amp;Pronostici!$P30)</f>
+        <v/>
+      </c>
+      <c r="T30" s="63">
+        <f>IF(OR(Pronostici!$R30="",Pronostici!$S30=""),"",Pronostici!$R30&amp;" a "&amp;Pronostici!$S30)</f>
         <v/>
       </c>
     </row>
@@ -9473,23 +10058,23 @@
         <v/>
       </c>
       <c r="D31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$F31&lt;&gt;"",Pronostici!$G31&lt;&gt;"",Pronostici!$F31=Partite!$G31,Pronostici!$G31=Partite!$H31),Config!$D$6,IF(AND($J31&lt;&gt;"",$J31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$F31&lt;&gt;"",Pronostici!$G31&lt;&gt;"",Pronostici!$F31=Partite!$G31,Pronostici!$G31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$P31)=1),Config!$D$9,Config!$D$6),IF(AND($J31&lt;&gt;"",$J31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$J31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$I31&lt;&gt;"",Pronostici!$J31&lt;&gt;"",Pronostici!$I31=Partite!$G31,Pronostici!$J31=Partite!$H31),Config!$D$6,IF(AND($K31&lt;&gt;"",$K31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$I31&lt;&gt;"",Pronostici!$J31&lt;&gt;"",Pronostici!$I31=Partite!$G31,Pronostici!$J31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$Q31)=1),Config!$D$9,Config!$D$6),IF(AND($K31&lt;&gt;"",$K31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$K31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$L31&lt;&gt;"",Pronostici!$M31&lt;&gt;"",Pronostici!$L31=Partite!$G31,Pronostici!$M31=Partite!$H31),Config!$D$6,IF(AND($L31&lt;&gt;"",$L31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$L31&lt;&gt;"",Pronostici!$M31&lt;&gt;"",Pronostici!$L31=Partite!$G31,Pronostici!$M31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$R31)=1),Config!$D$9,Config!$D$6),IF(AND($L31&lt;&gt;"",$L31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$L31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$O31&lt;&gt;"",Pronostici!$P31&lt;&gt;"",Pronostici!$O31=Partite!$G31,Pronostici!$P31=Partite!$H31),Config!$D$6,IF(AND($M31&lt;&gt;"",$M31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$O31&lt;&gt;"",Pronostici!$P31&lt;&gt;"",Pronostici!$O31=Partite!$G31,Pronostici!$P31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$S31)=1),Config!$D$9,Config!$D$6),IF(AND($M31&lt;&gt;"",$M31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$M31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H31" s="22">
-        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$R31&lt;&gt;"",Pronostici!$S31&lt;&gt;"",Pronostici!$R31=Partite!$G31,Pronostici!$S31=Partite!$H31),Config!$D$6,IF(AND($N31&lt;&gt;"",$N31=Partite!$I31),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K31&lt;&gt;"Giocata","",IF(AND(Pronostici!$R31&lt;&gt;"",Pronostici!$S31&lt;&gt;"",Pronostici!$R31=Partite!$G31,Pronostici!$S31=Partite!$H31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($P31:$T31,$T31)=1),Config!$D$9,Config!$D$6),IF(AND($N31&lt;&gt;"",$N31=Partite!$I31),IF(AND($B31&gt;=Config!$D$17,COUNTIF($J31:$N31,$N31)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J31" s="63">
@@ -9510,6 +10095,26 @@
       </c>
       <c r="N31" s="63">
         <f>IF(Pronostici!$Q31&lt;&gt;"",UPPER(Pronostici!$Q31),IF(OR(Pronostici!$R31="",Pronostici!$S31=""),"",IF(Pronostici!$R31&gt;Pronostici!$S31,"1",IF(Pronostici!$R31=Pronostici!$S31,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P31" s="63">
+        <f>IF(OR(Pronostici!$F31="",Pronostici!$G31=""),"",Pronostici!$F31&amp;" a "&amp;Pronostici!$G31)</f>
+        <v/>
+      </c>
+      <c r="Q31" s="63">
+        <f>IF(OR(Pronostici!$I31="",Pronostici!$J31=""),"",Pronostici!$I31&amp;" a "&amp;Pronostici!$J31)</f>
+        <v/>
+      </c>
+      <c r="R31" s="63">
+        <f>IF(OR(Pronostici!$L31="",Pronostici!$M31=""),"",Pronostici!$L31&amp;" a "&amp;Pronostici!$M31)</f>
+        <v/>
+      </c>
+      <c r="S31" s="63">
+        <f>IF(OR(Pronostici!$O31="",Pronostici!$P31=""),"",Pronostici!$O31&amp;" a "&amp;Pronostici!$P31)</f>
+        <v/>
+      </c>
+      <c r="T31" s="63">
+        <f>IF(OR(Pronostici!$R31="",Pronostici!$S31=""),"",Pronostici!$R31&amp;" a "&amp;Pronostici!$S31)</f>
         <v/>
       </c>
     </row>
@@ -9527,23 +10132,23 @@
         <v/>
       </c>
       <c r="D32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$F32&lt;&gt;"",Pronostici!$G32&lt;&gt;"",Pronostici!$F32=Partite!$G32,Pronostici!$G32=Partite!$H32),Config!$D$6,IF(AND($J32&lt;&gt;"",$J32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$F32&lt;&gt;"",Pronostici!$G32&lt;&gt;"",Pronostici!$F32=Partite!$G32,Pronostici!$G32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$P32)=1),Config!$D$9,Config!$D$6),IF(AND($J32&lt;&gt;"",$J32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$J32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$I32&lt;&gt;"",Pronostici!$J32&lt;&gt;"",Pronostici!$I32=Partite!$G32,Pronostici!$J32=Partite!$H32),Config!$D$6,IF(AND($K32&lt;&gt;"",$K32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$I32&lt;&gt;"",Pronostici!$J32&lt;&gt;"",Pronostici!$I32=Partite!$G32,Pronostici!$J32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$Q32)=1),Config!$D$9,Config!$D$6),IF(AND($K32&lt;&gt;"",$K32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$K32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$L32&lt;&gt;"",Pronostici!$M32&lt;&gt;"",Pronostici!$L32=Partite!$G32,Pronostici!$M32=Partite!$H32),Config!$D$6,IF(AND($L32&lt;&gt;"",$L32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$L32&lt;&gt;"",Pronostici!$M32&lt;&gt;"",Pronostici!$L32=Partite!$G32,Pronostici!$M32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$R32)=1),Config!$D$9,Config!$D$6),IF(AND($L32&lt;&gt;"",$L32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$L32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$O32&lt;&gt;"",Pronostici!$P32&lt;&gt;"",Pronostici!$O32=Partite!$G32,Pronostici!$P32=Partite!$H32),Config!$D$6,IF(AND($M32&lt;&gt;"",$M32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$O32&lt;&gt;"",Pronostici!$P32&lt;&gt;"",Pronostici!$O32=Partite!$G32,Pronostici!$P32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$S32)=1),Config!$D$9,Config!$D$6),IF(AND($M32&lt;&gt;"",$M32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$M32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H32" s="22">
-        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$R32&lt;&gt;"",Pronostici!$S32&lt;&gt;"",Pronostici!$R32=Partite!$G32,Pronostici!$S32=Partite!$H32),Config!$D$6,IF(AND($N32&lt;&gt;"",$N32=Partite!$I32),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K32&lt;&gt;"Giocata","",IF(AND(Pronostici!$R32&lt;&gt;"",Pronostici!$S32&lt;&gt;"",Pronostici!$R32=Partite!$G32,Pronostici!$S32=Partite!$H32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($P32:$T32,$T32)=1),Config!$D$9,Config!$D$6),IF(AND($N32&lt;&gt;"",$N32=Partite!$I32),IF(AND($B32&gt;=Config!$D$17,COUNTIF($J32:$N32,$N32)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J32" s="63">
@@ -9564,6 +10169,26 @@
       </c>
       <c r="N32" s="63">
         <f>IF(Pronostici!$Q32&lt;&gt;"",UPPER(Pronostici!$Q32),IF(OR(Pronostici!$R32="",Pronostici!$S32=""),"",IF(Pronostici!$R32&gt;Pronostici!$S32,"1",IF(Pronostici!$R32=Pronostici!$S32,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P32" s="63">
+        <f>IF(OR(Pronostici!$F32="",Pronostici!$G32=""),"",Pronostici!$F32&amp;" a "&amp;Pronostici!$G32)</f>
+        <v/>
+      </c>
+      <c r="Q32" s="63">
+        <f>IF(OR(Pronostici!$I32="",Pronostici!$J32=""),"",Pronostici!$I32&amp;" a "&amp;Pronostici!$J32)</f>
+        <v/>
+      </c>
+      <c r="R32" s="63">
+        <f>IF(OR(Pronostici!$L32="",Pronostici!$M32=""),"",Pronostici!$L32&amp;" a "&amp;Pronostici!$M32)</f>
+        <v/>
+      </c>
+      <c r="S32" s="63">
+        <f>IF(OR(Pronostici!$O32="",Pronostici!$P32=""),"",Pronostici!$O32&amp;" a "&amp;Pronostici!$P32)</f>
+        <v/>
+      </c>
+      <c r="T32" s="63">
+        <f>IF(OR(Pronostici!$R32="",Pronostici!$S32=""),"",Pronostici!$R32&amp;" a "&amp;Pronostici!$S32)</f>
         <v/>
       </c>
     </row>
@@ -9581,23 +10206,23 @@
         <v/>
       </c>
       <c r="D33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$F33&lt;&gt;"",Pronostici!$G33&lt;&gt;"",Pronostici!$F33=Partite!$G33,Pronostici!$G33=Partite!$H33),Config!$D$6,IF(AND($J33&lt;&gt;"",$J33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$F33&lt;&gt;"",Pronostici!$G33&lt;&gt;"",Pronostici!$F33=Partite!$G33,Pronostici!$G33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$P33)=1),Config!$D$9,Config!$D$6),IF(AND($J33&lt;&gt;"",$J33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$J33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$I33&lt;&gt;"",Pronostici!$J33&lt;&gt;"",Pronostici!$I33=Partite!$G33,Pronostici!$J33=Partite!$H33),Config!$D$6,IF(AND($K33&lt;&gt;"",$K33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$I33&lt;&gt;"",Pronostici!$J33&lt;&gt;"",Pronostici!$I33=Partite!$G33,Pronostici!$J33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$Q33)=1),Config!$D$9,Config!$D$6),IF(AND($K33&lt;&gt;"",$K33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$K33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$L33&lt;&gt;"",Pronostici!$M33&lt;&gt;"",Pronostici!$L33=Partite!$G33,Pronostici!$M33=Partite!$H33),Config!$D$6,IF(AND($L33&lt;&gt;"",$L33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$L33&lt;&gt;"",Pronostici!$M33&lt;&gt;"",Pronostici!$L33=Partite!$G33,Pronostici!$M33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$R33)=1),Config!$D$9,Config!$D$6),IF(AND($L33&lt;&gt;"",$L33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$L33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$O33&lt;&gt;"",Pronostici!$P33&lt;&gt;"",Pronostici!$O33=Partite!$G33,Pronostici!$P33=Partite!$H33),Config!$D$6,IF(AND($M33&lt;&gt;"",$M33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$O33&lt;&gt;"",Pronostici!$P33&lt;&gt;"",Pronostici!$O33=Partite!$G33,Pronostici!$P33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$S33)=1),Config!$D$9,Config!$D$6),IF(AND($M33&lt;&gt;"",$M33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$M33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H33" s="27">
-        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$R33&lt;&gt;"",Pronostici!$S33&lt;&gt;"",Pronostici!$R33=Partite!$G33,Pronostici!$S33=Partite!$H33),Config!$D$6,IF(AND($N33&lt;&gt;"",$N33=Partite!$I33),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K33&lt;&gt;"Giocata","",IF(AND(Pronostici!$R33&lt;&gt;"",Pronostici!$S33&lt;&gt;"",Pronostici!$R33=Partite!$G33,Pronostici!$S33=Partite!$H33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($P33:$T33,$T33)=1),Config!$D$9,Config!$D$6),IF(AND($N33&lt;&gt;"",$N33=Partite!$I33),IF(AND($B33&gt;=Config!$D$17,COUNTIF($J33:$N33,$N33)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J33" s="63">
@@ -9618,6 +10243,26 @@
       </c>
       <c r="N33" s="63">
         <f>IF(Pronostici!$Q33&lt;&gt;"",UPPER(Pronostici!$Q33),IF(OR(Pronostici!$R33="",Pronostici!$S33=""),"",IF(Pronostici!$R33&gt;Pronostici!$S33,"1",IF(Pronostici!$R33=Pronostici!$S33,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P33" s="63">
+        <f>IF(OR(Pronostici!$F33="",Pronostici!$G33=""),"",Pronostici!$F33&amp;" a "&amp;Pronostici!$G33)</f>
+        <v/>
+      </c>
+      <c r="Q33" s="63">
+        <f>IF(OR(Pronostici!$I33="",Pronostici!$J33=""),"",Pronostici!$I33&amp;" a "&amp;Pronostici!$J33)</f>
+        <v/>
+      </c>
+      <c r="R33" s="63">
+        <f>IF(OR(Pronostici!$L33="",Pronostici!$M33=""),"",Pronostici!$L33&amp;" a "&amp;Pronostici!$M33)</f>
+        <v/>
+      </c>
+      <c r="S33" s="63">
+        <f>IF(OR(Pronostici!$O33="",Pronostici!$P33=""),"",Pronostici!$O33&amp;" a "&amp;Pronostici!$P33)</f>
+        <v/>
+      </c>
+      <c r="T33" s="63">
+        <f>IF(OR(Pronostici!$R33="",Pronostici!$S33=""),"",Pronostici!$R33&amp;" a "&amp;Pronostici!$S33)</f>
         <v/>
       </c>
     </row>
@@ -9635,23 +10280,23 @@
         <v/>
       </c>
       <c r="D34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$F34&lt;&gt;"",Pronostici!$G34&lt;&gt;"",Pronostici!$F34=Partite!$G34,Pronostici!$G34=Partite!$H34),Config!$D$6,IF(AND($J34&lt;&gt;"",$J34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$F34&lt;&gt;"",Pronostici!$G34&lt;&gt;"",Pronostici!$F34=Partite!$G34,Pronostici!$G34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$P34)=1),Config!$D$9,Config!$D$6),IF(AND($J34&lt;&gt;"",$J34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$J34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$I34&lt;&gt;"",Pronostici!$J34&lt;&gt;"",Pronostici!$I34=Partite!$G34,Pronostici!$J34=Partite!$H34),Config!$D$6,IF(AND($K34&lt;&gt;"",$K34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$I34&lt;&gt;"",Pronostici!$J34&lt;&gt;"",Pronostici!$I34=Partite!$G34,Pronostici!$J34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$Q34)=1),Config!$D$9,Config!$D$6),IF(AND($K34&lt;&gt;"",$K34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$K34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$L34&lt;&gt;"",Pronostici!$M34&lt;&gt;"",Pronostici!$L34=Partite!$G34,Pronostici!$M34=Partite!$H34),Config!$D$6,IF(AND($L34&lt;&gt;"",$L34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$L34&lt;&gt;"",Pronostici!$M34&lt;&gt;"",Pronostici!$L34=Partite!$G34,Pronostici!$M34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$R34)=1),Config!$D$9,Config!$D$6),IF(AND($L34&lt;&gt;"",$L34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$L34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$O34&lt;&gt;"",Pronostici!$P34&lt;&gt;"",Pronostici!$O34=Partite!$G34,Pronostici!$P34=Partite!$H34),Config!$D$6,IF(AND($M34&lt;&gt;"",$M34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$O34&lt;&gt;"",Pronostici!$P34&lt;&gt;"",Pronostici!$O34=Partite!$G34,Pronostici!$P34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$S34)=1),Config!$D$9,Config!$D$6),IF(AND($M34&lt;&gt;"",$M34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$M34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H34" s="27">
-        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$R34&lt;&gt;"",Pronostici!$S34&lt;&gt;"",Pronostici!$R34=Partite!$G34,Pronostici!$S34=Partite!$H34),Config!$D$6,IF(AND($N34&lt;&gt;"",$N34=Partite!$I34),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K34&lt;&gt;"Giocata","",IF(AND(Pronostici!$R34&lt;&gt;"",Pronostici!$S34&lt;&gt;"",Pronostici!$R34=Partite!$G34,Pronostici!$S34=Partite!$H34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($P34:$T34,$T34)=1),Config!$D$9,Config!$D$6),IF(AND($N34&lt;&gt;"",$N34=Partite!$I34),IF(AND($B34&gt;=Config!$D$17,COUNTIF($J34:$N34,$N34)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J34" s="63">
@@ -9672,6 +10317,26 @@
       </c>
       <c r="N34" s="63">
         <f>IF(Pronostici!$Q34&lt;&gt;"",UPPER(Pronostici!$Q34),IF(OR(Pronostici!$R34="",Pronostici!$S34=""),"",IF(Pronostici!$R34&gt;Pronostici!$S34,"1",IF(Pronostici!$R34=Pronostici!$S34,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P34" s="63">
+        <f>IF(OR(Pronostici!$F34="",Pronostici!$G34=""),"",Pronostici!$F34&amp;" a "&amp;Pronostici!$G34)</f>
+        <v/>
+      </c>
+      <c r="Q34" s="63">
+        <f>IF(OR(Pronostici!$I34="",Pronostici!$J34=""),"",Pronostici!$I34&amp;" a "&amp;Pronostici!$J34)</f>
+        <v/>
+      </c>
+      <c r="R34" s="63">
+        <f>IF(OR(Pronostici!$L34="",Pronostici!$M34=""),"",Pronostici!$L34&amp;" a "&amp;Pronostici!$M34)</f>
+        <v/>
+      </c>
+      <c r="S34" s="63">
+        <f>IF(OR(Pronostici!$O34="",Pronostici!$P34=""),"",Pronostici!$O34&amp;" a "&amp;Pronostici!$P34)</f>
+        <v/>
+      </c>
+      <c r="T34" s="63">
+        <f>IF(OR(Pronostici!$R34="",Pronostici!$S34=""),"",Pronostici!$R34&amp;" a "&amp;Pronostici!$S34)</f>
         <v/>
       </c>
     </row>
@@ -9689,23 +10354,23 @@
         <v/>
       </c>
       <c r="D35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$F35&lt;&gt;"",Pronostici!$G35&lt;&gt;"",Pronostici!$F35=Partite!$G35,Pronostici!$G35=Partite!$H35),Config!$D$6,IF(AND($J35&lt;&gt;"",$J35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$F35&lt;&gt;"",Pronostici!$G35&lt;&gt;"",Pronostici!$F35=Partite!$G35,Pronostici!$G35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$P35)=1),Config!$D$9,Config!$D$6),IF(AND($J35&lt;&gt;"",$J35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$J35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$I35&lt;&gt;"",Pronostici!$J35&lt;&gt;"",Pronostici!$I35=Partite!$G35,Pronostici!$J35=Partite!$H35),Config!$D$6,IF(AND($K35&lt;&gt;"",$K35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$I35&lt;&gt;"",Pronostici!$J35&lt;&gt;"",Pronostici!$I35=Partite!$G35,Pronostici!$J35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$Q35)=1),Config!$D$9,Config!$D$6),IF(AND($K35&lt;&gt;"",$K35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$K35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$L35&lt;&gt;"",Pronostici!$M35&lt;&gt;"",Pronostici!$L35=Partite!$G35,Pronostici!$M35=Partite!$H35),Config!$D$6,IF(AND($L35&lt;&gt;"",$L35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$L35&lt;&gt;"",Pronostici!$M35&lt;&gt;"",Pronostici!$L35=Partite!$G35,Pronostici!$M35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$R35)=1),Config!$D$9,Config!$D$6),IF(AND($L35&lt;&gt;"",$L35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$L35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$O35&lt;&gt;"",Pronostici!$P35&lt;&gt;"",Pronostici!$O35=Partite!$G35,Pronostici!$P35=Partite!$H35),Config!$D$6,IF(AND($M35&lt;&gt;"",$M35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$O35&lt;&gt;"",Pronostici!$P35&lt;&gt;"",Pronostici!$O35=Partite!$G35,Pronostici!$P35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$S35)=1),Config!$D$9,Config!$D$6),IF(AND($M35&lt;&gt;"",$M35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$M35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H35" s="27">
-        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$R35&lt;&gt;"",Pronostici!$S35&lt;&gt;"",Pronostici!$R35=Partite!$G35,Pronostici!$S35=Partite!$H35),Config!$D$6,IF(AND($N35&lt;&gt;"",$N35=Partite!$I35),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K35&lt;&gt;"Giocata","",IF(AND(Pronostici!$R35&lt;&gt;"",Pronostici!$S35&lt;&gt;"",Pronostici!$R35=Partite!$G35,Pronostici!$S35=Partite!$H35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($P35:$T35,$T35)=1),Config!$D$9,Config!$D$6),IF(AND($N35&lt;&gt;"",$N35=Partite!$I35),IF(AND($B35&gt;=Config!$D$17,COUNTIF($J35:$N35,$N35)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J35" s="63">
@@ -9726,6 +10391,26 @@
       </c>
       <c r="N35" s="63">
         <f>IF(Pronostici!$Q35&lt;&gt;"",UPPER(Pronostici!$Q35),IF(OR(Pronostici!$R35="",Pronostici!$S35=""),"",IF(Pronostici!$R35&gt;Pronostici!$S35,"1",IF(Pronostici!$R35=Pronostici!$S35,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P35" s="63">
+        <f>IF(OR(Pronostici!$F35="",Pronostici!$G35=""),"",Pronostici!$F35&amp;" a "&amp;Pronostici!$G35)</f>
+        <v/>
+      </c>
+      <c r="Q35" s="63">
+        <f>IF(OR(Pronostici!$I35="",Pronostici!$J35=""),"",Pronostici!$I35&amp;" a "&amp;Pronostici!$J35)</f>
+        <v/>
+      </c>
+      <c r="R35" s="63">
+        <f>IF(OR(Pronostici!$L35="",Pronostici!$M35=""),"",Pronostici!$L35&amp;" a "&amp;Pronostici!$M35)</f>
+        <v/>
+      </c>
+      <c r="S35" s="63">
+        <f>IF(OR(Pronostici!$O35="",Pronostici!$P35=""),"",Pronostici!$O35&amp;" a "&amp;Pronostici!$P35)</f>
+        <v/>
+      </c>
+      <c r="T35" s="63">
+        <f>IF(OR(Pronostici!$R35="",Pronostici!$S35=""),"",Pronostici!$R35&amp;" a "&amp;Pronostici!$S35)</f>
         <v/>
       </c>
     </row>
@@ -9743,23 +10428,23 @@
         <v/>
       </c>
       <c r="D36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$F36&lt;&gt;"",Pronostici!$G36&lt;&gt;"",Pronostici!$F36=Partite!$G36,Pronostici!$G36=Partite!$H36),Config!$D$6,IF(AND($J36&lt;&gt;"",$J36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$F36&lt;&gt;"",Pronostici!$G36&lt;&gt;"",Pronostici!$F36=Partite!$G36,Pronostici!$G36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$P36)=1),Config!$D$9,Config!$D$6),IF(AND($J36&lt;&gt;"",$J36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$J36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$I36&lt;&gt;"",Pronostici!$J36&lt;&gt;"",Pronostici!$I36=Partite!$G36,Pronostici!$J36=Partite!$H36),Config!$D$6,IF(AND($K36&lt;&gt;"",$K36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$I36&lt;&gt;"",Pronostici!$J36&lt;&gt;"",Pronostici!$I36=Partite!$G36,Pronostici!$J36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$Q36)=1),Config!$D$9,Config!$D$6),IF(AND($K36&lt;&gt;"",$K36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$K36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$L36&lt;&gt;"",Pronostici!$M36&lt;&gt;"",Pronostici!$L36=Partite!$G36,Pronostici!$M36=Partite!$H36),Config!$D$6,IF(AND($L36&lt;&gt;"",$L36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$L36&lt;&gt;"",Pronostici!$M36&lt;&gt;"",Pronostici!$L36=Partite!$G36,Pronostici!$M36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$R36)=1),Config!$D$9,Config!$D$6),IF(AND($L36&lt;&gt;"",$L36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$L36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$O36&lt;&gt;"",Pronostici!$P36&lt;&gt;"",Pronostici!$O36=Partite!$G36,Pronostici!$P36=Partite!$H36),Config!$D$6,IF(AND($M36&lt;&gt;"",$M36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$O36&lt;&gt;"",Pronostici!$P36&lt;&gt;"",Pronostici!$O36=Partite!$G36,Pronostici!$P36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$S36)=1),Config!$D$9,Config!$D$6),IF(AND($M36&lt;&gt;"",$M36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$M36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H36" s="27">
-        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$R36&lt;&gt;"",Pronostici!$S36&lt;&gt;"",Pronostici!$R36=Partite!$G36,Pronostici!$S36=Partite!$H36),Config!$D$6,IF(AND($N36&lt;&gt;"",$N36=Partite!$I36),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K36&lt;&gt;"Giocata","",IF(AND(Pronostici!$R36&lt;&gt;"",Pronostici!$S36&lt;&gt;"",Pronostici!$R36=Partite!$G36,Pronostici!$S36=Partite!$H36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($P36:$T36,$T36)=1),Config!$D$9,Config!$D$6),IF(AND($N36&lt;&gt;"",$N36=Partite!$I36),IF(AND($B36&gt;=Config!$D$17,COUNTIF($J36:$N36,$N36)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J36" s="63">
@@ -9780,6 +10465,26 @@
       </c>
       <c r="N36" s="63">
         <f>IF(Pronostici!$Q36&lt;&gt;"",UPPER(Pronostici!$Q36),IF(OR(Pronostici!$R36="",Pronostici!$S36=""),"",IF(Pronostici!$R36&gt;Pronostici!$S36,"1",IF(Pronostici!$R36=Pronostici!$S36,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P36" s="63">
+        <f>IF(OR(Pronostici!$F36="",Pronostici!$G36=""),"",Pronostici!$F36&amp;" a "&amp;Pronostici!$G36)</f>
+        <v/>
+      </c>
+      <c r="Q36" s="63">
+        <f>IF(OR(Pronostici!$I36="",Pronostici!$J36=""),"",Pronostici!$I36&amp;" a "&amp;Pronostici!$J36)</f>
+        <v/>
+      </c>
+      <c r="R36" s="63">
+        <f>IF(OR(Pronostici!$L36="",Pronostici!$M36=""),"",Pronostici!$L36&amp;" a "&amp;Pronostici!$M36)</f>
+        <v/>
+      </c>
+      <c r="S36" s="63">
+        <f>IF(OR(Pronostici!$O36="",Pronostici!$P36=""),"",Pronostici!$O36&amp;" a "&amp;Pronostici!$P36)</f>
+        <v/>
+      </c>
+      <c r="T36" s="63">
+        <f>IF(OR(Pronostici!$R36="",Pronostici!$S36=""),"",Pronostici!$R36&amp;" a "&amp;Pronostici!$S36)</f>
         <v/>
       </c>
     </row>
@@ -9797,23 +10502,23 @@
         <v/>
       </c>
       <c r="D37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$F37&lt;&gt;"",Pronostici!$G37&lt;&gt;"",Pronostici!$F37=Partite!$G37,Pronostici!$G37=Partite!$H37),Config!$D$6,IF(AND($J37&lt;&gt;"",$J37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$F37&lt;&gt;"",Pronostici!$G37&lt;&gt;"",Pronostici!$F37=Partite!$G37,Pronostici!$G37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$P37)=1),Config!$D$9,Config!$D$6),IF(AND($J37&lt;&gt;"",$J37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$J37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$I37&lt;&gt;"",Pronostici!$J37&lt;&gt;"",Pronostici!$I37=Partite!$G37,Pronostici!$J37=Partite!$H37),Config!$D$6,IF(AND($K37&lt;&gt;"",$K37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$I37&lt;&gt;"",Pronostici!$J37&lt;&gt;"",Pronostici!$I37=Partite!$G37,Pronostici!$J37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$Q37)=1),Config!$D$9,Config!$D$6),IF(AND($K37&lt;&gt;"",$K37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$K37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$L37&lt;&gt;"",Pronostici!$M37&lt;&gt;"",Pronostici!$L37=Partite!$G37,Pronostici!$M37=Partite!$H37),Config!$D$6,IF(AND($L37&lt;&gt;"",$L37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$L37&lt;&gt;"",Pronostici!$M37&lt;&gt;"",Pronostici!$L37=Partite!$G37,Pronostici!$M37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$R37)=1),Config!$D$9,Config!$D$6),IF(AND($L37&lt;&gt;"",$L37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$L37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$O37&lt;&gt;"",Pronostici!$P37&lt;&gt;"",Pronostici!$O37=Partite!$G37,Pronostici!$P37=Partite!$H37),Config!$D$6,IF(AND($M37&lt;&gt;"",$M37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$O37&lt;&gt;"",Pronostici!$P37&lt;&gt;"",Pronostici!$O37=Partite!$G37,Pronostici!$P37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$S37)=1),Config!$D$9,Config!$D$6),IF(AND($M37&lt;&gt;"",$M37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$M37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H37" s="27">
-        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$R37&lt;&gt;"",Pronostici!$S37&lt;&gt;"",Pronostici!$R37=Partite!$G37,Pronostici!$S37=Partite!$H37),Config!$D$6,IF(AND($N37&lt;&gt;"",$N37=Partite!$I37),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K37&lt;&gt;"Giocata","",IF(AND(Pronostici!$R37&lt;&gt;"",Pronostici!$S37&lt;&gt;"",Pronostici!$R37=Partite!$G37,Pronostici!$S37=Partite!$H37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($P37:$T37,$T37)=1),Config!$D$9,Config!$D$6),IF(AND($N37&lt;&gt;"",$N37=Partite!$I37),IF(AND($B37&gt;=Config!$D$17,COUNTIF($J37:$N37,$N37)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J37" s="63">
@@ -9834,6 +10539,26 @@
       </c>
       <c r="N37" s="63">
         <f>IF(Pronostici!$Q37&lt;&gt;"",UPPER(Pronostici!$Q37),IF(OR(Pronostici!$R37="",Pronostici!$S37=""),"",IF(Pronostici!$R37&gt;Pronostici!$S37,"1",IF(Pronostici!$R37=Pronostici!$S37,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P37" s="63">
+        <f>IF(OR(Pronostici!$F37="",Pronostici!$G37=""),"",Pronostici!$F37&amp;" a "&amp;Pronostici!$G37)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="63">
+        <f>IF(OR(Pronostici!$I37="",Pronostici!$J37=""),"",Pronostici!$I37&amp;" a "&amp;Pronostici!$J37)</f>
+        <v/>
+      </c>
+      <c r="R37" s="63">
+        <f>IF(OR(Pronostici!$L37="",Pronostici!$M37=""),"",Pronostici!$L37&amp;" a "&amp;Pronostici!$M37)</f>
+        <v/>
+      </c>
+      <c r="S37" s="63">
+        <f>IF(OR(Pronostici!$O37="",Pronostici!$P37=""),"",Pronostici!$O37&amp;" a "&amp;Pronostici!$P37)</f>
+        <v/>
+      </c>
+      <c r="T37" s="63">
+        <f>IF(OR(Pronostici!$R37="",Pronostici!$S37=""),"",Pronostici!$R37&amp;" a "&amp;Pronostici!$S37)</f>
         <v/>
       </c>
     </row>
@@ -9851,23 +10576,23 @@
         <v/>
       </c>
       <c r="D38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$F38&lt;&gt;"",Pronostici!$G38&lt;&gt;"",Pronostici!$F38=Partite!$G38,Pronostici!$G38=Partite!$H38),Config!$D$6,IF(AND($J38&lt;&gt;"",$J38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$F38&lt;&gt;"",Pronostici!$G38&lt;&gt;"",Pronostici!$F38=Partite!$G38,Pronostici!$G38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$P38)=1),Config!$D$9,Config!$D$6),IF(AND($J38&lt;&gt;"",$J38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$J38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$I38&lt;&gt;"",Pronostici!$J38&lt;&gt;"",Pronostici!$I38=Partite!$G38,Pronostici!$J38=Partite!$H38),Config!$D$6,IF(AND($K38&lt;&gt;"",$K38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$I38&lt;&gt;"",Pronostici!$J38&lt;&gt;"",Pronostici!$I38=Partite!$G38,Pronostici!$J38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$Q38)=1),Config!$D$9,Config!$D$6),IF(AND($K38&lt;&gt;"",$K38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$K38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$L38&lt;&gt;"",Pronostici!$M38&lt;&gt;"",Pronostici!$L38=Partite!$G38,Pronostici!$M38=Partite!$H38),Config!$D$6,IF(AND($L38&lt;&gt;"",$L38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$L38&lt;&gt;"",Pronostici!$M38&lt;&gt;"",Pronostici!$L38=Partite!$G38,Pronostici!$M38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$R38)=1),Config!$D$9,Config!$D$6),IF(AND($L38&lt;&gt;"",$L38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$L38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$O38&lt;&gt;"",Pronostici!$P38&lt;&gt;"",Pronostici!$O38=Partite!$G38,Pronostici!$P38=Partite!$H38),Config!$D$6,IF(AND($M38&lt;&gt;"",$M38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$O38&lt;&gt;"",Pronostici!$P38&lt;&gt;"",Pronostici!$O38=Partite!$G38,Pronostici!$P38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$S38)=1),Config!$D$9,Config!$D$6),IF(AND($M38&lt;&gt;"",$M38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$M38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H38" s="27">
-        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$R38&lt;&gt;"",Pronostici!$S38&lt;&gt;"",Pronostici!$R38=Partite!$G38,Pronostici!$S38=Partite!$H38),Config!$D$6,IF(AND($N38&lt;&gt;"",$N38=Partite!$I38),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K38&lt;&gt;"Giocata","",IF(AND(Pronostici!$R38&lt;&gt;"",Pronostici!$S38&lt;&gt;"",Pronostici!$R38=Partite!$G38,Pronostici!$S38=Partite!$H38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($P38:$T38,$T38)=1),Config!$D$9,Config!$D$6),IF(AND($N38&lt;&gt;"",$N38=Partite!$I38),IF(AND($B38&gt;=Config!$D$17,COUNTIF($J38:$N38,$N38)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J38" s="63">
@@ -9888,6 +10613,26 @@
       </c>
       <c r="N38" s="63">
         <f>IF(Pronostici!$Q38&lt;&gt;"",UPPER(Pronostici!$Q38),IF(OR(Pronostici!$R38="",Pronostici!$S38=""),"",IF(Pronostici!$R38&gt;Pronostici!$S38,"1",IF(Pronostici!$R38=Pronostici!$S38,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P38" s="63">
+        <f>IF(OR(Pronostici!$F38="",Pronostici!$G38=""),"",Pronostici!$F38&amp;" a "&amp;Pronostici!$G38)</f>
+        <v/>
+      </c>
+      <c r="Q38" s="63">
+        <f>IF(OR(Pronostici!$I38="",Pronostici!$J38=""),"",Pronostici!$I38&amp;" a "&amp;Pronostici!$J38)</f>
+        <v/>
+      </c>
+      <c r="R38" s="63">
+        <f>IF(OR(Pronostici!$L38="",Pronostici!$M38=""),"",Pronostici!$L38&amp;" a "&amp;Pronostici!$M38)</f>
+        <v/>
+      </c>
+      <c r="S38" s="63">
+        <f>IF(OR(Pronostici!$O38="",Pronostici!$P38=""),"",Pronostici!$O38&amp;" a "&amp;Pronostici!$P38)</f>
+        <v/>
+      </c>
+      <c r="T38" s="63">
+        <f>IF(OR(Pronostici!$R38="",Pronostici!$S38=""),"",Pronostici!$R38&amp;" a "&amp;Pronostici!$S38)</f>
         <v/>
       </c>
     </row>
@@ -9905,23 +10650,23 @@
         <v/>
       </c>
       <c r="D39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$F39&lt;&gt;"",Pronostici!$G39&lt;&gt;"",Pronostici!$F39=Partite!$G39,Pronostici!$G39=Partite!$H39),Config!$D$6,IF(AND($J39&lt;&gt;"",$J39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$F39&lt;&gt;"",Pronostici!$G39&lt;&gt;"",Pronostici!$F39=Partite!$G39,Pronostici!$G39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$P39)=1),Config!$D$9,Config!$D$6),IF(AND($J39&lt;&gt;"",$J39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$J39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$I39&lt;&gt;"",Pronostici!$J39&lt;&gt;"",Pronostici!$I39=Partite!$G39,Pronostici!$J39=Partite!$H39),Config!$D$6,IF(AND($K39&lt;&gt;"",$K39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$I39&lt;&gt;"",Pronostici!$J39&lt;&gt;"",Pronostici!$I39=Partite!$G39,Pronostici!$J39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$Q39)=1),Config!$D$9,Config!$D$6),IF(AND($K39&lt;&gt;"",$K39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$K39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$L39&lt;&gt;"",Pronostici!$M39&lt;&gt;"",Pronostici!$L39=Partite!$G39,Pronostici!$M39=Partite!$H39),Config!$D$6,IF(AND($L39&lt;&gt;"",$L39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$L39&lt;&gt;"",Pronostici!$M39&lt;&gt;"",Pronostici!$L39=Partite!$G39,Pronostici!$M39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$R39)=1),Config!$D$9,Config!$D$6),IF(AND($L39&lt;&gt;"",$L39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$L39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$O39&lt;&gt;"",Pronostici!$P39&lt;&gt;"",Pronostici!$O39=Partite!$G39,Pronostici!$P39=Partite!$H39),Config!$D$6,IF(AND($M39&lt;&gt;"",$M39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$O39&lt;&gt;"",Pronostici!$P39&lt;&gt;"",Pronostici!$O39=Partite!$G39,Pronostici!$P39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$S39)=1),Config!$D$9,Config!$D$6),IF(AND($M39&lt;&gt;"",$M39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$M39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H39" s="27">
-        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$R39&lt;&gt;"",Pronostici!$S39&lt;&gt;"",Pronostici!$R39=Partite!$G39,Pronostici!$S39=Partite!$H39),Config!$D$6,IF(AND($N39&lt;&gt;"",$N39=Partite!$I39),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K39&lt;&gt;"Giocata","",IF(AND(Pronostici!$R39&lt;&gt;"",Pronostici!$S39&lt;&gt;"",Pronostici!$R39=Partite!$G39,Pronostici!$S39=Partite!$H39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($P39:$T39,$T39)=1),Config!$D$9,Config!$D$6),IF(AND($N39&lt;&gt;"",$N39=Partite!$I39),IF(AND($B39&gt;=Config!$D$17,COUNTIF($J39:$N39,$N39)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J39" s="63">
@@ -9942,6 +10687,26 @@
       </c>
       <c r="N39" s="63">
         <f>IF(Pronostici!$Q39&lt;&gt;"",UPPER(Pronostici!$Q39),IF(OR(Pronostici!$R39="",Pronostici!$S39=""),"",IF(Pronostici!$R39&gt;Pronostici!$S39,"1",IF(Pronostici!$R39=Pronostici!$S39,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P39" s="63">
+        <f>IF(OR(Pronostici!$F39="",Pronostici!$G39=""),"",Pronostici!$F39&amp;" a "&amp;Pronostici!$G39)</f>
+        <v/>
+      </c>
+      <c r="Q39" s="63">
+        <f>IF(OR(Pronostici!$I39="",Pronostici!$J39=""),"",Pronostici!$I39&amp;" a "&amp;Pronostici!$J39)</f>
+        <v/>
+      </c>
+      <c r="R39" s="63">
+        <f>IF(OR(Pronostici!$L39="",Pronostici!$M39=""),"",Pronostici!$L39&amp;" a "&amp;Pronostici!$M39)</f>
+        <v/>
+      </c>
+      <c r="S39" s="63">
+        <f>IF(OR(Pronostici!$O39="",Pronostici!$P39=""),"",Pronostici!$O39&amp;" a "&amp;Pronostici!$P39)</f>
+        <v/>
+      </c>
+      <c r="T39" s="63">
+        <f>IF(OR(Pronostici!$R39="",Pronostici!$S39=""),"",Pronostici!$R39&amp;" a "&amp;Pronostici!$S39)</f>
         <v/>
       </c>
     </row>
@@ -9959,23 +10724,23 @@
         <v/>
       </c>
       <c r="D40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$F40&lt;&gt;"",Pronostici!$G40&lt;&gt;"",Pronostici!$F40=Partite!$G40,Pronostici!$G40=Partite!$H40),Config!$D$6,IF(AND($J40&lt;&gt;"",$J40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$F40&lt;&gt;"",Pronostici!$G40&lt;&gt;"",Pronostici!$F40=Partite!$G40,Pronostici!$G40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$P40)=1),Config!$D$9,Config!$D$6),IF(AND($J40&lt;&gt;"",$J40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$J40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$I40&lt;&gt;"",Pronostici!$J40&lt;&gt;"",Pronostici!$I40=Partite!$G40,Pronostici!$J40=Partite!$H40),Config!$D$6,IF(AND($K40&lt;&gt;"",$K40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$I40&lt;&gt;"",Pronostici!$J40&lt;&gt;"",Pronostici!$I40=Partite!$G40,Pronostici!$J40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$Q40)=1),Config!$D$9,Config!$D$6),IF(AND($K40&lt;&gt;"",$K40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$K40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$L40&lt;&gt;"",Pronostici!$M40&lt;&gt;"",Pronostici!$L40=Partite!$G40,Pronostici!$M40=Partite!$H40),Config!$D$6,IF(AND($L40&lt;&gt;"",$L40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$L40&lt;&gt;"",Pronostici!$M40&lt;&gt;"",Pronostici!$L40=Partite!$G40,Pronostici!$M40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$R40)=1),Config!$D$9,Config!$D$6),IF(AND($L40&lt;&gt;"",$L40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$L40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$O40&lt;&gt;"",Pronostici!$P40&lt;&gt;"",Pronostici!$O40=Partite!$G40,Pronostici!$P40=Partite!$H40),Config!$D$6,IF(AND($M40&lt;&gt;"",$M40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$O40&lt;&gt;"",Pronostici!$P40&lt;&gt;"",Pronostici!$O40=Partite!$G40,Pronostici!$P40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$S40)=1),Config!$D$9,Config!$D$6),IF(AND($M40&lt;&gt;"",$M40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$M40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H40" s="27">
-        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$R40&lt;&gt;"",Pronostici!$S40&lt;&gt;"",Pronostici!$R40=Partite!$G40,Pronostici!$S40=Partite!$H40),Config!$D$6,IF(AND($N40&lt;&gt;"",$N40=Partite!$I40),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K40&lt;&gt;"Giocata","",IF(AND(Pronostici!$R40&lt;&gt;"",Pronostici!$S40&lt;&gt;"",Pronostici!$R40=Partite!$G40,Pronostici!$S40=Partite!$H40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($P40:$T40,$T40)=1),Config!$D$9,Config!$D$6),IF(AND($N40&lt;&gt;"",$N40=Partite!$I40),IF(AND($B40&gt;=Config!$D$17,COUNTIF($J40:$N40,$N40)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J40" s="63">
@@ -9996,6 +10761,26 @@
       </c>
       <c r="N40" s="63">
         <f>IF(Pronostici!$Q40&lt;&gt;"",UPPER(Pronostici!$Q40),IF(OR(Pronostici!$R40="",Pronostici!$S40=""),"",IF(Pronostici!$R40&gt;Pronostici!$S40,"1",IF(Pronostici!$R40=Pronostici!$S40,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P40" s="63">
+        <f>IF(OR(Pronostici!$F40="",Pronostici!$G40=""),"",Pronostici!$F40&amp;" a "&amp;Pronostici!$G40)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="63">
+        <f>IF(OR(Pronostici!$I40="",Pronostici!$J40=""),"",Pronostici!$I40&amp;" a "&amp;Pronostici!$J40)</f>
+        <v/>
+      </c>
+      <c r="R40" s="63">
+        <f>IF(OR(Pronostici!$L40="",Pronostici!$M40=""),"",Pronostici!$L40&amp;" a "&amp;Pronostici!$M40)</f>
+        <v/>
+      </c>
+      <c r="S40" s="63">
+        <f>IF(OR(Pronostici!$O40="",Pronostici!$P40=""),"",Pronostici!$O40&amp;" a "&amp;Pronostici!$P40)</f>
+        <v/>
+      </c>
+      <c r="T40" s="63">
+        <f>IF(OR(Pronostici!$R40="",Pronostici!$S40=""),"",Pronostici!$R40&amp;" a "&amp;Pronostici!$S40)</f>
         <v/>
       </c>
     </row>
@@ -10013,23 +10798,23 @@
         <v/>
       </c>
       <c r="D41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$F41&lt;&gt;"",Pronostici!$G41&lt;&gt;"",Pronostici!$F41=Partite!$G41,Pronostici!$G41=Partite!$H41),Config!$D$6,IF(AND($J41&lt;&gt;"",$J41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$F41&lt;&gt;"",Pronostici!$G41&lt;&gt;"",Pronostici!$F41=Partite!$G41,Pronostici!$G41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$P41)=1),Config!$D$9,Config!$D$6),IF(AND($J41&lt;&gt;"",$J41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$J41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$I41&lt;&gt;"",Pronostici!$J41&lt;&gt;"",Pronostici!$I41=Partite!$G41,Pronostici!$J41=Partite!$H41),Config!$D$6,IF(AND($K41&lt;&gt;"",$K41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$I41&lt;&gt;"",Pronostici!$J41&lt;&gt;"",Pronostici!$I41=Partite!$G41,Pronostici!$J41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$Q41)=1),Config!$D$9,Config!$D$6),IF(AND($K41&lt;&gt;"",$K41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$K41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$L41&lt;&gt;"",Pronostici!$M41&lt;&gt;"",Pronostici!$L41=Partite!$G41,Pronostici!$M41=Partite!$H41),Config!$D$6,IF(AND($L41&lt;&gt;"",$L41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$L41&lt;&gt;"",Pronostici!$M41&lt;&gt;"",Pronostici!$L41=Partite!$G41,Pronostici!$M41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$R41)=1),Config!$D$9,Config!$D$6),IF(AND($L41&lt;&gt;"",$L41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$L41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$O41&lt;&gt;"",Pronostici!$P41&lt;&gt;"",Pronostici!$O41=Partite!$G41,Pronostici!$P41=Partite!$H41),Config!$D$6,IF(AND($M41&lt;&gt;"",$M41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$O41&lt;&gt;"",Pronostici!$P41&lt;&gt;"",Pronostici!$O41=Partite!$G41,Pronostici!$P41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$S41)=1),Config!$D$9,Config!$D$6),IF(AND($M41&lt;&gt;"",$M41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$M41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H41" s="27">
-        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$R41&lt;&gt;"",Pronostici!$S41&lt;&gt;"",Pronostici!$R41=Partite!$G41,Pronostici!$S41=Partite!$H41),Config!$D$6,IF(AND($N41&lt;&gt;"",$N41=Partite!$I41),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K41&lt;&gt;"Giocata","",IF(AND(Pronostici!$R41&lt;&gt;"",Pronostici!$S41&lt;&gt;"",Pronostici!$R41=Partite!$G41,Pronostici!$S41=Partite!$H41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($P41:$T41,$T41)=1),Config!$D$9,Config!$D$6),IF(AND($N41&lt;&gt;"",$N41=Partite!$I41),IF(AND($B41&gt;=Config!$D$17,COUNTIF($J41:$N41,$N41)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J41" s="63">
@@ -10050,6 +10835,26 @@
       </c>
       <c r="N41" s="63">
         <f>IF(Pronostici!$Q41&lt;&gt;"",UPPER(Pronostici!$Q41),IF(OR(Pronostici!$R41="",Pronostici!$S41=""),"",IF(Pronostici!$R41&gt;Pronostici!$S41,"1",IF(Pronostici!$R41=Pronostici!$S41,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P41" s="63">
+        <f>IF(OR(Pronostici!$F41="",Pronostici!$G41=""),"",Pronostici!$F41&amp;" a "&amp;Pronostici!$G41)</f>
+        <v/>
+      </c>
+      <c r="Q41" s="63">
+        <f>IF(OR(Pronostici!$I41="",Pronostici!$J41=""),"",Pronostici!$I41&amp;" a "&amp;Pronostici!$J41)</f>
+        <v/>
+      </c>
+      <c r="R41" s="63">
+        <f>IF(OR(Pronostici!$L41="",Pronostici!$M41=""),"",Pronostici!$L41&amp;" a "&amp;Pronostici!$M41)</f>
+        <v/>
+      </c>
+      <c r="S41" s="63">
+        <f>IF(OR(Pronostici!$O41="",Pronostici!$P41=""),"",Pronostici!$O41&amp;" a "&amp;Pronostici!$P41)</f>
+        <v/>
+      </c>
+      <c r="T41" s="63">
+        <f>IF(OR(Pronostici!$R41="",Pronostici!$S41=""),"",Pronostici!$R41&amp;" a "&amp;Pronostici!$S41)</f>
         <v/>
       </c>
     </row>
@@ -10067,23 +10872,23 @@
         <v/>
       </c>
       <c r="D42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$F42&lt;&gt;"",Pronostici!$G42&lt;&gt;"",Pronostici!$F42=Partite!$G42,Pronostici!$G42=Partite!$H42),Config!$D$6,IF(AND($J42&lt;&gt;"",$J42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$F42&lt;&gt;"",Pronostici!$G42&lt;&gt;"",Pronostici!$F42=Partite!$G42,Pronostici!$G42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$P42)=1),Config!$D$9,Config!$D$6),IF(AND($J42&lt;&gt;"",$J42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$J42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$I42&lt;&gt;"",Pronostici!$J42&lt;&gt;"",Pronostici!$I42=Partite!$G42,Pronostici!$J42=Partite!$H42),Config!$D$6,IF(AND($K42&lt;&gt;"",$K42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$I42&lt;&gt;"",Pronostici!$J42&lt;&gt;"",Pronostici!$I42=Partite!$G42,Pronostici!$J42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$Q42)=1),Config!$D$9,Config!$D$6),IF(AND($K42&lt;&gt;"",$K42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$K42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$L42&lt;&gt;"",Pronostici!$M42&lt;&gt;"",Pronostici!$L42=Partite!$G42,Pronostici!$M42=Partite!$H42),Config!$D$6,IF(AND($L42&lt;&gt;"",$L42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$L42&lt;&gt;"",Pronostici!$M42&lt;&gt;"",Pronostici!$L42=Partite!$G42,Pronostici!$M42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$R42)=1),Config!$D$9,Config!$D$6),IF(AND($L42&lt;&gt;"",$L42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$L42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$O42&lt;&gt;"",Pronostici!$P42&lt;&gt;"",Pronostici!$O42=Partite!$G42,Pronostici!$P42=Partite!$H42),Config!$D$6,IF(AND($M42&lt;&gt;"",$M42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$O42&lt;&gt;"",Pronostici!$P42&lt;&gt;"",Pronostici!$O42=Partite!$G42,Pronostici!$P42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$S42)=1),Config!$D$9,Config!$D$6),IF(AND($M42&lt;&gt;"",$M42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$M42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H42" s="27">
-        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$R42&lt;&gt;"",Pronostici!$S42&lt;&gt;"",Pronostici!$R42=Partite!$G42,Pronostici!$S42=Partite!$H42),Config!$D$6,IF(AND($N42&lt;&gt;"",$N42=Partite!$I42),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K42&lt;&gt;"Giocata","",IF(AND(Pronostici!$R42&lt;&gt;"",Pronostici!$S42&lt;&gt;"",Pronostici!$R42=Partite!$G42,Pronostici!$S42=Partite!$H42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($P42:$T42,$T42)=1),Config!$D$9,Config!$D$6),IF(AND($N42&lt;&gt;"",$N42=Partite!$I42),IF(AND($B42&gt;=Config!$D$17,COUNTIF($J42:$N42,$N42)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J42" s="63">
@@ -10104,6 +10909,26 @@
       </c>
       <c r="N42" s="63">
         <f>IF(Pronostici!$Q42&lt;&gt;"",UPPER(Pronostici!$Q42),IF(OR(Pronostici!$R42="",Pronostici!$S42=""),"",IF(Pronostici!$R42&gt;Pronostici!$S42,"1",IF(Pronostici!$R42=Pronostici!$S42,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P42" s="63">
+        <f>IF(OR(Pronostici!$F42="",Pronostici!$G42=""),"",Pronostici!$F42&amp;" a "&amp;Pronostici!$G42)</f>
+        <v/>
+      </c>
+      <c r="Q42" s="63">
+        <f>IF(OR(Pronostici!$I42="",Pronostici!$J42=""),"",Pronostici!$I42&amp;" a "&amp;Pronostici!$J42)</f>
+        <v/>
+      </c>
+      <c r="R42" s="63">
+        <f>IF(OR(Pronostici!$L42="",Pronostici!$M42=""),"",Pronostici!$L42&amp;" a "&amp;Pronostici!$M42)</f>
+        <v/>
+      </c>
+      <c r="S42" s="63">
+        <f>IF(OR(Pronostici!$O42="",Pronostici!$P42=""),"",Pronostici!$O42&amp;" a "&amp;Pronostici!$P42)</f>
+        <v/>
+      </c>
+      <c r="T42" s="63">
+        <f>IF(OR(Pronostici!$R42="",Pronostici!$S42=""),"",Pronostici!$R42&amp;" a "&amp;Pronostici!$S42)</f>
         <v/>
       </c>
     </row>
@@ -10121,23 +10946,23 @@
         <v/>
       </c>
       <c r="D43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$F43&lt;&gt;"",Pronostici!$G43&lt;&gt;"",Pronostici!$F43=Partite!$G43,Pronostici!$G43=Partite!$H43),Config!$D$6,IF(AND($J43&lt;&gt;"",$J43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$F43&lt;&gt;"",Pronostici!$G43&lt;&gt;"",Pronostici!$F43=Partite!$G43,Pronostici!$G43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$P43)=1),Config!$D$9,Config!$D$6),IF(AND($J43&lt;&gt;"",$J43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$J43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$I43&lt;&gt;"",Pronostici!$J43&lt;&gt;"",Pronostici!$I43=Partite!$G43,Pronostici!$J43=Partite!$H43),Config!$D$6,IF(AND($K43&lt;&gt;"",$K43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$I43&lt;&gt;"",Pronostici!$J43&lt;&gt;"",Pronostici!$I43=Partite!$G43,Pronostici!$J43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$Q43)=1),Config!$D$9,Config!$D$6),IF(AND($K43&lt;&gt;"",$K43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$K43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$L43&lt;&gt;"",Pronostici!$M43&lt;&gt;"",Pronostici!$L43=Partite!$G43,Pronostici!$M43=Partite!$H43),Config!$D$6,IF(AND($L43&lt;&gt;"",$L43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$L43&lt;&gt;"",Pronostici!$M43&lt;&gt;"",Pronostici!$L43=Partite!$G43,Pronostici!$M43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$R43)=1),Config!$D$9,Config!$D$6),IF(AND($L43&lt;&gt;"",$L43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$L43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$O43&lt;&gt;"",Pronostici!$P43&lt;&gt;"",Pronostici!$O43=Partite!$G43,Pronostici!$P43=Partite!$H43),Config!$D$6,IF(AND($M43&lt;&gt;"",$M43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$O43&lt;&gt;"",Pronostici!$P43&lt;&gt;"",Pronostici!$O43=Partite!$G43,Pronostici!$P43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$S43)=1),Config!$D$9,Config!$D$6),IF(AND($M43&lt;&gt;"",$M43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$M43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H43" s="22">
-        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$R43&lt;&gt;"",Pronostici!$S43&lt;&gt;"",Pronostici!$R43=Partite!$G43,Pronostici!$S43=Partite!$H43),Config!$D$6,IF(AND($N43&lt;&gt;"",$N43=Partite!$I43),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K43&lt;&gt;"Giocata","",IF(AND(Pronostici!$R43&lt;&gt;"",Pronostici!$S43&lt;&gt;"",Pronostici!$R43=Partite!$G43,Pronostici!$S43=Partite!$H43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($P43:$T43,$T43)=1),Config!$D$9,Config!$D$6),IF(AND($N43&lt;&gt;"",$N43=Partite!$I43),IF(AND($B43&gt;=Config!$D$17,COUNTIF($J43:$N43,$N43)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J43" s="63">
@@ -10158,6 +10983,26 @@
       </c>
       <c r="N43" s="63">
         <f>IF(Pronostici!$Q43&lt;&gt;"",UPPER(Pronostici!$Q43),IF(OR(Pronostici!$R43="",Pronostici!$S43=""),"",IF(Pronostici!$R43&gt;Pronostici!$S43,"1",IF(Pronostici!$R43=Pronostici!$S43,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P43" s="63">
+        <f>IF(OR(Pronostici!$F43="",Pronostici!$G43=""),"",Pronostici!$F43&amp;" a "&amp;Pronostici!$G43)</f>
+        <v/>
+      </c>
+      <c r="Q43" s="63">
+        <f>IF(OR(Pronostici!$I43="",Pronostici!$J43=""),"",Pronostici!$I43&amp;" a "&amp;Pronostici!$J43)</f>
+        <v/>
+      </c>
+      <c r="R43" s="63">
+        <f>IF(OR(Pronostici!$L43="",Pronostici!$M43=""),"",Pronostici!$L43&amp;" a "&amp;Pronostici!$M43)</f>
+        <v/>
+      </c>
+      <c r="S43" s="63">
+        <f>IF(OR(Pronostici!$O43="",Pronostici!$P43=""),"",Pronostici!$O43&amp;" a "&amp;Pronostici!$P43)</f>
+        <v/>
+      </c>
+      <c r="T43" s="63">
+        <f>IF(OR(Pronostici!$R43="",Pronostici!$S43=""),"",Pronostici!$R43&amp;" a "&amp;Pronostici!$S43)</f>
         <v/>
       </c>
     </row>
@@ -10175,23 +11020,23 @@
         <v/>
       </c>
       <c r="D44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$F44&lt;&gt;"",Pronostici!$G44&lt;&gt;"",Pronostici!$F44=Partite!$G44,Pronostici!$G44=Partite!$H44),Config!$D$6,IF(AND($J44&lt;&gt;"",$J44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$F44&lt;&gt;"",Pronostici!$G44&lt;&gt;"",Pronostici!$F44=Partite!$G44,Pronostici!$G44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$P44)=1),Config!$D$9,Config!$D$6),IF(AND($J44&lt;&gt;"",$J44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$J44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$I44&lt;&gt;"",Pronostici!$J44&lt;&gt;"",Pronostici!$I44=Partite!$G44,Pronostici!$J44=Partite!$H44),Config!$D$6,IF(AND($K44&lt;&gt;"",$K44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$I44&lt;&gt;"",Pronostici!$J44&lt;&gt;"",Pronostici!$I44=Partite!$G44,Pronostici!$J44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$Q44)=1),Config!$D$9,Config!$D$6),IF(AND($K44&lt;&gt;"",$K44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$K44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$L44&lt;&gt;"",Pronostici!$M44&lt;&gt;"",Pronostici!$L44=Partite!$G44,Pronostici!$M44=Partite!$H44),Config!$D$6,IF(AND($L44&lt;&gt;"",$L44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$L44&lt;&gt;"",Pronostici!$M44&lt;&gt;"",Pronostici!$L44=Partite!$G44,Pronostici!$M44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$R44)=1),Config!$D$9,Config!$D$6),IF(AND($L44&lt;&gt;"",$L44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$L44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$O44&lt;&gt;"",Pronostici!$P44&lt;&gt;"",Pronostici!$O44=Partite!$G44,Pronostici!$P44=Partite!$H44),Config!$D$6,IF(AND($M44&lt;&gt;"",$M44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$O44&lt;&gt;"",Pronostici!$P44&lt;&gt;"",Pronostici!$O44=Partite!$G44,Pronostici!$P44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$S44)=1),Config!$D$9,Config!$D$6),IF(AND($M44&lt;&gt;"",$M44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$M44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H44" s="22">
-        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$R44&lt;&gt;"",Pronostici!$S44&lt;&gt;"",Pronostici!$R44=Partite!$G44,Pronostici!$S44=Partite!$H44),Config!$D$6,IF(AND($N44&lt;&gt;"",$N44=Partite!$I44),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K44&lt;&gt;"Giocata","",IF(AND(Pronostici!$R44&lt;&gt;"",Pronostici!$S44&lt;&gt;"",Pronostici!$R44=Partite!$G44,Pronostici!$S44=Partite!$H44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($P44:$T44,$T44)=1),Config!$D$9,Config!$D$6),IF(AND($N44&lt;&gt;"",$N44=Partite!$I44),IF(AND($B44&gt;=Config!$D$17,COUNTIF($J44:$N44,$N44)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J44" s="63">
@@ -10212,6 +11057,26 @@
       </c>
       <c r="N44" s="63">
         <f>IF(Pronostici!$Q44&lt;&gt;"",UPPER(Pronostici!$Q44),IF(OR(Pronostici!$R44="",Pronostici!$S44=""),"",IF(Pronostici!$R44&gt;Pronostici!$S44,"1",IF(Pronostici!$R44=Pronostici!$S44,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P44" s="63">
+        <f>IF(OR(Pronostici!$F44="",Pronostici!$G44=""),"",Pronostici!$F44&amp;" a "&amp;Pronostici!$G44)</f>
+        <v/>
+      </c>
+      <c r="Q44" s="63">
+        <f>IF(OR(Pronostici!$I44="",Pronostici!$J44=""),"",Pronostici!$I44&amp;" a "&amp;Pronostici!$J44)</f>
+        <v/>
+      </c>
+      <c r="R44" s="63">
+        <f>IF(OR(Pronostici!$L44="",Pronostici!$M44=""),"",Pronostici!$L44&amp;" a "&amp;Pronostici!$M44)</f>
+        <v/>
+      </c>
+      <c r="S44" s="63">
+        <f>IF(OR(Pronostici!$O44="",Pronostici!$P44=""),"",Pronostici!$O44&amp;" a "&amp;Pronostici!$P44)</f>
+        <v/>
+      </c>
+      <c r="T44" s="63">
+        <f>IF(OR(Pronostici!$R44="",Pronostici!$S44=""),"",Pronostici!$R44&amp;" a "&amp;Pronostici!$S44)</f>
         <v/>
       </c>
     </row>
@@ -10229,23 +11094,23 @@
         <v/>
       </c>
       <c r="D45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$F45&lt;&gt;"",Pronostici!$G45&lt;&gt;"",Pronostici!$F45=Partite!$G45,Pronostici!$G45=Partite!$H45),Config!$D$6,IF(AND($J45&lt;&gt;"",$J45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$F45&lt;&gt;"",Pronostici!$G45&lt;&gt;"",Pronostici!$F45=Partite!$G45,Pronostici!$G45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$P45)=1),Config!$D$9,Config!$D$6),IF(AND($J45&lt;&gt;"",$J45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$J45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$I45&lt;&gt;"",Pronostici!$J45&lt;&gt;"",Pronostici!$I45=Partite!$G45,Pronostici!$J45=Partite!$H45),Config!$D$6,IF(AND($K45&lt;&gt;"",$K45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$I45&lt;&gt;"",Pronostici!$J45&lt;&gt;"",Pronostici!$I45=Partite!$G45,Pronostici!$J45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$Q45)=1),Config!$D$9,Config!$D$6),IF(AND($K45&lt;&gt;"",$K45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$K45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$L45&lt;&gt;"",Pronostici!$M45&lt;&gt;"",Pronostici!$L45=Partite!$G45,Pronostici!$M45=Partite!$H45),Config!$D$6,IF(AND($L45&lt;&gt;"",$L45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$L45&lt;&gt;"",Pronostici!$M45&lt;&gt;"",Pronostici!$L45=Partite!$G45,Pronostici!$M45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$R45)=1),Config!$D$9,Config!$D$6),IF(AND($L45&lt;&gt;"",$L45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$L45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$O45&lt;&gt;"",Pronostici!$P45&lt;&gt;"",Pronostici!$O45=Partite!$G45,Pronostici!$P45=Partite!$H45),Config!$D$6,IF(AND($M45&lt;&gt;"",$M45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$O45&lt;&gt;"",Pronostici!$P45&lt;&gt;"",Pronostici!$O45=Partite!$G45,Pronostici!$P45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$S45)=1),Config!$D$9,Config!$D$6),IF(AND($M45&lt;&gt;"",$M45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$M45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H45" s="22">
-        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$R45&lt;&gt;"",Pronostici!$S45&lt;&gt;"",Pronostici!$R45=Partite!$G45,Pronostici!$S45=Partite!$H45),Config!$D$6,IF(AND($N45&lt;&gt;"",$N45=Partite!$I45),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K45&lt;&gt;"Giocata","",IF(AND(Pronostici!$R45&lt;&gt;"",Pronostici!$S45&lt;&gt;"",Pronostici!$R45=Partite!$G45,Pronostici!$S45=Partite!$H45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($P45:$T45,$T45)=1),Config!$D$9,Config!$D$6),IF(AND($N45&lt;&gt;"",$N45=Partite!$I45),IF(AND($B45&gt;=Config!$D$17,COUNTIF($J45:$N45,$N45)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J45" s="63">
@@ -10266,6 +11131,26 @@
       </c>
       <c r="N45" s="63">
         <f>IF(Pronostici!$Q45&lt;&gt;"",UPPER(Pronostici!$Q45),IF(OR(Pronostici!$R45="",Pronostici!$S45=""),"",IF(Pronostici!$R45&gt;Pronostici!$S45,"1",IF(Pronostici!$R45=Pronostici!$S45,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P45" s="63">
+        <f>IF(OR(Pronostici!$F45="",Pronostici!$G45=""),"",Pronostici!$F45&amp;" a "&amp;Pronostici!$G45)</f>
+        <v/>
+      </c>
+      <c r="Q45" s="63">
+        <f>IF(OR(Pronostici!$I45="",Pronostici!$J45=""),"",Pronostici!$I45&amp;" a "&amp;Pronostici!$J45)</f>
+        <v/>
+      </c>
+      <c r="R45" s="63">
+        <f>IF(OR(Pronostici!$L45="",Pronostici!$M45=""),"",Pronostici!$L45&amp;" a "&amp;Pronostici!$M45)</f>
+        <v/>
+      </c>
+      <c r="S45" s="63">
+        <f>IF(OR(Pronostici!$O45="",Pronostici!$P45=""),"",Pronostici!$O45&amp;" a "&amp;Pronostici!$P45)</f>
+        <v/>
+      </c>
+      <c r="T45" s="63">
+        <f>IF(OR(Pronostici!$R45="",Pronostici!$S45=""),"",Pronostici!$R45&amp;" a "&amp;Pronostici!$S45)</f>
         <v/>
       </c>
     </row>
@@ -10283,23 +11168,23 @@
         <v/>
       </c>
       <c r="D46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$F46&lt;&gt;"",Pronostici!$G46&lt;&gt;"",Pronostici!$F46=Partite!$G46,Pronostici!$G46=Partite!$H46),Config!$D$6,IF(AND($J46&lt;&gt;"",$J46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$F46&lt;&gt;"",Pronostici!$G46&lt;&gt;"",Pronostici!$F46=Partite!$G46,Pronostici!$G46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$P46)=1),Config!$D$9,Config!$D$6),IF(AND($J46&lt;&gt;"",$J46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$J46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$I46&lt;&gt;"",Pronostici!$J46&lt;&gt;"",Pronostici!$I46=Partite!$G46,Pronostici!$J46=Partite!$H46),Config!$D$6,IF(AND($K46&lt;&gt;"",$K46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$I46&lt;&gt;"",Pronostici!$J46&lt;&gt;"",Pronostici!$I46=Partite!$G46,Pronostici!$J46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$Q46)=1),Config!$D$9,Config!$D$6),IF(AND($K46&lt;&gt;"",$K46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$K46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$L46&lt;&gt;"",Pronostici!$M46&lt;&gt;"",Pronostici!$L46=Partite!$G46,Pronostici!$M46=Partite!$H46),Config!$D$6,IF(AND($L46&lt;&gt;"",$L46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$L46&lt;&gt;"",Pronostici!$M46&lt;&gt;"",Pronostici!$L46=Partite!$G46,Pronostici!$M46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$R46)=1),Config!$D$9,Config!$D$6),IF(AND($L46&lt;&gt;"",$L46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$L46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$O46&lt;&gt;"",Pronostici!$P46&lt;&gt;"",Pronostici!$O46=Partite!$G46,Pronostici!$P46=Partite!$H46),Config!$D$6,IF(AND($M46&lt;&gt;"",$M46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$O46&lt;&gt;"",Pronostici!$P46&lt;&gt;"",Pronostici!$O46=Partite!$G46,Pronostici!$P46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$S46)=1),Config!$D$9,Config!$D$6),IF(AND($M46&lt;&gt;"",$M46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$M46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H46" s="22">
-        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$R46&lt;&gt;"",Pronostici!$S46&lt;&gt;"",Pronostici!$R46=Partite!$G46,Pronostici!$S46=Partite!$H46),Config!$D$6,IF(AND($N46&lt;&gt;"",$N46=Partite!$I46),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K46&lt;&gt;"Giocata","",IF(AND(Pronostici!$R46&lt;&gt;"",Pronostici!$S46&lt;&gt;"",Pronostici!$R46=Partite!$G46,Pronostici!$S46=Partite!$H46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($P46:$T46,$T46)=1),Config!$D$9,Config!$D$6),IF(AND($N46&lt;&gt;"",$N46=Partite!$I46),IF(AND($B46&gt;=Config!$D$17,COUNTIF($J46:$N46,$N46)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J46" s="63">
@@ -10320,6 +11205,26 @@
       </c>
       <c r="N46" s="63">
         <f>IF(Pronostici!$Q46&lt;&gt;"",UPPER(Pronostici!$Q46),IF(OR(Pronostici!$R46="",Pronostici!$S46=""),"",IF(Pronostici!$R46&gt;Pronostici!$S46,"1",IF(Pronostici!$R46=Pronostici!$S46,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P46" s="63">
+        <f>IF(OR(Pronostici!$F46="",Pronostici!$G46=""),"",Pronostici!$F46&amp;" a "&amp;Pronostici!$G46)</f>
+        <v/>
+      </c>
+      <c r="Q46" s="63">
+        <f>IF(OR(Pronostici!$I46="",Pronostici!$J46=""),"",Pronostici!$I46&amp;" a "&amp;Pronostici!$J46)</f>
+        <v/>
+      </c>
+      <c r="R46" s="63">
+        <f>IF(OR(Pronostici!$L46="",Pronostici!$M46=""),"",Pronostici!$L46&amp;" a "&amp;Pronostici!$M46)</f>
+        <v/>
+      </c>
+      <c r="S46" s="63">
+        <f>IF(OR(Pronostici!$O46="",Pronostici!$P46=""),"",Pronostici!$O46&amp;" a "&amp;Pronostici!$P46)</f>
+        <v/>
+      </c>
+      <c r="T46" s="63">
+        <f>IF(OR(Pronostici!$R46="",Pronostici!$S46=""),"",Pronostici!$R46&amp;" a "&amp;Pronostici!$S46)</f>
         <v/>
       </c>
     </row>
@@ -10337,23 +11242,23 @@
         <v/>
       </c>
       <c r="D47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$F47&lt;&gt;"",Pronostici!$G47&lt;&gt;"",Pronostici!$F47=Partite!$G47,Pronostici!$G47=Partite!$H47),Config!$D$6,IF(AND($J47&lt;&gt;"",$J47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$F47&lt;&gt;"",Pronostici!$G47&lt;&gt;"",Pronostici!$F47=Partite!$G47,Pronostici!$G47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$P47)=1),Config!$D$9,Config!$D$6),IF(AND($J47&lt;&gt;"",$J47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$J47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$I47&lt;&gt;"",Pronostici!$J47&lt;&gt;"",Pronostici!$I47=Partite!$G47,Pronostici!$J47=Partite!$H47),Config!$D$6,IF(AND($K47&lt;&gt;"",$K47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$I47&lt;&gt;"",Pronostici!$J47&lt;&gt;"",Pronostici!$I47=Partite!$G47,Pronostici!$J47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$Q47)=1),Config!$D$9,Config!$D$6),IF(AND($K47&lt;&gt;"",$K47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$K47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$L47&lt;&gt;"",Pronostici!$M47&lt;&gt;"",Pronostici!$L47=Partite!$G47,Pronostici!$M47=Partite!$H47),Config!$D$6,IF(AND($L47&lt;&gt;"",$L47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$L47&lt;&gt;"",Pronostici!$M47&lt;&gt;"",Pronostici!$L47=Partite!$G47,Pronostici!$M47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$R47)=1),Config!$D$9,Config!$D$6),IF(AND($L47&lt;&gt;"",$L47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$L47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$O47&lt;&gt;"",Pronostici!$P47&lt;&gt;"",Pronostici!$O47=Partite!$G47,Pronostici!$P47=Partite!$H47),Config!$D$6,IF(AND($M47&lt;&gt;"",$M47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$O47&lt;&gt;"",Pronostici!$P47&lt;&gt;"",Pronostici!$O47=Partite!$G47,Pronostici!$P47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$S47)=1),Config!$D$9,Config!$D$6),IF(AND($M47&lt;&gt;"",$M47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$M47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H47" s="22">
-        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$R47&lt;&gt;"",Pronostici!$S47&lt;&gt;"",Pronostici!$R47=Partite!$G47,Pronostici!$S47=Partite!$H47),Config!$D$6,IF(AND($N47&lt;&gt;"",$N47=Partite!$I47),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K47&lt;&gt;"Giocata","",IF(AND(Pronostici!$R47&lt;&gt;"",Pronostici!$S47&lt;&gt;"",Pronostici!$R47=Partite!$G47,Pronostici!$S47=Partite!$H47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($P47:$T47,$T47)=1),Config!$D$9,Config!$D$6),IF(AND($N47&lt;&gt;"",$N47=Partite!$I47),IF(AND($B47&gt;=Config!$D$17,COUNTIF($J47:$N47,$N47)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J47" s="63">
@@ -10374,6 +11279,26 @@
       </c>
       <c r="N47" s="63">
         <f>IF(Pronostici!$Q47&lt;&gt;"",UPPER(Pronostici!$Q47),IF(OR(Pronostici!$R47="",Pronostici!$S47=""),"",IF(Pronostici!$R47&gt;Pronostici!$S47,"1",IF(Pronostici!$R47=Pronostici!$S47,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P47" s="63">
+        <f>IF(OR(Pronostici!$F47="",Pronostici!$G47=""),"",Pronostici!$F47&amp;" a "&amp;Pronostici!$G47)</f>
+        <v/>
+      </c>
+      <c r="Q47" s="63">
+        <f>IF(OR(Pronostici!$I47="",Pronostici!$J47=""),"",Pronostici!$I47&amp;" a "&amp;Pronostici!$J47)</f>
+        <v/>
+      </c>
+      <c r="R47" s="63">
+        <f>IF(OR(Pronostici!$L47="",Pronostici!$M47=""),"",Pronostici!$L47&amp;" a "&amp;Pronostici!$M47)</f>
+        <v/>
+      </c>
+      <c r="S47" s="63">
+        <f>IF(OR(Pronostici!$O47="",Pronostici!$P47=""),"",Pronostici!$O47&amp;" a "&amp;Pronostici!$P47)</f>
+        <v/>
+      </c>
+      <c r="T47" s="63">
+        <f>IF(OR(Pronostici!$R47="",Pronostici!$S47=""),"",Pronostici!$R47&amp;" a "&amp;Pronostici!$S47)</f>
         <v/>
       </c>
     </row>
@@ -10391,23 +11316,23 @@
         <v/>
       </c>
       <c r="D48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$F48&lt;&gt;"",Pronostici!$G48&lt;&gt;"",Pronostici!$F48=Partite!$G48,Pronostici!$G48=Partite!$H48),Config!$D$6,IF(AND($J48&lt;&gt;"",$J48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$F48&lt;&gt;"",Pronostici!$G48&lt;&gt;"",Pronostici!$F48=Partite!$G48,Pronostici!$G48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$P48)=1),Config!$D$9,Config!$D$6),IF(AND($J48&lt;&gt;"",$J48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$J48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$I48&lt;&gt;"",Pronostici!$J48&lt;&gt;"",Pronostici!$I48=Partite!$G48,Pronostici!$J48=Partite!$H48),Config!$D$6,IF(AND($K48&lt;&gt;"",$K48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$I48&lt;&gt;"",Pronostici!$J48&lt;&gt;"",Pronostici!$I48=Partite!$G48,Pronostici!$J48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$Q48)=1),Config!$D$9,Config!$D$6),IF(AND($K48&lt;&gt;"",$K48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$K48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$L48&lt;&gt;"",Pronostici!$M48&lt;&gt;"",Pronostici!$L48=Partite!$G48,Pronostici!$M48=Partite!$H48),Config!$D$6,IF(AND($L48&lt;&gt;"",$L48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$L48&lt;&gt;"",Pronostici!$M48&lt;&gt;"",Pronostici!$L48=Partite!$G48,Pronostici!$M48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$R48)=1),Config!$D$9,Config!$D$6),IF(AND($L48&lt;&gt;"",$L48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$L48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$O48&lt;&gt;"",Pronostici!$P48&lt;&gt;"",Pronostici!$O48=Partite!$G48,Pronostici!$P48=Partite!$H48),Config!$D$6,IF(AND($M48&lt;&gt;"",$M48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$O48&lt;&gt;"",Pronostici!$P48&lt;&gt;"",Pronostici!$O48=Partite!$G48,Pronostici!$P48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$S48)=1),Config!$D$9,Config!$D$6),IF(AND($M48&lt;&gt;"",$M48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$M48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H48" s="22">
-        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$R48&lt;&gt;"",Pronostici!$S48&lt;&gt;"",Pronostici!$R48=Partite!$G48,Pronostici!$S48=Partite!$H48),Config!$D$6,IF(AND($N48&lt;&gt;"",$N48=Partite!$I48),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K48&lt;&gt;"Giocata","",IF(AND(Pronostici!$R48&lt;&gt;"",Pronostici!$S48&lt;&gt;"",Pronostici!$R48=Partite!$G48,Pronostici!$S48=Partite!$H48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($P48:$T48,$T48)=1),Config!$D$9,Config!$D$6),IF(AND($N48&lt;&gt;"",$N48=Partite!$I48),IF(AND($B48&gt;=Config!$D$17,COUNTIF($J48:$N48,$N48)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J48" s="63">
@@ -10428,6 +11353,26 @@
       </c>
       <c r="N48" s="63">
         <f>IF(Pronostici!$Q48&lt;&gt;"",UPPER(Pronostici!$Q48),IF(OR(Pronostici!$R48="",Pronostici!$S48=""),"",IF(Pronostici!$R48&gt;Pronostici!$S48,"1",IF(Pronostici!$R48=Pronostici!$S48,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P48" s="63">
+        <f>IF(OR(Pronostici!$F48="",Pronostici!$G48=""),"",Pronostici!$F48&amp;" a "&amp;Pronostici!$G48)</f>
+        <v/>
+      </c>
+      <c r="Q48" s="63">
+        <f>IF(OR(Pronostici!$I48="",Pronostici!$J48=""),"",Pronostici!$I48&amp;" a "&amp;Pronostici!$J48)</f>
+        <v/>
+      </c>
+      <c r="R48" s="63">
+        <f>IF(OR(Pronostici!$L48="",Pronostici!$M48=""),"",Pronostici!$L48&amp;" a "&amp;Pronostici!$M48)</f>
+        <v/>
+      </c>
+      <c r="S48" s="63">
+        <f>IF(OR(Pronostici!$O48="",Pronostici!$P48=""),"",Pronostici!$O48&amp;" a "&amp;Pronostici!$P48)</f>
+        <v/>
+      </c>
+      <c r="T48" s="63">
+        <f>IF(OR(Pronostici!$R48="",Pronostici!$S48=""),"",Pronostici!$R48&amp;" a "&amp;Pronostici!$S48)</f>
         <v/>
       </c>
     </row>
@@ -10445,23 +11390,23 @@
         <v/>
       </c>
       <c r="D49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$F49&lt;&gt;"",Pronostici!$G49&lt;&gt;"",Pronostici!$F49=Partite!$G49,Pronostici!$G49=Partite!$H49),Config!$D$6,IF(AND($J49&lt;&gt;"",$J49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$F49&lt;&gt;"",Pronostici!$G49&lt;&gt;"",Pronostici!$F49=Partite!$G49,Pronostici!$G49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$P49)=1),Config!$D$9,Config!$D$6),IF(AND($J49&lt;&gt;"",$J49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$J49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$I49&lt;&gt;"",Pronostici!$J49&lt;&gt;"",Pronostici!$I49=Partite!$G49,Pronostici!$J49=Partite!$H49),Config!$D$6,IF(AND($K49&lt;&gt;"",$K49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$I49&lt;&gt;"",Pronostici!$J49&lt;&gt;"",Pronostici!$I49=Partite!$G49,Pronostici!$J49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$Q49)=1),Config!$D$9,Config!$D$6),IF(AND($K49&lt;&gt;"",$K49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$K49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$L49&lt;&gt;"",Pronostici!$M49&lt;&gt;"",Pronostici!$L49=Partite!$G49,Pronostici!$M49=Partite!$H49),Config!$D$6,IF(AND($L49&lt;&gt;"",$L49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$L49&lt;&gt;"",Pronostici!$M49&lt;&gt;"",Pronostici!$L49=Partite!$G49,Pronostici!$M49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$R49)=1),Config!$D$9,Config!$D$6),IF(AND($L49&lt;&gt;"",$L49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$L49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$O49&lt;&gt;"",Pronostici!$P49&lt;&gt;"",Pronostici!$O49=Partite!$G49,Pronostici!$P49=Partite!$H49),Config!$D$6,IF(AND($M49&lt;&gt;"",$M49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$O49&lt;&gt;"",Pronostici!$P49&lt;&gt;"",Pronostici!$O49=Partite!$G49,Pronostici!$P49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$S49)=1),Config!$D$9,Config!$D$6),IF(AND($M49&lt;&gt;"",$M49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$M49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H49" s="22">
-        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$R49&lt;&gt;"",Pronostici!$S49&lt;&gt;"",Pronostici!$R49=Partite!$G49,Pronostici!$S49=Partite!$H49),Config!$D$6,IF(AND($N49&lt;&gt;"",$N49=Partite!$I49),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K49&lt;&gt;"Giocata","",IF(AND(Pronostici!$R49&lt;&gt;"",Pronostici!$S49&lt;&gt;"",Pronostici!$R49=Partite!$G49,Pronostici!$S49=Partite!$H49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($P49:$T49,$T49)=1),Config!$D$9,Config!$D$6),IF(AND($N49&lt;&gt;"",$N49=Partite!$I49),IF(AND($B49&gt;=Config!$D$17,COUNTIF($J49:$N49,$N49)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J49" s="63">
@@ -10482,6 +11427,26 @@
       </c>
       <c r="N49" s="63">
         <f>IF(Pronostici!$Q49&lt;&gt;"",UPPER(Pronostici!$Q49),IF(OR(Pronostici!$R49="",Pronostici!$S49=""),"",IF(Pronostici!$R49&gt;Pronostici!$S49,"1",IF(Pronostici!$R49=Pronostici!$S49,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P49" s="63">
+        <f>IF(OR(Pronostici!$F49="",Pronostici!$G49=""),"",Pronostici!$F49&amp;" a "&amp;Pronostici!$G49)</f>
+        <v/>
+      </c>
+      <c r="Q49" s="63">
+        <f>IF(OR(Pronostici!$I49="",Pronostici!$J49=""),"",Pronostici!$I49&amp;" a "&amp;Pronostici!$J49)</f>
+        <v/>
+      </c>
+      <c r="R49" s="63">
+        <f>IF(OR(Pronostici!$L49="",Pronostici!$M49=""),"",Pronostici!$L49&amp;" a "&amp;Pronostici!$M49)</f>
+        <v/>
+      </c>
+      <c r="S49" s="63">
+        <f>IF(OR(Pronostici!$O49="",Pronostici!$P49=""),"",Pronostici!$O49&amp;" a "&amp;Pronostici!$P49)</f>
+        <v/>
+      </c>
+      <c r="T49" s="63">
+        <f>IF(OR(Pronostici!$R49="",Pronostici!$S49=""),"",Pronostici!$R49&amp;" a "&amp;Pronostici!$S49)</f>
         <v/>
       </c>
     </row>
@@ -10499,23 +11464,23 @@
         <v/>
       </c>
       <c r="D50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$F50&lt;&gt;"",Pronostici!$G50&lt;&gt;"",Pronostici!$F50=Partite!$G50,Pronostici!$G50=Partite!$H50),Config!$D$6,IF(AND($J50&lt;&gt;"",$J50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$F50&lt;&gt;"",Pronostici!$G50&lt;&gt;"",Pronostici!$F50=Partite!$G50,Pronostici!$G50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$P50)=1),Config!$D$9,Config!$D$6),IF(AND($J50&lt;&gt;"",$J50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$J50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$I50&lt;&gt;"",Pronostici!$J50&lt;&gt;"",Pronostici!$I50=Partite!$G50,Pronostici!$J50=Partite!$H50),Config!$D$6,IF(AND($K50&lt;&gt;"",$K50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$I50&lt;&gt;"",Pronostici!$J50&lt;&gt;"",Pronostici!$I50=Partite!$G50,Pronostici!$J50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$Q50)=1),Config!$D$9,Config!$D$6),IF(AND($K50&lt;&gt;"",$K50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$K50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$L50&lt;&gt;"",Pronostici!$M50&lt;&gt;"",Pronostici!$L50=Partite!$G50,Pronostici!$M50=Partite!$H50),Config!$D$6,IF(AND($L50&lt;&gt;"",$L50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$L50&lt;&gt;"",Pronostici!$M50&lt;&gt;"",Pronostici!$L50=Partite!$G50,Pronostici!$M50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$R50)=1),Config!$D$9,Config!$D$6),IF(AND($L50&lt;&gt;"",$L50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$L50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$O50&lt;&gt;"",Pronostici!$P50&lt;&gt;"",Pronostici!$O50=Partite!$G50,Pronostici!$P50=Partite!$H50),Config!$D$6,IF(AND($M50&lt;&gt;"",$M50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$O50&lt;&gt;"",Pronostici!$P50&lt;&gt;"",Pronostici!$O50=Partite!$G50,Pronostici!$P50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$S50)=1),Config!$D$9,Config!$D$6),IF(AND($M50&lt;&gt;"",$M50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$M50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H50" s="22">
-        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$R50&lt;&gt;"",Pronostici!$S50&lt;&gt;"",Pronostici!$R50=Partite!$G50,Pronostici!$S50=Partite!$H50),Config!$D$6,IF(AND($N50&lt;&gt;"",$N50=Partite!$I50),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K50&lt;&gt;"Giocata","",IF(AND(Pronostici!$R50&lt;&gt;"",Pronostici!$S50&lt;&gt;"",Pronostici!$R50=Partite!$G50,Pronostici!$S50=Partite!$H50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($P50:$T50,$T50)=1),Config!$D$9,Config!$D$6),IF(AND($N50&lt;&gt;"",$N50=Partite!$I50),IF(AND($B50&gt;=Config!$D$17,COUNTIF($J50:$N50,$N50)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J50" s="63">
@@ -10536,6 +11501,26 @@
       </c>
       <c r="N50" s="63">
         <f>IF(Pronostici!$Q50&lt;&gt;"",UPPER(Pronostici!$Q50),IF(OR(Pronostici!$R50="",Pronostici!$S50=""),"",IF(Pronostici!$R50&gt;Pronostici!$S50,"1",IF(Pronostici!$R50=Pronostici!$S50,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P50" s="63">
+        <f>IF(OR(Pronostici!$F50="",Pronostici!$G50=""),"",Pronostici!$F50&amp;" a "&amp;Pronostici!$G50)</f>
+        <v/>
+      </c>
+      <c r="Q50" s="63">
+        <f>IF(OR(Pronostici!$I50="",Pronostici!$J50=""),"",Pronostici!$I50&amp;" a "&amp;Pronostici!$J50)</f>
+        <v/>
+      </c>
+      <c r="R50" s="63">
+        <f>IF(OR(Pronostici!$L50="",Pronostici!$M50=""),"",Pronostici!$L50&amp;" a "&amp;Pronostici!$M50)</f>
+        <v/>
+      </c>
+      <c r="S50" s="63">
+        <f>IF(OR(Pronostici!$O50="",Pronostici!$P50=""),"",Pronostici!$O50&amp;" a "&amp;Pronostici!$P50)</f>
+        <v/>
+      </c>
+      <c r="T50" s="63">
+        <f>IF(OR(Pronostici!$R50="",Pronostici!$S50=""),"",Pronostici!$R50&amp;" a "&amp;Pronostici!$S50)</f>
         <v/>
       </c>
     </row>
@@ -10553,23 +11538,23 @@
         <v/>
       </c>
       <c r="D51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$F51&lt;&gt;"",Pronostici!$G51&lt;&gt;"",Pronostici!$F51=Partite!$G51,Pronostici!$G51=Partite!$H51),Config!$D$6,IF(AND($J51&lt;&gt;"",$J51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$F51&lt;&gt;"",Pronostici!$G51&lt;&gt;"",Pronostici!$F51=Partite!$G51,Pronostici!$G51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$P51)=1),Config!$D$9,Config!$D$6),IF(AND($J51&lt;&gt;"",$J51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$J51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$I51&lt;&gt;"",Pronostici!$J51&lt;&gt;"",Pronostici!$I51=Partite!$G51,Pronostici!$J51=Partite!$H51),Config!$D$6,IF(AND($K51&lt;&gt;"",$K51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$I51&lt;&gt;"",Pronostici!$J51&lt;&gt;"",Pronostici!$I51=Partite!$G51,Pronostici!$J51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$Q51)=1),Config!$D$9,Config!$D$6),IF(AND($K51&lt;&gt;"",$K51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$K51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$L51&lt;&gt;"",Pronostici!$M51&lt;&gt;"",Pronostici!$L51=Partite!$G51,Pronostici!$M51=Partite!$H51),Config!$D$6,IF(AND($L51&lt;&gt;"",$L51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$L51&lt;&gt;"",Pronostici!$M51&lt;&gt;"",Pronostici!$L51=Partite!$G51,Pronostici!$M51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$R51)=1),Config!$D$9,Config!$D$6),IF(AND($L51&lt;&gt;"",$L51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$L51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$O51&lt;&gt;"",Pronostici!$P51&lt;&gt;"",Pronostici!$O51=Partite!$G51,Pronostici!$P51=Partite!$H51),Config!$D$6,IF(AND($M51&lt;&gt;"",$M51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$O51&lt;&gt;"",Pronostici!$P51&lt;&gt;"",Pronostici!$O51=Partite!$G51,Pronostici!$P51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$S51)=1),Config!$D$9,Config!$D$6),IF(AND($M51&lt;&gt;"",$M51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$M51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H51" s="22">
-        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$R51&lt;&gt;"",Pronostici!$S51&lt;&gt;"",Pronostici!$R51=Partite!$G51,Pronostici!$S51=Partite!$H51),Config!$D$6,IF(AND($N51&lt;&gt;"",$N51=Partite!$I51),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K51&lt;&gt;"Giocata","",IF(AND(Pronostici!$R51&lt;&gt;"",Pronostici!$S51&lt;&gt;"",Pronostici!$R51=Partite!$G51,Pronostici!$S51=Partite!$H51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($P51:$T51,$T51)=1),Config!$D$9,Config!$D$6),IF(AND($N51&lt;&gt;"",$N51=Partite!$I51),IF(AND($B51&gt;=Config!$D$17,COUNTIF($J51:$N51,$N51)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J51" s="63">
@@ -10590,6 +11575,26 @@
       </c>
       <c r="N51" s="63">
         <f>IF(Pronostici!$Q51&lt;&gt;"",UPPER(Pronostici!$Q51),IF(OR(Pronostici!$R51="",Pronostici!$S51=""),"",IF(Pronostici!$R51&gt;Pronostici!$S51,"1",IF(Pronostici!$R51=Pronostici!$S51,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P51" s="63">
+        <f>IF(OR(Pronostici!$F51="",Pronostici!$G51=""),"",Pronostici!$F51&amp;" a "&amp;Pronostici!$G51)</f>
+        <v/>
+      </c>
+      <c r="Q51" s="63">
+        <f>IF(OR(Pronostici!$I51="",Pronostici!$J51=""),"",Pronostici!$I51&amp;" a "&amp;Pronostici!$J51)</f>
+        <v/>
+      </c>
+      <c r="R51" s="63">
+        <f>IF(OR(Pronostici!$L51="",Pronostici!$M51=""),"",Pronostici!$L51&amp;" a "&amp;Pronostici!$M51)</f>
+        <v/>
+      </c>
+      <c r="S51" s="63">
+        <f>IF(OR(Pronostici!$O51="",Pronostici!$P51=""),"",Pronostici!$O51&amp;" a "&amp;Pronostici!$P51)</f>
+        <v/>
+      </c>
+      <c r="T51" s="63">
+        <f>IF(OR(Pronostici!$R51="",Pronostici!$S51=""),"",Pronostici!$R51&amp;" a "&amp;Pronostici!$S51)</f>
         <v/>
       </c>
     </row>
@@ -10607,23 +11612,23 @@
         <v/>
       </c>
       <c r="D52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$F52&lt;&gt;"",Pronostici!$G52&lt;&gt;"",Pronostici!$F52=Partite!$G52,Pronostici!$G52=Partite!$H52),Config!$D$6,IF(AND($J52&lt;&gt;"",$J52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$F52&lt;&gt;"",Pronostici!$G52&lt;&gt;"",Pronostici!$F52=Partite!$G52,Pronostici!$G52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$P52)=1),Config!$D$9,Config!$D$6),IF(AND($J52&lt;&gt;"",$J52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$J52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="E52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$I52&lt;&gt;"",Pronostici!$J52&lt;&gt;"",Pronostici!$I52=Partite!$G52,Pronostici!$J52=Partite!$H52),Config!$D$6,IF(AND($K52&lt;&gt;"",$K52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$I52&lt;&gt;"",Pronostici!$J52&lt;&gt;"",Pronostici!$I52=Partite!$G52,Pronostici!$J52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$Q52)=1),Config!$D$9,Config!$D$6),IF(AND($K52&lt;&gt;"",$K52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$K52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="F52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$L52&lt;&gt;"",Pronostici!$M52&lt;&gt;"",Pronostici!$L52=Partite!$G52,Pronostici!$M52=Partite!$H52),Config!$D$6,IF(AND($L52&lt;&gt;"",$L52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$L52&lt;&gt;"",Pronostici!$M52&lt;&gt;"",Pronostici!$L52=Partite!$G52,Pronostici!$M52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$R52)=1),Config!$D$9,Config!$D$6),IF(AND($L52&lt;&gt;"",$L52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$L52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="G52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$O52&lt;&gt;"",Pronostici!$P52&lt;&gt;"",Pronostici!$O52=Partite!$G52,Pronostici!$P52=Partite!$H52),Config!$D$6,IF(AND($M52&lt;&gt;"",$M52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$O52&lt;&gt;"",Pronostici!$P52&lt;&gt;"",Pronostici!$O52=Partite!$G52,Pronostici!$P52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$S52)=1),Config!$D$9,Config!$D$6),IF(AND($M52&lt;&gt;"",$M52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$M52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="H52" s="22">
-        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$R52&lt;&gt;"",Pronostici!$S52&lt;&gt;"",Pronostici!$R52=Partite!$G52,Pronostici!$S52=Partite!$H52),Config!$D$6,IF(AND($N52&lt;&gt;"",$N52=Partite!$I52),Config!$D$7,Config!$D$8)))</f>
+        <f>IF(Partite!$K52&lt;&gt;"Giocata","",IF(AND(Pronostici!$R52&lt;&gt;"",Pronostici!$S52&lt;&gt;"",Pronostici!$R52=Partite!$G52,Pronostici!$S52=Partite!$H52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($P52:$T52,$T52)=1),Config!$D$9,Config!$D$6),IF(AND($N52&lt;&gt;"",$N52=Partite!$I52),IF(AND($B52&gt;=Config!$D$17,COUNTIF($J52:$N52,$N52)=1),Config!$D$10,Config!$D$7),Config!$D$8)))</f>
         <v/>
       </c>
       <c r="J52" s="63">
@@ -10644,6 +11649,26 @@
       </c>
       <c r="N52" s="63">
         <f>IF(Pronostici!$Q52&lt;&gt;"",UPPER(Pronostici!$Q52),IF(OR(Pronostici!$R52="",Pronostici!$S52=""),"",IF(Pronostici!$R52&gt;Pronostici!$S52,"1",IF(Pronostici!$R52=Pronostici!$S52,"X","2"))))</f>
+        <v/>
+      </c>
+      <c r="P52" s="63">
+        <f>IF(OR(Pronostici!$F52="",Pronostici!$G52=""),"",Pronostici!$F52&amp;" a "&amp;Pronostici!$G52)</f>
+        <v/>
+      </c>
+      <c r="Q52" s="63">
+        <f>IF(OR(Pronostici!$I52="",Pronostici!$J52=""),"",Pronostici!$I52&amp;" a "&amp;Pronostici!$J52)</f>
+        <v/>
+      </c>
+      <c r="R52" s="63">
+        <f>IF(OR(Pronostici!$L52="",Pronostici!$M52=""),"",Pronostici!$L52&amp;" a "&amp;Pronostici!$M52)</f>
+        <v/>
+      </c>
+      <c r="S52" s="63">
+        <f>IF(OR(Pronostici!$O52="",Pronostici!$P52=""),"",Pronostici!$O52&amp;" a "&amp;Pronostici!$P52)</f>
+        <v/>
+      </c>
+      <c r="T52" s="63">
+        <f>IF(OR(Pronostici!$R52="",Pronostici!$S52=""),"",Pronostici!$R52&amp;" a "&amp;Pronostici!$S52)</f>
         <v/>
       </c>
     </row>
@@ -10652,43 +11677,48 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D52">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
       <formula>1</formula>
+      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E52">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="4" operator="between" dxfId="1">
       <formula>1</formula>
+      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F52">
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="6" operator="between" dxfId="1">
       <formula>1</formula>
+      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G52">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="8" operator="between" dxfId="1">
       <formula>1</formula>
+      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H52">
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="10" operator="between" dxfId="1">
       <formula>1</formula>
+      <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10806,6 +11836,14 @@
           <t>Just Lele</t>
         </is>
       </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>Risultato esatto, e nessun altro lo aveva scritto</t>
+        </is>
+      </c>
+      <c r="D9" s="96" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="100" t="inlineStr">
@@ -10813,49 +11851,69 @@
           <t>Lippi</t>
         </is>
       </c>
-      <c r="C10" s="35" t="inlineStr">
-        <is>
-          <t>Il risultato esatto non si somma al segno: vale 3 punti in tutto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Segno giusto, e nessun altro lo aveva scelto</t>
+        </is>
+      </c>
+      <c r="D10" s="96" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>Il risultato esatto non si somma al segno. Gli ultimi due sono il solitario: valgono il doppio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="36" t="inlineStr">
         <is>
           <t>PARAMETRI</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="C13" s="43" t="inlineStr">
+    <row r="14">
+      <c r="C14" s="43" t="inlineStr">
         <is>
           <t>Stagione</t>
         </is>
       </c>
-      <c r="D13" s="71" t="inlineStr">
+      <c r="D14" s="71" t="inlineStr">
         <is>
           <t>Serie A 2026/27</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="C14" s="47" t="inlineStr">
+    <row r="15">
+      <c r="C15" s="47" t="inlineStr">
         <is>
           <t>Prima giornata in gioco</t>
         </is>
       </c>
-      <c r="D14" s="71" t="n">
+      <c r="D15" s="71" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="15">
-      <c r="C15" s="43" t="inlineStr">
+    <row r="16">
+      <c r="C16" s="43" t="inlineStr">
         <is>
           <t>Partite per giornata</t>
         </is>
       </c>
-      <c r="D15" s="71" t="n">
+      <c r="D16" s="71" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="47" t="inlineStr">
+        <is>
+          <t>Il solitario vale dalla giornata</t>
+        </is>
+      </c>
+      <c r="D17" s="71" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -10889,14 +11947,21 @@
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="102" t="inlineStr">
         <is>
-          <t>4.  Parita' in classifica generale: passa avanti chi ha piu' risultati esatti.</t>
+          <t>4.  Dalla giornata 5 chi indovina da solo vale doppio: 2 il segno, 6 il risultato esatto.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
       <c r="A25" s="101" t="inlineStr">
         <is>
-          <t>5.  Re della giornata = chi fa piu' punti in quella giornata (solo giornate complete).</t>
+          <t>5.  Parita' in classifica generale: passa avanti chi ha piu' risultati esatti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="102" t="inlineStr">
+        <is>
+          <t>6.  Re della giornata = chi fa piu' punti in quella giornata (solo giornate complete).</t>
         </is>
       </c>
     </row>
@@ -11029,11 +12094,11 @@
         <v>1</v>
       </c>
       <c r="E38" s="105" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F38" s="106" t="inlineStr">
         <is>
-          <t>segno e risultato esatti</t>
+          <t>risultato esatto, e nessun altro aveva scritto 2-1</t>
         </is>
       </c>
     </row>
@@ -11059,7 +12124,7 @@
       </c>
       <c r="F39" s="106" t="inlineStr">
         <is>
-          <t>segno giusto, risultato no</t>
+          <t>segno giusto, ma l'1 lo avevano in tre</t>
         </is>
       </c>
     </row>
@@ -11081,7 +12146,7 @@
       </c>
       <c r="F40" s="106" t="inlineStr">
         <is>
-          <t>solo il segno, ed e' giusto</t>
+          <t>solo il segno, giusto ma in compagnia</t>
         </is>
       </c>
     </row>
@@ -11129,6 +12194,13 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>Esempio dalla giornata 5 in poi. Se il segno giusto lo avesse scelto una persona sola, a lei varrebbe 2 punti invece di 1.</t>
+        </is>
+      </c>
+    </row>
     <row r="45">
       <c r="A45" s="35" t="inlineStr">
         <is>
@@ -11144,13 +12216,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A21:D21"/>
     <mergeCell ref="A1:F2"/>
     <mergeCell ref="A25:D25"/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 11/09/2026 alle 23:03
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3502,8 +3502,12 @@
           <t>Fiorentina</t>
         </is>
       </c>
-      <c r="G23" s="71" t="n"/>
-      <c r="H23" s="71" t="n"/>
+      <c r="G23" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="71" t="n">
+        <v>4</v>
+      </c>
       <c r="I23" s="72">
         <f>IF(OR($G23="",$H23=""),"",IF($G23&gt;$H23,"1",IF($G23=$H23,"X","2")))</f>
         <v/>
@@ -11838,7 +11842,7 @@
       </c>
       <c r="C9" s="47" t="inlineStr">
         <is>
-          <t>Risultato esatto, e nessun altro lo aveva scritto</t>
+          <t>CORAGGIO - risultato esatto, e nessun altro lo aveva scritto</t>
         </is>
       </c>
       <c r="D9" s="96" t="n">
@@ -11853,7 +11857,7 @@
       </c>
       <c r="C10" s="43" t="inlineStr">
         <is>
-          <t>Segno giusto, e nessun altro lo aveva scelto</t>
+          <t>CORAGGIO - segno giusto, e nessun altro lo aveva scelto</t>
         </is>
       </c>
       <c r="D10" s="96" t="n">
@@ -11863,7 +11867,7 @@
     <row r="11">
       <c r="C11" s="35" t="inlineStr">
         <is>
-          <t>Il risultato esatto non si somma al segno. Gli ultimi due sono il solitario: valgono il doppio.</t>
+          <t>Il risultato esatto non si somma al segno. Gli ultimi due sono i punti coraggio: chi indovina da solo prende il doppio.</t>
         </is>
       </c>
     </row>
@@ -11909,7 +11913,7 @@
     <row r="17">
       <c r="C17" s="47" t="inlineStr">
         <is>
-          <t>Il solitario vale dalla giornata</t>
+          <t>I punti coraggio valgono dalla giornata</t>
         </is>
       </c>
       <c r="D17" s="71" t="n">
@@ -11947,7 +11951,7 @@
     <row r="24" ht="17" customHeight="1">
       <c r="A24" s="102" t="inlineStr">
         <is>
-          <t>4.  Dalla giornata 5 chi indovina da solo vale doppio: 2 il segno, 6 il risultato esatto.</t>
+          <t>4.  Punti coraggio, dalla giornata 5: chi indovina da solo vale doppio, 2 il segno e 6 il risultato esatto.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggiornamento automatico del 12/09/2026 alle 17:48
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3550,8 +3550,12 @@
           <t>Frosinone</t>
         </is>
       </c>
-      <c r="G24" s="71" t="n"/>
-      <c r="H24" s="71" t="n"/>
+      <c r="G24" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="71" t="n">
+        <v>1</v>
+      </c>
       <c r="I24" s="72">
         <f>IF(OR($G24="",$H24=""),"",IF($G24&gt;$H24,"1",IF($G24=$H24,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 12/09/2026 alle 21:57
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3598,8 +3598,12 @@
           <t>Milan</t>
         </is>
       </c>
-      <c r="G25" s="71" t="n"/>
-      <c r="H25" s="71" t="n"/>
+      <c r="G25" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I25" s="72">
         <f>IF(OR($G25="",$H25=""),"",IF($G25&gt;$H25,"1",IF($G25=$H25,"X","2")))</f>
         <v/>

</xml_diff>

<commit_message>
Aggiornamento automatico del 12/09/2026 alle 23:59
</commit_message>
<xml_diff>
--- a/docs/Trofeo_Ovalmo.xlsx
+++ b/docs/Trofeo_Ovalmo.xlsx
@@ -3690,8 +3690,12 @@
           <t>Cagliari</t>
         </is>
       </c>
-      <c r="G27" s="71" t="n"/>
-      <c r="H27" s="71" t="n"/>
+      <c r="G27" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="71" t="n">
+        <v>2</v>
+      </c>
       <c r="I27" s="72">
         <f>IF(OR($G27="",$H27=""),"",IF($G27&gt;$H27,"1",IF($G27=$H27,"X","2")))</f>
         <v/>

</xml_diff>